<commit_message>
Menü güncelleme 18.09.2026 13:57
</commit_message>
<xml_diff>
--- a/KULE-alerjen-kontrol.xlsx
+++ b/KULE-alerjen-kontrol.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nasıl kullanılır" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Menü'!$A$1:$AB$174</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Menü'!$A$1:$AC$174</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -497,7 +497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB174"/>
+  <dimension ref="A1:AC174"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -527,7 +527,8 @@
     <col width="13" customWidth="1" min="25" max="25"/>
     <col width="9" customWidth="1" min="26" max="26"/>
     <col width="11" customWidth="1" min="27" max="27"/>
-    <col width="26" customWidth="1" min="28" max="28"/>
+    <col width="18" customWidth="1" min="28" max="28"/>
+    <col width="26" customWidth="1" min="29" max="29"/>
   </cols>
   <sheetData>
     <row r="1" ht="40" customHeight="1">
@@ -668,6 +669,11 @@
       </c>
       <c r="AB1" s="1" t="inlineStr">
         <is>
+          <t>Sos kartı</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
           <t>Notunuz</t>
         </is>
       </c>
@@ -698,12 +704,12 @@
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>Sahanda yumurta, menemen, kalem böreği, patates tabağı, söğüş tabağı, beyaz peynir, taze kaşar, çeçil peyniri, burgu peynir, lor peyniri, jambon, kaymak, tereyağı, siyah–yeşil zeytin, zeytin salatası, acuka, bal, Nutella, reçel</t>
+          <t>Sahanda yumurta, menemen, kalem böreği, patates tabağı, söğüş tabağı, beyaz peynir, taze kaşar, çeçil peyniri, burgu peynir, lor peyniri, jambon, kaymak, tereyağı, siyah–yeşil zeytin, zeytin salatası, acuka, bal, Nutella, reçel, sınırsız ekmek sepeti, sınırsız çay</t>
         </is>
       </c>
       <c r="G2" s="4" t="inlineStr">
         <is>
-          <t>Fried eggs, menemen, cheese rolls, potato plate, sliced tomato &amp; cucumber, white cheese, fresh kashar, chechil cheese, braided cheese, curd cheese, ham, clotted cream, butter, black &amp; green olives, olive salad, acuka, honey, Nutella, jam</t>
+          <t>Fried eggs, menemen, cheese rolls, potato plate, sliced tomato &amp; cucumber, white cheese, fresh kashar, chechil cheese, braided cheese, curd cheese, ham, clotted cream, butter, black &amp; green olives, olive salad, acuka, honey, Nutella, jam, unlimited bread basket, unlimited tea</t>
         </is>
       </c>
       <c r="H2" s="5" t="inlineStr">
@@ -750,7 +756,8 @@
       </c>
       <c r="Z2" s="8" t="inlineStr"/>
       <c r="AA2" s="8" t="inlineStr"/>
-      <c r="AB2" s="9" t="inlineStr"/>
+      <c r="AB2" s="8" t="inlineStr"/>
+      <c r="AC2" s="9" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -778,12 +785,12 @@
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>Yumurta, tereyağı, tuz</t>
+          <t>Yumurta, tereyağı, tuz, ayçiçek yağı</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>Egg, butter, salt</t>
+          <t>Egg, butter, salt, sunflower oil</t>
         </is>
       </c>
       <c r="H3" s="5" t="inlineStr"/>
@@ -822,7 +829,8 @@
       </c>
       <c r="Z3" s="8" t="inlineStr"/>
       <c r="AA3" s="8" t="inlineStr"/>
-      <c r="AB3" s="9" t="inlineStr"/>
+      <c r="AB3" s="8" t="inlineStr"/>
+      <c r="AC3" s="9" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -850,12 +858,12 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>Yumurta, beyaz peynir, tereyağı, tuz</t>
+          <t>Yumurta, beyaz peynir, tereyağı, tuz, ayçiçek yağı</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>Egg, white cheese, butter, salt</t>
+          <t>Egg, white cheese, butter, salt, sunflower oil</t>
         </is>
       </c>
       <c r="H4" s="5" t="inlineStr"/>
@@ -894,7 +902,8 @@
       </c>
       <c r="Z4" s="8" t="inlineStr"/>
       <c r="AA4" s="8" t="inlineStr"/>
-      <c r="AB4" s="9" t="inlineStr"/>
+      <c r="AB4" s="8" t="inlineStr"/>
+      <c r="AC4" s="9" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -922,12 +931,12 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>Yumurta, kaşar peyniri, tereyağı, tuz</t>
+          <t>Yumurta, kaşar peyniri, tereyağı, tuz, ayçiçek yağı</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>Egg, kashar cheese, butter, salt</t>
+          <t>Egg, kashar cheese, butter, salt, sunflower oil</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr"/>
@@ -966,7 +975,8 @@
       </c>
       <c r="Z5" s="8" t="inlineStr"/>
       <c r="AA5" s="8" t="inlineStr"/>
-      <c r="AB5" s="9" t="inlineStr"/>
+      <c r="AB5" s="8" t="inlineStr"/>
+      <c r="AC5" s="9" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -994,12 +1004,12 @@
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>Yumurta, kaşar peyniri, sucuk, sosis, biber, tereyağı, tuz</t>
+          <t>Yumurta, kaşar peyniri, sucuk, sosis, biber, tereyağı, tuz, ayçiçek yağı</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>Egg, kashar cheese, sucuk, sausage, pepper, butter, salt</t>
+          <t>Egg, kashar cheese, sucuk, sausage, pepper, butter, salt, sunflower oil</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr"/>
@@ -1038,7 +1048,8 @@
       </c>
       <c r="Z6" s="8" t="inlineStr"/>
       <c r="AA6" s="8" t="inlineStr"/>
-      <c r="AB6" s="9" t="inlineStr"/>
+      <c r="AB6" s="8" t="inlineStr"/>
+      <c r="AC6" s="9" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1066,12 +1077,12 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>Yumurta, et kavurma, tereyağı, tuz</t>
+          <t>Yumurta, et kavurma, tereyağı, tuz, ayçiçek yağı</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>Egg, roasted meat, butter, salt</t>
+          <t>Egg, roasted meat, butter, salt, sunflower oil</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr"/>
@@ -1110,7 +1121,8 @@
       </c>
       <c r="Z7" s="8" t="inlineStr"/>
       <c r="AA7" s="8" t="inlineStr"/>
-      <c r="AB7" s="9" t="inlineStr"/>
+      <c r="AB7" s="8" t="inlineStr"/>
+      <c r="AC7" s="9" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1138,12 +1150,12 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>Yumurta, sucuk, tereyağı, tuz</t>
+          <t>Yumurta, sucuk, tereyağı, tuz, ayçiçek yağı</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>Egg, sucuk, butter, salt</t>
+          <t>Egg, sucuk, butter, salt, sunflower oil</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr"/>
@@ -1182,7 +1194,8 @@
       </c>
       <c r="Z8" s="8" t="inlineStr"/>
       <c r="AA8" s="8" t="inlineStr"/>
-      <c r="AB8" s="9" t="inlineStr"/>
+      <c r="AB8" s="8" t="inlineStr"/>
+      <c r="AC8" s="9" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1210,12 +1223,12 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>Yumurta, tereyağı, tuz</t>
+          <t>Yumurta, tereyağı, tuz, ayçiçek yağı</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>Egg, butter, salt</t>
+          <t>Egg, butter, salt, sunflower oil</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr"/>
@@ -1254,7 +1267,8 @@
       </c>
       <c r="Z9" s="8" t="inlineStr"/>
       <c r="AA9" s="8" t="inlineStr"/>
-      <c r="AB9" s="9" t="inlineStr"/>
+      <c r="AB9" s="8" t="inlineStr"/>
+      <c r="AC9" s="9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1282,12 +1296,12 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>Sucuk, tereyağı</t>
+          <t>Sucuk, tereyağı, ayçiçek yağı</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>Sucuk, butter</t>
+          <t>Sucuk, butter, sunflower oil</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr"/>
@@ -1322,7 +1336,8 @@
       </c>
       <c r="Z10" s="8" t="inlineStr"/>
       <c r="AA10" s="8" t="inlineStr"/>
-      <c r="AB10" s="9" t="inlineStr"/>
+      <c r="AB10" s="8" t="inlineStr"/>
+      <c r="AC10" s="9" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1350,12 +1365,12 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>Yumurta, domates, sivri biber, tereyağı, tuz, karabiber</t>
+          <t>Yumurta, domates, sivri biber, tereyağı, tuz, karabiber, ayçiçek yağı</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>Egg, tomato, green pepper, butter, salt, black pepper</t>
+          <t>Egg, tomato, green pepper, butter, salt, black pepper, sunflower oil</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr"/>
@@ -1394,7 +1409,8 @@
       </c>
       <c r="Z11" s="8" t="inlineStr"/>
       <c r="AA11" s="8" t="inlineStr"/>
-      <c r="AB11" s="9" t="inlineStr"/>
+      <c r="AB11" s="8" t="inlineStr"/>
+      <c r="AC11" s="9" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1422,12 +1438,12 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>Yumurta, domates, sivri biber, kaşar peyniri, tereyağı, tuz, karabiber</t>
+          <t>Yumurta, domates, sivri biber, kaşar peyniri, tereyağı, tuz, karabiber, ayçiçek yağı</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>Egg, tomato, green pepper, kashar cheese, butter, salt, black pepper</t>
+          <t>Egg, tomato, green pepper, kashar cheese, butter, salt, black pepper, sunflower oil</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr"/>
@@ -1466,7 +1482,8 @@
       </c>
       <c r="Z12" s="8" t="inlineStr"/>
       <c r="AA12" s="8" t="inlineStr"/>
-      <c r="AB12" s="9" t="inlineStr"/>
+      <c r="AB12" s="8" t="inlineStr"/>
+      <c r="AC12" s="9" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1534,7 +1551,8 @@
       </c>
       <c r="Z13" s="8" t="inlineStr"/>
       <c r="AA13" s="8" t="inlineStr"/>
-      <c r="AB13" s="9" t="inlineStr"/>
+      <c r="AB13" s="8" t="inlineStr"/>
+      <c r="AC13" s="9" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1562,12 +1580,12 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>Tost ekmeği, çift kaşar peyniri, tereyağı; domates, salatalık, patates</t>
+          <t>Tost ekmeği, çift kaşar peyniri, tereyağı; domates, salatalık, parmak patates eşliğinde</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>Toast bread, double kashar cheese, butter; tomato, cucumber, fries</t>
+          <t>Toast bread, double kashar cheese, butter; served with tomato, cucumber and french fries</t>
         </is>
       </c>
       <c r="H14" s="5" t="inlineStr">
@@ -1606,7 +1624,8 @@
       </c>
       <c r="Z14" s="8" t="inlineStr"/>
       <c r="AA14" s="8" t="inlineStr"/>
-      <c r="AB14" s="9" t="inlineStr"/>
+      <c r="AB14" s="8" t="inlineStr"/>
+      <c r="AC14" s="9" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1634,12 +1653,12 @@
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>Tost ekmeği, kaşar peyniri, sucuk, tereyağı; domates, salatalık, patates</t>
+          <t>Tost ekmeği, kaşar peyniri, sucuk, tereyağı; domates, salatalık, parmak patates eşliğinde</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>Toast bread, kashar cheese, sucuk, butter; tomato, cucumber, fries</t>
+          <t>Toast bread, kashar cheese, sucuk, butter; served with tomato, cucumber and french fries</t>
         </is>
       </c>
       <c r="H15" s="5" t="inlineStr">
@@ -1678,7 +1697,8 @@
       </c>
       <c r="Z15" s="8" t="inlineStr"/>
       <c r="AA15" s="8" t="inlineStr"/>
-      <c r="AB15" s="9" t="inlineStr"/>
+      <c r="AB15" s="8" t="inlineStr"/>
+      <c r="AC15" s="9" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1742,7 +1762,8 @@
       </c>
       <c r="Z16" s="8" t="inlineStr"/>
       <c r="AA16" s="8" t="inlineStr"/>
-      <c r="AB16" s="9" t="inlineStr"/>
+      <c r="AB16" s="8" t="inlineStr"/>
+      <c r="AC16" s="9" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1770,12 +1791,12 @@
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>Cajun baharatlı çıtır tavuk parçaları, patates, sos (yumurta, un, süt, Cajun baharatı, tuz, karabiber, soya sosu)</t>
+          <t>180 g Cajun baharatlı çıtır tavuk parçaları, sos (yumurta, un, süt, Cajun baharatı, tuz, karabiber, soya sosu), elma dilim patates eşliğinde</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>Cajun-spiced crispy chicken strips, fries, sauce (egg, flour, milk, Cajun spice, salt, black pepper, soy sauce)</t>
+          <t>180 g Cajun-spiced crispy chicken pieces, sauce (egg, flour, milk, Cajun spice, salt, black pepper, soy sauce), served with wedge potatoes</t>
         </is>
       </c>
       <c r="H17" s="5" t="inlineStr">
@@ -1809,20 +1830,21 @@
       <c r="T17" s="5" t="inlineStr"/>
       <c r="U17" s="5" t="inlineStr"/>
       <c r="V17" s="6" t="n">
-        <v>640</v>
+        <v>680</v>
       </c>
       <c r="W17" s="7" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="X17" s="7" t="n">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="Y17" s="7" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="Z17" s="8" t="inlineStr"/>
       <c r="AA17" s="8" t="inlineStr"/>
-      <c r="AB17" s="9" t="inlineStr"/>
+      <c r="AB17" s="8" t="inlineStr"/>
+      <c r="AC17" s="9" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1850,12 +1872,12 @@
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>Çıtır tavuk, soğan halkası, mozzarella stick, sosis, patates, soslar</t>
+          <t>2 adet çıtır tavuk (yumurta, un, süt, Cajun baharatı, tuz, karabiber, soya sosu), 2 adet sigara böreği, 2 adet soğan halkası, 2 adet mozzarella stick, 2 adet sosis, elma dilim patates eşliğinde</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>Crispy chicken, onion rings, mozzarella sticks, sausage, fries, dips</t>
+          <t>2 crispy chicken pieces (egg, flour, milk, Cajun spice, salt, black pepper, soy sauce), 2 cheese rolls, 2 onion rings, 2 mozzarella sticks, 2 sausages, served with wedge potatoes</t>
         </is>
       </c>
       <c r="H18" s="5" t="inlineStr">
@@ -1875,34 +1897,35 @@
       </c>
       <c r="K18" s="5" t="inlineStr"/>
       <c r="L18" s="5" t="inlineStr"/>
-      <c r="M18" s="5" t="inlineStr"/>
+      <c r="M18" s="5" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="N18" s="5" t="inlineStr"/>
       <c r="O18" s="5" t="inlineStr"/>
       <c r="P18" s="5" t="inlineStr"/>
-      <c r="Q18" s="5" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="Q18" s="5" t="inlineStr"/>
       <c r="R18" s="5" t="inlineStr"/>
       <c r="S18" s="5" t="inlineStr"/>
       <c r="T18" s="5" t="inlineStr"/>
       <c r="U18" s="5" t="inlineStr"/>
       <c r="V18" s="6" t="n">
-        <v>950</v>
+        <v>1180</v>
       </c>
       <c r="W18" s="7" t="n">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="X18" s="7" t="n">
-        <v>52</v>
+        <v>66</v>
       </c>
       <c r="Y18" s="7" t="n">
-        <v>78</v>
+        <v>92</v>
       </c>
       <c r="Z18" s="8" t="inlineStr"/>
       <c r="AA18" s="8" t="inlineStr"/>
-      <c r="AB18" s="9" t="inlineStr"/>
+      <c r="AB18" s="8" t="inlineStr"/>
+      <c r="AC18" s="9" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1966,7 +1989,8 @@
       </c>
       <c r="Z19" s="8" t="inlineStr"/>
       <c r="AA19" s="8" t="inlineStr"/>
-      <c r="AB19" s="9" t="inlineStr"/>
+      <c r="AB19" s="8" t="inlineStr"/>
+      <c r="AC19" s="9" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1994,12 +2018,12 @@
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>Patates, tuz</t>
+          <t>Patates</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>Potato, salt</t>
+          <t>Potato</t>
         </is>
       </c>
       <c r="H20" s="5" t="inlineStr"/>
@@ -2030,7 +2054,8 @@
       </c>
       <c r="Z20" s="8" t="inlineStr"/>
       <c r="AA20" s="8" t="inlineStr"/>
-      <c r="AB20" s="9" t="inlineStr"/>
+      <c r="AB20" s="8" t="inlineStr"/>
+      <c r="AC20" s="9" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -2058,12 +2083,12 @@
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>Izgara sosis, patates</t>
+          <t>8 adet ızgara sosis, parmak patates eşliğinde</t>
         </is>
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
-          <t>Grilled sausages, fries</t>
+          <t>8 grilled sausages, served with french fries</t>
         </is>
       </c>
       <c r="H21" s="5" t="inlineStr">
@@ -2085,20 +2110,21 @@
       <c r="T21" s="5" t="inlineStr"/>
       <c r="U21" s="5" t="inlineStr"/>
       <c r="V21" s="6" t="n">
-        <v>620</v>
+        <v>900</v>
       </c>
       <c r="W21" s="7" t="n">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="X21" s="7" t="n">
-        <v>40</v>
+        <v>58</v>
       </c>
       <c r="Y21" s="7" t="n">
-        <v>40</v>
+        <v>56</v>
       </c>
       <c r="Z21" s="8" t="inlineStr"/>
       <c r="AA21" s="8" t="inlineStr"/>
-      <c r="AB21" s="9" t="inlineStr"/>
+      <c r="AB21" s="8" t="inlineStr"/>
+      <c r="AC21" s="9" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -2126,12 +2152,12 @@
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>Soğan, galeta unu</t>
+          <t>8 adet soğan halkası (soğan, galeta unu), parmak patates eşliğinde</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">
         <is>
-          <t>Onion, breadcrumbs</t>
+          <t>8 onion rings (onion, breadcrumbs), served with french fries</t>
         </is>
       </c>
       <c r="H22" s="5" t="inlineStr">
@@ -2157,20 +2183,21 @@
       <c r="T22" s="5" t="inlineStr"/>
       <c r="U22" s="5" t="inlineStr"/>
       <c r="V22" s="6" t="n">
-        <v>430</v>
+        <v>700</v>
       </c>
       <c r="W22" s="7" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="X22" s="7" t="n">
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="Y22" s="7" t="n">
-        <v>48</v>
+        <v>84</v>
       </c>
       <c r="Z22" s="8" t="inlineStr"/>
       <c r="AA22" s="8" t="inlineStr"/>
-      <c r="AB22" s="9" t="inlineStr"/>
+      <c r="AB22" s="8" t="inlineStr"/>
+      <c r="AC22" s="9" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -2198,12 +2225,12 @@
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>Yufka, beyaz peynir, maydanoz, tuz</t>
+          <t>10 adet sigara böreği (yufka, beyaz peynir, maydanoz, soda, tuz), domates ve salatalık eşliğinde</t>
         </is>
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
-          <t>Yufka pastry, white cheese, parsley, salt</t>
+          <t>10 cheese rolls (yufka pastry, white cheese, parsley, sparkling water, salt), served with tomato and cucumber</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
@@ -2229,20 +2256,21 @@
       <c r="T23" s="5" t="inlineStr"/>
       <c r="U23" s="5" t="inlineStr"/>
       <c r="V23" s="6" t="n">
-        <v>380</v>
+        <v>620</v>
       </c>
       <c r="W23" s="7" t="n">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="X23" s="7" t="n">
-        <v>24</v>
+        <v>38</v>
       </c>
       <c r="Y23" s="7" t="n">
-        <v>28</v>
+        <v>46</v>
       </c>
       <c r="Z23" s="8" t="inlineStr"/>
       <c r="AA23" s="8" t="inlineStr"/>
-      <c r="AB23" s="9" t="inlineStr"/>
+      <c r="AB23" s="8" t="inlineStr"/>
+      <c r="AC23" s="9" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -2270,12 +2298,12 @@
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>Domates, salatalık, soğan, biber, maydanoz, zeytinyağı</t>
+          <t>Domates, salatalık, soğan, biber, maydanoz, zeytinyağı, limon eşliğinde</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>Tomato, cucumber, onion, pepper, parsley, olive oil</t>
+          <t>Tomato, cucumber, onion, pepper, parsley, olive oil, served with lemon</t>
         </is>
       </c>
       <c r="H24" s="5" t="inlineStr"/>
@@ -2306,7 +2334,8 @@
       </c>
       <c r="Z24" s="8" t="inlineStr"/>
       <c r="AA24" s="8" t="inlineStr"/>
-      <c r="AB24" s="9" t="inlineStr"/>
+      <c r="AB24" s="8" t="inlineStr"/>
+      <c r="AC24" s="9" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -2370,7 +2399,8 @@
       </c>
       <c r="Z25" s="8" t="inlineStr"/>
       <c r="AA25" s="8" t="inlineStr"/>
-      <c r="AB25" s="9" t="inlineStr"/>
+      <c r="AB25" s="8" t="inlineStr"/>
+      <c r="AC25" s="9" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -2438,7 +2468,8 @@
       </c>
       <c r="Z26" s="8" t="inlineStr"/>
       <c r="AA26" s="8" t="inlineStr"/>
-      <c r="AB26" s="9" t="inlineStr"/>
+      <c r="AB26" s="8" t="inlineStr"/>
+      <c r="AC26" s="9" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2466,12 +2497,12 @@
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>160 g tavuk, göbek salata, kruton ekmek, parmesan, Sezar sos (mayonez, hardal, kapari çiçeği, ançüez)</t>
+          <t>160 g tavuk (zeytinyağı, taze kekik, tatlı kırmızı toz biber ile marine edilmiş), göbek salata, kruton ekmek, parmesan, Sezar sos (mayonez, hardal, kapari çiçeği, ançüez)</t>
         </is>
       </c>
       <c r="G27" s="4" t="inlineStr">
         <is>
-          <t>160 g chicken, iceberg lettuce, croutons, parmesan, Caesar dressing (mayonnaise, mustard, capers, anchovy)</t>
+          <t>160 g chicken (marinated in olive oil, fresh thyme and sweet paprika), iceberg lettuce, croutons, parmesan, Caesar dressing (mayonnaise, mustard, capers, anchovy)</t>
         </is>
       </c>
       <c r="H27" s="5" t="inlineStr">
@@ -2522,7 +2553,8 @@
       </c>
       <c r="Z27" s="8" t="inlineStr"/>
       <c r="AA27" s="8" t="inlineStr"/>
-      <c r="AB27" s="9" t="inlineStr"/>
+      <c r="AB27" s="8" t="inlineStr"/>
+      <c r="AC27" s="9" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2550,20 +2582,36 @@
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>160 g Cajun tavuk, taze yeşillikler, ballı hardal sos</t>
+          <t>160 g Cajun tavuk (yumurta, süt, un, pane, galeta unu, soya sosu, Cajun baharatı, tuz), taze yeşillikler, ballı hardal sos</t>
         </is>
       </c>
       <c r="G28" s="4" t="inlineStr">
         <is>
-          <t>160 g Cajun chicken, fresh greens, honey mustard dressing</t>
-        </is>
-      </c>
-      <c r="H28" s="5" t="inlineStr"/>
-      <c r="I28" s="5" t="inlineStr"/>
-      <c r="J28" s="5" t="inlineStr"/>
+          <t>160 g Cajun chicken (egg, milk, flour, breading, breadcrumbs, soy sauce, Cajun spice, salt), fresh greens, honey mustard dressing</t>
+        </is>
+      </c>
+      <c r="H28" s="5" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I28" s="5" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J28" s="5" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="K28" s="5" t="inlineStr"/>
       <c r="L28" s="5" t="inlineStr"/>
-      <c r="M28" s="5" t="inlineStr"/>
+      <c r="M28" s="5" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="N28" s="5" t="inlineStr"/>
       <c r="O28" s="5" t="inlineStr"/>
       <c r="P28" s="5" t="inlineStr"/>
@@ -2577,20 +2625,21 @@
       <c r="T28" s="5" t="inlineStr"/>
       <c r="U28" s="5" t="inlineStr"/>
       <c r="V28" s="6" t="n">
-        <v>430</v>
+        <v>560</v>
       </c>
       <c r="W28" s="7" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="X28" s="7" t="n">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="Y28" s="7" t="n">
-        <v>18</v>
+        <v>34</v>
       </c>
       <c r="Z28" s="8" t="inlineStr"/>
       <c r="AA28" s="8" t="inlineStr"/>
-      <c r="AB28" s="9" t="inlineStr"/>
+      <c r="AB28" s="8" t="inlineStr"/>
+      <c r="AC28" s="9" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2618,12 +2667,12 @@
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>200 g spagetti, dana kıyma, domates sos (salça, domates, karabiber, tuz), fesleğenli pesto sos, parmesan</t>
+          <t>200 g spagetti, dana kıyma, domates sos (domates, salça, tuz, karabiber), fesleğenli pesto sos, parmesan, ayçiçek yağı</t>
         </is>
       </c>
       <c r="G29" s="4" t="inlineStr">
         <is>
-          <t>200 g spaghetti, minced beef, tomato sauce (tomato paste, tomato, black pepper, salt), basil pesto, parmesan</t>
+          <t>200 g spaghetti, minced beef, tomato sauce (tomato, tomato paste, salt, black pepper), basil pesto, parmesan, sunflower oil</t>
         </is>
       </c>
       <c r="H29" s="5" t="inlineStr">
@@ -2666,7 +2715,8 @@
       </c>
       <c r="Z29" s="8" t="inlineStr"/>
       <c r="AA29" s="8" t="inlineStr"/>
-      <c r="AB29" s="9" t="inlineStr"/>
+      <c r="AB29" s="8" t="inlineStr"/>
+      <c r="AC29" s="9" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2694,12 +2744,12 @@
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>200 g makarna, cheddar, kaşar, krema, tereyağı</t>
+          <t>200 g makarna, cheddar, kaşar, krema, tereyağı, ayçiçek yağı</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t>200 g macaroni, cheddar, kashar cheese, cream, butter</t>
+          <t>200 g macaroni, cheddar, kashar cheese, cream, butter, sunflower oil</t>
         </is>
       </c>
       <c r="H30" s="5" t="inlineStr">
@@ -2738,7 +2788,8 @@
       </c>
       <c r="Z30" s="8" t="inlineStr"/>
       <c r="AA30" s="8" t="inlineStr"/>
-      <c r="AB30" s="9" t="inlineStr"/>
+      <c r="AB30" s="8" t="inlineStr"/>
+      <c r="AC30" s="9" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2766,12 +2817,12 @@
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>200 g penne, domates sos (salça, domates, karabiber, tuz), fesleğenli pesto sos, pul biber, siyah zeytin, zeytinyağı</t>
+          <t>200 g penne, domates sos (domates, salça, tuz, karabiber), fesleğenli pesto sos, acı sos, pul biber, siyah zeytin, zeytinyağı, ayçiçek yağı</t>
         </is>
       </c>
       <c r="G31" s="4" t="inlineStr">
         <is>
-          <t>200 g penne, tomato sauce (tomato paste, tomato, black pepper, salt), basil pesto, chilli flakes, black olives, olive oil</t>
+          <t>200 g penne, tomato sauce (tomato, tomato paste, salt, black pepper), basil pesto, hot sauce, chilli flakes, black olives, olive oil, sunflower oil</t>
         </is>
       </c>
       <c r="H31" s="5" t="inlineStr">
@@ -2814,7 +2865,8 @@
       </c>
       <c r="Z31" s="8" t="inlineStr"/>
       <c r="AA31" s="8" t="inlineStr"/>
-      <c r="AB31" s="9" t="inlineStr"/>
+      <c r="AB31" s="8" t="inlineStr"/>
+      <c r="AC31" s="9" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2842,12 +2894,12 @@
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>200 g fettuccine, 80 g tavuk, krema, parmesan, tereyağı, mantar, tuz, karabiber</t>
+          <t>200 g fettuccine, 80 g tavuk, krema, parmesan, tereyağı, mantar, tuz, karabiber, ayçiçek yağı</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr">
         <is>
-          <t>200 g fettuccine, 80 g chicken, cream, parmesan, butter, mushroom, salt, black pepper</t>
+          <t>200 g fettuccine, 80 g chicken, cream, parmesan, butter, mushroom, salt, black pepper, sunflower oil</t>
         </is>
       </c>
       <c r="H32" s="5" t="inlineStr">
@@ -2890,7 +2942,8 @@
       </c>
       <c r="Z32" s="8" t="inlineStr"/>
       <c r="AA32" s="8" t="inlineStr"/>
-      <c r="AB32" s="9" t="inlineStr"/>
+      <c r="AB32" s="8" t="inlineStr"/>
+      <c r="AC32" s="9" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2918,12 +2971,12 @@
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>200 g noodle, renkli biber, havuç, soya filizi, soya sos, susam yağı, susam</t>
+          <t>200 g noodle, renkli biber, havuç, kabak, soya filizi, soya sos, susam yağı, susam, ayçiçek yağı</t>
         </is>
       </c>
       <c r="G33" s="4" t="inlineStr">
         <is>
-          <t>200 g noodles, bell peppers, carrot, bean sprouts, soy sauce, sesame oil, sesame</t>
+          <t>200 g noodles, bell peppers, carrot, courgette, bean sprouts, soy sauce, sesame oil, sesame, sunflower oil</t>
         </is>
       </c>
       <c r="H33" s="5" t="inlineStr">
@@ -2970,7 +3023,8 @@
       </c>
       <c r="Z33" s="8" t="inlineStr"/>
       <c r="AA33" s="8" t="inlineStr"/>
-      <c r="AB33" s="9" t="inlineStr"/>
+      <c r="AB33" s="8" t="inlineStr"/>
+      <c r="AC33" s="9" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2998,12 +3052,12 @@
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>200 g noodle, 80 g tavuk, renkli biber, havuç, soya filizi, soya sos, susam yağı, susam</t>
+          <t>200 g noodle, 80 g tavuk, renkli biber, havuç, kabak, soya filizi, soya sos, susam yağı, susam, ayçiçek yağı</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr">
         <is>
-          <t>200 g noodles, 80 g chicken, bell peppers, carrot, bean sprouts, soy sauce, sesame oil, sesame</t>
+          <t>200 g noodles, 80 g chicken, bell peppers, carrot, courgette, bean sprouts, soy sauce, sesame oil, sesame, sunflower oil</t>
         </is>
       </c>
       <c r="H34" s="5" t="inlineStr">
@@ -3050,7 +3104,8 @@
       </c>
       <c r="Z34" s="8" t="inlineStr"/>
       <c r="AA34" s="8" t="inlineStr"/>
-      <c r="AB34" s="9" t="inlineStr"/>
+      <c r="AB34" s="8" t="inlineStr"/>
+      <c r="AC34" s="9" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -3078,12 +3133,12 @@
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>180 g burger köftesi, kıvırcık, domates, turşu, mantar sos (mantar, krema, tuz, karabiber), patates</t>
+          <t>180 g burger köftesi, kıvırcık, domates, turşu, mantar sos (mantar, krema, tuz, karabiber), hamburger sosu (mayonez, Sweet Chili sos, az acı, tuz, pul biber), patates ve Sweet Chili sos eşliğinde</t>
         </is>
       </c>
       <c r="G35" s="4" t="inlineStr">
         <is>
-          <t>180 g beef patty, lettuce, tomato, pickles, mushroom sauce (mushroom, cream, salt, black pepper), fries</t>
+          <t>180 g beef patty, lettuce, tomato, pickles, mushroom sauce (mushroom, cream, salt, black pepper), burger sauce (mayonnaise, sweet chilli sauce, mild chilli, salt, chilli flakes), served with fries and sweet chilli sauce</t>
         </is>
       </c>
       <c r="H35" s="5" t="inlineStr">
@@ -3117,20 +3172,25 @@
       <c r="T35" s="5" t="inlineStr"/>
       <c r="U35" s="5" t="inlineStr"/>
       <c r="V35" s="6" t="n">
-        <v>1060</v>
+        <v>1130</v>
       </c>
       <c r="W35" s="7" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="X35" s="7" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="Y35" s="7" t="n">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="Z35" s="8" t="inlineStr"/>
       <c r="AA35" s="8" t="inlineStr"/>
-      <c r="AB35" s="9" t="inlineStr"/>
+      <c r="AB35" s="8" t="inlineStr">
+        <is>
+          <t>sweetchili</t>
+        </is>
+      </c>
+      <c r="AC35" s="9" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -3158,12 +3218,12 @@
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>180 g burger köftesi, kıvırcık, domates, turşu, cheddar peyniri, patates</t>
+          <t>180 g burger köftesi, kıvırcık, domates, turşu, cheddar peyniri, hamburger sosu (mayonez, Sweet Chili sos, az acı, tuz, pul biber), patates ve Sweet Chili sos eşliğinde</t>
         </is>
       </c>
       <c r="G36" s="4" t="inlineStr">
         <is>
-          <t>180 g beef patty, lettuce, tomato, pickles, cheddar, fries</t>
+          <t>180 g beef patty, lettuce, tomato, pickles, cheddar, burger sauce (mayonnaise, sweet chilli sauce, mild chilli, salt, chilli flakes), served with fries and sweet chilli sauce</t>
         </is>
       </c>
       <c r="H36" s="5" t="inlineStr">
@@ -3176,7 +3236,11 @@
           <t>X</t>
         </is>
       </c>
-      <c r="J36" s="5" t="inlineStr"/>
+      <c r="J36" s="5" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="K36" s="5" t="inlineStr"/>
       <c r="L36" s="5" t="inlineStr"/>
       <c r="M36" s="5" t="inlineStr"/>
@@ -3193,20 +3257,25 @@
       <c r="T36" s="5" t="inlineStr"/>
       <c r="U36" s="5" t="inlineStr"/>
       <c r="V36" s="6" t="n">
-        <v>1080</v>
+        <v>1150</v>
       </c>
       <c r="W36" s="7" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="X36" s="7" t="n">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="Y36" s="7" t="n">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="Z36" s="8" t="inlineStr"/>
       <c r="AA36" s="8" t="inlineStr"/>
-      <c r="AB36" s="9" t="inlineStr"/>
+      <c r="AB36" s="8" t="inlineStr">
+        <is>
+          <t>sweetchili</t>
+        </is>
+      </c>
+      <c r="AC36" s="9" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -3234,12 +3303,12 @@
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>360 g burger köftesi, kıvırcık, domates, turşu, cheddar peyniri, patates</t>
+          <t>360 g burger köftesi, kıvırcık, domates, turşu, cheddar peyniri, hamburger sosu (mayonez, Sweet Chili sos, az acı, tuz, pul biber), patates ve Sweet Chili sos eşliğinde</t>
         </is>
       </c>
       <c r="G37" s="4" t="inlineStr">
         <is>
-          <t>360 g beef patty, lettuce, tomato, pickles, cheddar, fries</t>
+          <t>360 g beef patty, lettuce, tomato, pickles, cheddar, burger sauce (mayonnaise, sweet chilli sauce, mild chilli, salt, chilli flakes), served with fries and sweet chilli sauce</t>
         </is>
       </c>
       <c r="H37" s="5" t="inlineStr">
@@ -3252,7 +3321,11 @@
           <t>X</t>
         </is>
       </c>
-      <c r="J37" s="5" t="inlineStr"/>
+      <c r="J37" s="5" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="K37" s="5" t="inlineStr"/>
       <c r="L37" s="5" t="inlineStr"/>
       <c r="M37" s="5" t="inlineStr"/>
@@ -3269,20 +3342,25 @@
       <c r="T37" s="5" t="inlineStr"/>
       <c r="U37" s="5" t="inlineStr"/>
       <c r="V37" s="6" t="n">
-        <v>1450</v>
+        <v>1520</v>
       </c>
       <c r="W37" s="7" t="n">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="X37" s="7" t="n">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="Y37" s="7" t="n">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="Z37" s="8" t="inlineStr"/>
       <c r="AA37" s="8" t="inlineStr"/>
-      <c r="AB37" s="9" t="inlineStr"/>
+      <c r="AB37" s="8" t="inlineStr">
+        <is>
+          <t>sweetchili</t>
+        </is>
+      </c>
+      <c r="AC37" s="9" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -3310,12 +3388,12 @@
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>180 g özel soslu tavuk (yumurta, un, süt, soya sosu, tuz, karabiber, Cajun baharatı), kıvırcık, domates, turşu, cheddar peyniri, patates</t>
+          <t>180 g özel soslu tavuk (yumurta, un, süt, panko, galeta unu, pane, soya sosu, tuz, karabiber, Cajun baharatı), kıvırcık, domates, turşu, cheddar peyniri, hamburger sosu (mayonez, Sweet Chili sos, az acı, tuz, pul biber), patates ve Sweet Chili sos eşliğinde</t>
         </is>
       </c>
       <c r="G38" s="4" t="inlineStr">
         <is>
-          <t>180 g chicken in special sauce (egg, flour, milk, soy sauce, salt, black pepper, Cajun spice), lettuce, tomato, pickles, cheddar, fries</t>
+          <t>180 g chicken in special coating (egg, flour, milk, panko, breadcrumbs, breading, soy sauce, salt, black pepper, Cajun spice), lettuce, tomato, pickles, cheddar, burger sauce (mayonnaise, sweet chilli sauce, mild chilli, salt, chilli flakes), served with fries and sweet chilli sauce</t>
         </is>
       </c>
       <c r="H38" s="5" t="inlineStr">
@@ -3353,20 +3431,25 @@
       <c r="T38" s="5" t="inlineStr"/>
       <c r="U38" s="5" t="inlineStr"/>
       <c r="V38" s="6" t="n">
-        <v>1000</v>
+        <v>1090</v>
       </c>
       <c r="W38" s="7" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="X38" s="7" t="n">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="Y38" s="7" t="n">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="Z38" s="8" t="inlineStr"/>
       <c r="AA38" s="8" t="inlineStr"/>
-      <c r="AB38" s="9" t="inlineStr"/>
+      <c r="AB38" s="8" t="inlineStr">
+        <is>
+          <t>sweetchili</t>
+        </is>
+      </c>
+      <c r="AC38" s="9" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -3394,12 +3477,12 @@
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>170 g jülyen et, soğan, renkli biberler, özel sos, patates</t>
+          <t>170 g jülyen et, soğan, renkli biberler, kaşar peyniri, özel sos (soya sosu, Cajun baharatı), patates ve Sweet Chili sos eşliğinde</t>
         </is>
       </c>
       <c r="G39" s="4" t="inlineStr">
         <is>
-          <t>170 g julienne beef, onion, bell peppers, special sauce, fries</t>
+          <t>170 g julienne beef, onion, bell peppers, kashar cheese, special sauce (soy sauce, Cajun spice), served with fries and sweet chilli sauce</t>
         </is>
       </c>
       <c r="H39" s="5" t="inlineStr">
@@ -3419,7 +3502,11 @@
       </c>
       <c r="K39" s="5" t="inlineStr"/>
       <c r="L39" s="5" t="inlineStr"/>
-      <c r="M39" s="5" t="inlineStr"/>
+      <c r="M39" s="5" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="N39" s="5" t="inlineStr"/>
       <c r="O39" s="5" t="inlineStr"/>
       <c r="P39" s="5" t="inlineStr"/>
@@ -3429,20 +3516,25 @@
       <c r="T39" s="5" t="inlineStr"/>
       <c r="U39" s="5" t="inlineStr"/>
       <c r="V39" s="6" t="n">
-        <v>900</v>
+        <v>1000</v>
       </c>
       <c r="W39" s="7" t="n">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="X39" s="7" t="n">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="Y39" s="7" t="n">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="Z39" s="8" t="inlineStr"/>
       <c r="AA39" s="8" t="inlineStr"/>
-      <c r="AB39" s="9" t="inlineStr"/>
+      <c r="AB39" s="8" t="inlineStr">
+        <is>
+          <t>sweetchili</t>
+        </is>
+      </c>
+      <c r="AC39" s="9" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -3470,12 +3562,12 @@
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>170 g jülyen tavuk, soğan, renkli biberler, Sweet Chili sos, patates</t>
+          <t>170 g jülyen tavuk, soğan, renkli biberler, kaşar peyniri, özel sos (soya sosu, Cajun baharatı), patates ve Sweet Chili sos eşliğinde</t>
         </is>
       </c>
       <c r="G40" s="4" t="inlineStr">
         <is>
-          <t>170 g julienne chicken, onion, bell peppers, sweet chilli sauce, fries</t>
+          <t>170 g julienne chicken, onion, bell peppers, kashar cheese, special sauce (soy sauce, Cajun spice), served with fries and sweet chilli sauce</t>
         </is>
       </c>
       <c r="H40" s="5" t="inlineStr">
@@ -3483,11 +3575,19 @@
           <t>X</t>
         </is>
       </c>
-      <c r="I40" s="5" t="inlineStr"/>
+      <c r="I40" s="5" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="J40" s="5" t="inlineStr"/>
       <c r="K40" s="5" t="inlineStr"/>
       <c r="L40" s="5" t="inlineStr"/>
-      <c r="M40" s="5" t="inlineStr"/>
+      <c r="M40" s="5" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="N40" s="5" t="inlineStr"/>
       <c r="O40" s="5" t="inlineStr"/>
       <c r="P40" s="5" t="inlineStr"/>
@@ -3497,20 +3597,25 @@
       <c r="T40" s="5" t="inlineStr"/>
       <c r="U40" s="5" t="inlineStr"/>
       <c r="V40" s="6" t="n">
-        <v>830</v>
+        <v>930</v>
       </c>
       <c r="W40" s="7" t="n">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="X40" s="7" t="n">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="Y40" s="7" t="n">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="Z40" s="8" t="inlineStr"/>
       <c r="AA40" s="8" t="inlineStr"/>
-      <c r="AB40" s="9" t="inlineStr"/>
+      <c r="AB40" s="8" t="inlineStr">
+        <is>
+          <t>sweetchili</t>
+        </is>
+      </c>
+      <c r="AC40" s="9" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -3538,12 +3643,12 @@
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>170 g köfte, soğan, renkli biberler, kaşar peyniri, soya sosu, patates</t>
+          <t>170 g köfte, soğan, renkli biberler, kaşar peyniri, özel sos (soya sosu, Cajun baharatı), patates ve Sweet Chili sos eşliğinde</t>
         </is>
       </c>
       <c r="G41" s="4" t="inlineStr">
         <is>
-          <t>170 g meatballs, onion, bell peppers, kashar cheese, soy sauce, fries</t>
+          <t>170 g meatballs, onion, bell peppers, kashar cheese, special sauce (soy sauce, Cajun spice), served with fries and sweet chilli sauce</t>
         </is>
       </c>
       <c r="H41" s="5" t="inlineStr">
@@ -3573,20 +3678,25 @@
       <c r="T41" s="5" t="inlineStr"/>
       <c r="U41" s="5" t="inlineStr"/>
       <c r="V41" s="6" t="n">
-        <v>950</v>
+        <v>1010</v>
       </c>
       <c r="W41" s="7" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="X41" s="7" t="n">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="Y41" s="7" t="n">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="Z41" s="8" t="inlineStr"/>
       <c r="AA41" s="8" t="inlineStr"/>
-      <c r="AB41" s="9" t="inlineStr"/>
+      <c r="AB41" s="8" t="inlineStr">
+        <is>
+          <t>sweetchili</t>
+        </is>
+      </c>
+      <c r="AC41" s="9" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -3614,12 +3724,12 @@
       </c>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t>180 g anne köfte, közlenmiş biber &amp; domates, pilav ve patates</t>
+          <t>180 g anne köfte, lavaş, közlenmiş biber &amp; domates, pilav ve patates eşliğinde</t>
         </is>
       </c>
       <c r="G42" s="4" t="inlineStr">
         <is>
-          <t>180 g homestyle meatballs, roasted pepper &amp; tomato, rice and fries</t>
+          <t>180 g homestyle meatballs, lavash, served with roasted pepper &amp; tomato, rice and fries</t>
         </is>
       </c>
       <c r="H42" s="5" t="inlineStr">
@@ -3641,20 +3751,21 @@
       <c r="T42" s="5" t="inlineStr"/>
       <c r="U42" s="5" t="inlineStr"/>
       <c r="V42" s="6" t="n">
-        <v>820</v>
+        <v>900</v>
       </c>
       <c r="W42" s="7" t="n">
+        <v>47</v>
+      </c>
+      <c r="X42" s="7" t="n">
         <v>44</v>
       </c>
-      <c r="X42" s="7" t="n">
-        <v>42</v>
-      </c>
       <c r="Y42" s="7" t="n">
-        <v>66</v>
+        <v>80</v>
       </c>
       <c r="Z42" s="8" t="inlineStr"/>
       <c r="AA42" s="8" t="inlineStr"/>
-      <c r="AB42" s="9" t="inlineStr"/>
+      <c r="AB42" s="8" t="inlineStr"/>
+      <c r="AC42" s="9" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -3682,12 +3793,12 @@
       </c>
       <c r="F43" s="4" t="inlineStr">
         <is>
-          <t>180 g özel soslu köfte, süzme yoğurt, közlenmiş biber &amp; domates, patates</t>
+          <t>180 g köfte, domates sos (domates, salça, tuz, karabiber), süzme yoğurt, közlenmiş biber &amp; domates, patates eşliğinde</t>
         </is>
       </c>
       <c r="G43" s="4" t="inlineStr">
         <is>
-          <t>180 g meatballs in special sauce, strained yoghurt, roasted pepper &amp; tomato, fries</t>
+          <t>180 g meatballs, tomato sauce (tomato, tomato paste, salt, black pepper), strained yoghurt, roasted pepper &amp; tomato, served with fries</t>
         </is>
       </c>
       <c r="H43" s="5" t="inlineStr">
@@ -3726,7 +3837,8 @@
       </c>
       <c r="Z43" s="8" t="inlineStr"/>
       <c r="AA43" s="8" t="inlineStr"/>
-      <c r="AB43" s="9" t="inlineStr"/>
+      <c r="AB43" s="8" t="inlineStr"/>
+      <c r="AC43" s="9" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -3754,12 +3866,12 @@
       </c>
       <c r="F44" s="4" t="inlineStr">
         <is>
-          <t>180 g köfte, patlıcan beğendi, közlenmiş biber &amp; domates, patates</t>
+          <t>180 g köfte, patlıcan beğendi (süt, kaşar peyniri, tuz, karabiber), közlenmiş biber &amp; domates, patates eşliğinde</t>
         </is>
       </c>
       <c r="G44" s="4" t="inlineStr">
         <is>
-          <t>180 g meatballs, smoked aubergine purée, roasted pepper &amp; tomato, fries</t>
+          <t>180 g meatballs, smoked aubergine purée (milk, kashar cheese, salt, black pepper), roasted pepper &amp; tomato, served with fries</t>
         </is>
       </c>
       <c r="H44" s="5" t="inlineStr">
@@ -3798,7 +3910,8 @@
       </c>
       <c r="Z44" s="8" t="inlineStr"/>
       <c r="AA44" s="8" t="inlineStr"/>
-      <c r="AB44" s="9" t="inlineStr"/>
+      <c r="AB44" s="8" t="inlineStr"/>
+      <c r="AC44" s="9" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -3826,12 +3939,12 @@
       </c>
       <c r="F45" s="4" t="inlineStr">
         <is>
-          <t>180 g tavuk, süzme yoğurt, çıtır yufka, közlenmiş biber &amp; domates, özel kaymak sos (kaymak, tereyağı, barbekü sos), patates</t>
+          <t>180 g tavuk, süzme yoğurt, çıtır yufka, közlenmiş biber &amp; domates, özel kaymak sos (kaymak, tereyağı, barbekü sos), pilav eşliğinde</t>
         </is>
       </c>
       <c r="G45" s="4" t="inlineStr">
         <is>
-          <t>180 g chicken, strained yoghurt, crispy yufka, roasted pepper &amp; tomato, special cream sauce (clotted cream, butter, BBQ sauce), fries</t>
+          <t>180 g chicken, strained yoghurt, crispy yufka, roasted pepper &amp; tomato, special cream sauce (clotted cream, butter, BBQ sauce), served with rice</t>
         </is>
       </c>
       <c r="H45" s="5" t="inlineStr">
@@ -3857,20 +3970,21 @@
       <c r="T45" s="5" t="inlineStr"/>
       <c r="U45" s="5" t="inlineStr"/>
       <c r="V45" s="6" t="n">
-        <v>860</v>
+        <v>880</v>
       </c>
       <c r="W45" s="7" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="X45" s="7" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="Y45" s="7" t="n">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="Z45" s="8" t="inlineStr"/>
       <c r="AA45" s="8" t="inlineStr"/>
-      <c r="AB45" s="9" t="inlineStr"/>
+      <c r="AB45" s="8" t="inlineStr"/>
+      <c r="AC45" s="9" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -3898,12 +4012,12 @@
       </c>
       <c r="F46" s="4" t="inlineStr">
         <is>
-          <t>180 g tavuk, renkli biberler, mantar, köri sos, pilav ve patates</t>
+          <t>180 g tavuk, renkli biberler, mantar, köri sos, krema, tuz, karabiber, pilav ve patates eşliğinde</t>
         </is>
       </c>
       <c r="G46" s="4" t="inlineStr">
         <is>
-          <t>180 g chicken, bell peppers, mushroom, curry sauce, rice and fries</t>
+          <t>180 g chicken, bell peppers, mushroom, curry sauce, cream, salt, black pepper, served with rice and fries</t>
         </is>
       </c>
       <c r="H46" s="5" t="inlineStr"/>
@@ -3925,20 +4039,21 @@
       <c r="T46" s="5" t="inlineStr"/>
       <c r="U46" s="5" t="inlineStr"/>
       <c r="V46" s="6" t="n">
-        <v>780</v>
+        <v>830</v>
       </c>
       <c r="W46" s="7" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="X46" s="7" t="n">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="Y46" s="7" t="n">
         <v>66</v>
       </c>
       <c r="Z46" s="8" t="inlineStr"/>
       <c r="AA46" s="8" t="inlineStr"/>
-      <c r="AB46" s="9" t="inlineStr"/>
+      <c r="AB46" s="8" t="inlineStr"/>
+      <c r="AC46" s="9" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -3966,16 +4081,20 @@
       </c>
       <c r="F47" s="4" t="inlineStr">
         <is>
-          <t>180 g tavuk, BBQ sos, renkli biberler, mantar, pilav ve patates</t>
+          <t>180 g tavuk, barbekü sos (barbekü, krema, tuz, karabiber), renkli biberler, mantar, krema, tuz, karabiber, pilav ve patates eşliğinde</t>
         </is>
       </c>
       <c r="G47" s="4" t="inlineStr">
         <is>
-          <t>180 g chicken, BBQ sauce, bell peppers, mushroom, rice and fries</t>
+          <t>180 g chicken, BBQ sauce (BBQ, cream, salt, black pepper), bell peppers, mushroom, cream, salt, black pepper, served with rice and fries</t>
         </is>
       </c>
       <c r="H47" s="5" t="inlineStr"/>
-      <c r="I47" s="5" t="inlineStr"/>
+      <c r="I47" s="5" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="J47" s="5" t="inlineStr"/>
       <c r="K47" s="5" t="inlineStr"/>
       <c r="L47" s="5" t="inlineStr"/>
@@ -3989,20 +4108,21 @@
       <c r="T47" s="5" t="inlineStr"/>
       <c r="U47" s="5" t="inlineStr"/>
       <c r="V47" s="6" t="n">
-        <v>760</v>
+        <v>820</v>
       </c>
       <c r="W47" s="7" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="X47" s="7" t="n">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="Y47" s="7" t="n">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="Z47" s="8" t="inlineStr"/>
       <c r="AA47" s="8" t="inlineStr"/>
-      <c r="AB47" s="9" t="inlineStr"/>
+      <c r="AB47" s="8" t="inlineStr"/>
+      <c r="AC47" s="9" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -4030,12 +4150,12 @@
       </c>
       <c r="F48" s="4" t="inlineStr">
         <is>
-          <t>180 g tavuk, renkli biberler, soğan, domates, sarımsak, pilav ve patates</t>
+          <t>180 g tavuk, renkli biberler, soğan, domates, sarımsak, tuz, karabiber, pilav ve patates eşliğinde</t>
         </is>
       </c>
       <c r="G48" s="4" t="inlineStr">
         <is>
-          <t>180 g chicken, bell peppers, onion, tomato, garlic, rice and fries</t>
+          <t>180 g chicken, bell peppers, onion, tomato, garlic, salt, black pepper, served with rice and fries</t>
         </is>
       </c>
       <c r="H48" s="5" t="inlineStr"/>
@@ -4066,7 +4186,8 @@
       </c>
       <c r="Z48" s="8" t="inlineStr"/>
       <c r="AA48" s="8" t="inlineStr"/>
-      <c r="AB48" s="9" t="inlineStr"/>
+      <c r="AB48" s="8" t="inlineStr"/>
+      <c r="AC48" s="9" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -4094,12 +4215,12 @@
       </c>
       <c r="F49" s="4" t="inlineStr">
         <is>
-          <t>180 g tavuk but, közlenmiş biber &amp; domates, pilav ve patates</t>
+          <t>180 g tavuk but (taze kekik, kırmızı tatlı toz biber, pul biber ile marine edilmiş), közlenmiş biber &amp; domates, pilav ve patates eşliğinde</t>
         </is>
       </c>
       <c r="G49" s="4" t="inlineStr">
         <is>
-          <t>180 g chicken thigh, roasted pepper &amp; tomato, rice and fries</t>
+          <t>180 g chicken thigh (marinated in fresh thyme, sweet paprika and chilli flakes), served with roasted pepper &amp; tomato, rice and fries</t>
         </is>
       </c>
       <c r="H49" s="5" t="inlineStr"/>
@@ -4130,7 +4251,8 @@
       </c>
       <c r="Z49" s="8" t="inlineStr"/>
       <c r="AA49" s="8" t="inlineStr"/>
-      <c r="AB49" s="9" t="inlineStr"/>
+      <c r="AB49" s="8" t="inlineStr"/>
+      <c r="AC49" s="9" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -4158,12 +4280,12 @@
       </c>
       <c r="F50" s="4" t="inlineStr">
         <is>
-          <t>180 g marine edilmiş tavuk göğsü, patlıcan beğendi, közlenmiş biber &amp; domates, patates</t>
+          <t>180 g marine edilmiş tavuk göğsü (taze kekik, kırmızı tatlı toz biber, pul biber), patlıcan beğendi (süt, kaşar peyniri, tuz, karabiber), közlenmiş biber &amp; domates, patates eşliğinde</t>
         </is>
       </c>
       <c r="G50" s="4" t="inlineStr">
         <is>
-          <t>180 g marinated chicken breast, smoked aubergine purée, roasted pepper &amp; tomato, fries</t>
+          <t>180 g marinated chicken breast (fresh thyme, sweet paprika, chilli flakes), smoked aubergine purée (milk, kashar cheese, salt, black pepper), roasted pepper &amp; tomato, served with fries</t>
         </is>
       </c>
       <c r="H50" s="5" t="inlineStr"/>
@@ -4198,7 +4320,8 @@
       </c>
       <c r="Z50" s="8" t="inlineStr"/>
       <c r="AA50" s="8" t="inlineStr"/>
-      <c r="AB50" s="9" t="inlineStr"/>
+      <c r="AB50" s="8" t="inlineStr"/>
+      <c r="AC50" s="9" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -4226,12 +4349,12 @@
       </c>
       <c r="F51" s="4" t="inlineStr">
         <is>
-          <t>200 g panelenmiş tavuk, schnitzel sosu (galeta unu, pane, yumurta, un, soya sosu, tuz, Cajun baharatı), mini salata, patates</t>
+          <t>180 g panelenmiş tavuk (pane, galeta unu), schnitzel sosu (galeta unu, pane, yumurta, un, soya sosu, tuz, Cajun baharatı), mini salata, patates eşliğinde</t>
         </is>
       </c>
       <c r="G51" s="4" t="inlineStr">
         <is>
-          <t>200 g breaded chicken, schnitzel coating (breadcrumbs, breading, egg, flour, soy sauce, salt, Cajun spice), side salad, fries</t>
+          <t>180 g breaded chicken (breading, breadcrumbs), schnitzel coating (breadcrumbs, breading, egg, flour, soy sauce, salt, Cajun spice), side salad, served with fries</t>
         </is>
       </c>
       <c r="H51" s="5" t="inlineStr">
@@ -4261,20 +4384,21 @@
       <c r="T51" s="5" t="inlineStr"/>
       <c r="U51" s="5" t="inlineStr"/>
       <c r="V51" s="6" t="n">
-        <v>820</v>
+        <v>780</v>
       </c>
       <c r="W51" s="7" t="n">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="X51" s="7" t="n">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="Y51" s="7" t="n">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="Z51" s="8" t="inlineStr"/>
       <c r="AA51" s="8" t="inlineStr"/>
-      <c r="AB51" s="9" t="inlineStr"/>
+      <c r="AB51" s="8" t="inlineStr"/>
+      <c r="AC51" s="9" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -4302,12 +4426,12 @@
       </c>
       <c r="F52" s="4" t="inlineStr">
         <is>
-          <t>180 g panelenmiş tavuk, schnitzel sosu (galeta unu, pane, yumurta, un, soya sosu, tuz, Cajun baharatı), mantar sos, mini salata, patates</t>
+          <t>180 g panelenmiş tavuk (pane, galeta unu), schnitzel sosu (galeta unu, pane, yumurta, un, soya sosu, tuz, Cajun baharatı), mantar sos, mini salata, patates eşliğinde</t>
         </is>
       </c>
       <c r="G52" s="4" t="inlineStr">
         <is>
-          <t>180 g breaded chicken, schnitzel coating (breadcrumbs, breading, egg, flour, soy sauce, salt, Cajun spice), mushroom sauce, side salad, fries</t>
+          <t>180 g breaded chicken (breading, breadcrumbs), schnitzel coating (breadcrumbs, breading, egg, flour, soy sauce, salt, Cajun spice), mushroom sauce, side salad, served with fries</t>
         </is>
       </c>
       <c r="H52" s="5" t="inlineStr">
@@ -4354,7 +4478,8 @@
       </c>
       <c r="Z52" s="8" t="inlineStr"/>
       <c r="AA52" s="8" t="inlineStr"/>
-      <c r="AB52" s="9" t="inlineStr"/>
+      <c r="AB52" s="8" t="inlineStr"/>
+      <c r="AC52" s="9" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -4382,12 +4507,12 @@
       </c>
       <c r="F53" s="4" t="inlineStr">
         <is>
-          <t>180 g panelenmiş tavuk, schnitzel sosu (galeta unu, pane, yumurta, un, soya sosu, tuz, Cajun baharatı), cheddar sos, krema, mini salata, patates</t>
+          <t>180 g panelenmiş tavuk (pane, galeta unu), schnitzel sosu (galeta unu, pane, yumurta, un, soya sosu, tuz, Cajun baharatı), cheddar sos (cheddar, krema), mini salata, patates eşliğinde</t>
         </is>
       </c>
       <c r="G53" s="4" t="inlineStr">
         <is>
-          <t>180 g breaded chicken, schnitzel coating (breadcrumbs, breading, egg, flour, soy sauce, salt, Cajun spice), cheddar sauce, cream, side salad, fries</t>
+          <t>180 g breaded chicken (breading, breadcrumbs), schnitzel coating (breadcrumbs, breading, egg, flour, soy sauce, salt, Cajun spice), cheddar sauce (cheddar, cream), side salad, served with fries</t>
         </is>
       </c>
       <c r="H53" s="5" t="inlineStr">
@@ -4434,7 +4559,8 @@
       </c>
       <c r="Z53" s="8" t="inlineStr"/>
       <c r="AA53" s="8" t="inlineStr"/>
-      <c r="AB53" s="9" t="inlineStr"/>
+      <c r="AB53" s="8" t="inlineStr"/>
+      <c r="AC53" s="9" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -4462,15 +4588,19 @@
       </c>
       <c r="F54" s="4" t="inlineStr">
         <is>
-          <t>180 g tavuk parçaları, Cafe de Paris sos</t>
+          <t>180 g tavuk parçaları, Cafe de Paris sos, krema</t>
         </is>
       </c>
       <c r="G54" s="4" t="inlineStr">
         <is>
-          <t>180 g chicken pieces, Café de Paris sauce</t>
-        </is>
-      </c>
-      <c r="H54" s="5" t="inlineStr"/>
+          <t>180 g chicken pieces, Café de Paris sauce, cream</t>
+        </is>
+      </c>
+      <c r="H54" s="5" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="I54" s="5" t="inlineStr">
         <is>
           <t>X</t>
@@ -4493,20 +4623,25 @@
       <c r="T54" s="5" t="inlineStr"/>
       <c r="U54" s="5" t="inlineStr"/>
       <c r="V54" s="6" t="n">
-        <v>560</v>
+        <v>600</v>
       </c>
       <c r="W54" s="7" t="n">
+        <v>43</v>
+      </c>
+      <c r="X54" s="7" t="n">
         <v>42</v>
       </c>
-      <c r="X54" s="7" t="n">
-        <v>38</v>
-      </c>
       <c r="Y54" s="7" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="Z54" s="8" t="inlineStr"/>
       <c r="AA54" s="8" t="inlineStr"/>
-      <c r="AB54" s="9" t="inlineStr"/>
+      <c r="AB54" s="8" t="inlineStr">
+        <is>
+          <t>cafedeparis</t>
+        </is>
+      </c>
+      <c r="AC54" s="9" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -4534,12 +4669,12 @@
       </c>
       <c r="F55" s="4" t="inlineStr">
         <is>
-          <t>180 g tavuk parçaları, cheddar sos</t>
+          <t>180 g tavuk parçaları, cheddar sos, krema</t>
         </is>
       </c>
       <c r="G55" s="4" t="inlineStr">
         <is>
-          <t>180 g chicken pieces, cheddar sauce</t>
+          <t>180 g chicken pieces, cheddar sauce, cream</t>
         </is>
       </c>
       <c r="H55" s="5" t="inlineStr"/>
@@ -4561,20 +4696,21 @@
       <c r="T55" s="5" t="inlineStr"/>
       <c r="U55" s="5" t="inlineStr"/>
       <c r="V55" s="6" t="n">
-        <v>580</v>
+        <v>620</v>
       </c>
       <c r="W55" s="7" t="n">
+        <v>45</v>
+      </c>
+      <c r="X55" s="7" t="n">
         <v>44</v>
       </c>
-      <c r="X55" s="7" t="n">
-        <v>40</v>
-      </c>
       <c r="Y55" s="7" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="Z55" s="8" t="inlineStr"/>
       <c r="AA55" s="8" t="inlineStr"/>
-      <c r="AB55" s="9" t="inlineStr"/>
+      <c r="AB55" s="8" t="inlineStr"/>
+      <c r="AC55" s="9" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -4602,12 +4738,12 @@
       </c>
       <c r="F56" s="4" t="inlineStr">
         <is>
-          <t>180 g tavuk parçaları, Sweet Chili sos</t>
+          <t>180 g tavuk parçaları, Sweet Chili sos, maydanoz</t>
         </is>
       </c>
       <c r="G56" s="4" t="inlineStr">
         <is>
-          <t>180 g chicken pieces, sweet chilli sauce</t>
+          <t>180 g chicken pieces, sweet chilli sauce, parsley</t>
         </is>
       </c>
       <c r="H56" s="5" t="inlineStr">
@@ -4646,7 +4782,12 @@
       </c>
       <c r="Z56" s="8" t="inlineStr"/>
       <c r="AA56" s="8" t="inlineStr"/>
-      <c r="AB56" s="9" t="inlineStr"/>
+      <c r="AB56" s="8" t="inlineStr">
+        <is>
+          <t>sweetchili</t>
+        </is>
+      </c>
+      <c r="AC56" s="9" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -4674,12 +4815,12 @@
       </c>
       <c r="F57" s="4" t="inlineStr">
         <is>
-          <t>1 kuzu pirzola, 200 g antrikot, 2 köfte, 2 tavuk kanat, 1 tavuk bonfile (zeytinyağı ve kekikle marine edilmiş), közlenmiş biber &amp; domates, pilav ve patates</t>
+          <t>1 kuzu pirzola, 200 g antrikot, 2 köfte, 2 tavuk kanat, 1 tavuk bonfile (zeytinyağı, kekik ve pul biber ile marine edilmiş), közlenmiş biber &amp; domates, pilav ve patates eşliğinde</t>
         </is>
       </c>
       <c r="G57" s="4" t="inlineStr">
         <is>
-          <t>1 lamb chop, 200 g ribeye, 2 meatballs, 2 chicken wings, 1 chicken fillet (marinated in olive oil and thyme), roasted pepper &amp; tomato, rice and fries</t>
+          <t>1 lamb chop, 200 g ribeye, 2 meatballs, 2 chicken wings, 1 chicken fillet (marinated in olive oil, thyme and chilli flakes), served with roasted pepper &amp; tomato, rice and fries</t>
         </is>
       </c>
       <c r="H57" s="5" t="inlineStr">
@@ -4714,7 +4855,8 @@
       </c>
       <c r="Z57" s="8" t="inlineStr"/>
       <c r="AA57" s="8" t="inlineStr"/>
-      <c r="AB57" s="9" t="inlineStr"/>
+      <c r="AB57" s="8" t="inlineStr"/>
+      <c r="AC57" s="9" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -4742,12 +4884,12 @@
       </c>
       <c r="F58" s="4" t="inlineStr">
         <is>
-          <t>3 parça kuzu pirzola (zeytinyağı ve kekikle marine edilmiş), közlenmiş biber &amp; domates, pilav ve patates</t>
+          <t>3 parça kuzu pirzola (zeytinyağı, kekik ve pul biber ile marine edilmiş), közlenmiş biber &amp; domates, pilav ve patates eşliğinde</t>
         </is>
       </c>
       <c r="G58" s="4" t="inlineStr">
         <is>
-          <t>3 lamb chops (marinated in olive oil and thyme), roasted pepper &amp; tomato, rice and fries</t>
+          <t>3 lamb chops (marinated in olive oil, thyme and chilli flakes), served with roasted pepper &amp; tomato, rice and fries</t>
         </is>
       </c>
       <c r="H58" s="5" t="inlineStr"/>
@@ -4778,7 +4920,8 @@
       </c>
       <c r="Z58" s="8" t="inlineStr"/>
       <c r="AA58" s="8" t="inlineStr"/>
-      <c r="AB58" s="9" t="inlineStr"/>
+      <c r="AB58" s="8" t="inlineStr"/>
+      <c r="AC58" s="9" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -4806,12 +4949,12 @@
       </c>
       <c r="F59" s="4" t="inlineStr">
         <is>
-          <t>4 parça kuzu pirzola (zeytinyağı ve kekikle marine edilmiş), közlenmiş biber &amp; domates, pilav ve patates</t>
+          <t>4 parça kuzu pirzola (zeytinyağı, kekik ve pul biber ile marine edilmiş), közlenmiş biber &amp; domates, pilav ve patates eşliğinde</t>
         </is>
       </c>
       <c r="G59" s="4" t="inlineStr">
         <is>
-          <t>4 lamb chops (marinated in olive oil and thyme), roasted pepper &amp; tomato, rice and fries</t>
+          <t>4 lamb chops (marinated in olive oil, thyme and chilli flakes), served with roasted pepper &amp; tomato, rice and fries</t>
         </is>
       </c>
       <c r="H59" s="5" t="inlineStr"/>
@@ -4842,7 +4985,8 @@
       </c>
       <c r="Z59" s="8" t="inlineStr"/>
       <c r="AA59" s="8" t="inlineStr"/>
-      <c r="AB59" s="9" t="inlineStr"/>
+      <c r="AB59" s="8" t="inlineStr"/>
+      <c r="AC59" s="9" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -4870,12 +5014,12 @@
       </c>
       <c r="F60" s="4" t="inlineStr">
         <is>
-          <t>200 g antrikot (zeytinyağı ve kekikle marine edilmiş), közlenmiş biber &amp; domates, pilav ve patates</t>
+          <t>200 g antrikot (zeytinyağı, kekik ve pul biber ile marine edilmiş), közlenmiş biber &amp; domates, pilav ve patates eşliğinde</t>
         </is>
       </c>
       <c r="G60" s="4" t="inlineStr">
         <is>
-          <t>200 g ribeye (marinated in olive oil and thyme), roasted pepper &amp; tomato, rice and fries</t>
+          <t>200 g ribeye (marinated in olive oil, thyme and chilli flakes), served with roasted pepper &amp; tomato, rice and fries</t>
         </is>
       </c>
       <c r="H60" s="5" t="inlineStr"/>
@@ -4906,7 +5050,8 @@
       </c>
       <c r="Z60" s="8" t="inlineStr"/>
       <c r="AA60" s="8" t="inlineStr"/>
-      <c r="AB60" s="9" t="inlineStr"/>
+      <c r="AB60" s="8" t="inlineStr"/>
+      <c r="AC60" s="9" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -4934,12 +5079,12 @@
       </c>
       <c r="F61" s="4" t="inlineStr">
         <is>
-          <t>200 g bonfile (zeytinyağı ve kekikle marine edilmiş), közlenmiş biber &amp; domates, pilav ve patates</t>
+          <t>200 g bonfile (zeytinyağı, kekik ve pul biber ile marine edilmiş), közlenmiş biber &amp; domates, pilav ve patates eşliğinde</t>
         </is>
       </c>
       <c r="G61" s="4" t="inlineStr">
         <is>
-          <t>200 g tenderloin (marinated in olive oil and thyme), roasted pepper &amp; tomato, rice and fries</t>
+          <t>200 g tenderloin (marinated in olive oil, thyme and chilli flakes), served with roasted pepper &amp; tomato, rice and fries</t>
         </is>
       </c>
       <c r="H61" s="5" t="inlineStr"/>
@@ -4970,7 +5115,8 @@
       </c>
       <c r="Z61" s="8" t="inlineStr"/>
       <c r="AA61" s="8" t="inlineStr"/>
-      <c r="AB61" s="9" t="inlineStr"/>
+      <c r="AB61" s="8" t="inlineStr"/>
+      <c r="AC61" s="9" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -4998,15 +5144,19 @@
       </c>
       <c r="F62" s="4" t="inlineStr">
         <is>
-          <t>200 g bonfile (zeytinyağı ve kekikle marine edilmiş), mantar sos, közlenmiş biber &amp; domates, pilav ve patates</t>
+          <t>200 g bonfile (zeytinyağı, kekik ve pul biber ile marine edilmiş), mantar sos (krema, Cafe de Paris sos), közlenmiş biber &amp; domates, pilav ve patates eşliğinde</t>
         </is>
       </c>
       <c r="G62" s="4" t="inlineStr">
         <is>
-          <t>200 g tenderloin (marinated in olive oil and thyme), mushroom sauce, roasted pepper &amp; tomato, rice and fries</t>
-        </is>
-      </c>
-      <c r="H62" s="5" t="inlineStr"/>
+          <t>200 g tenderloin (marinated in olive oil, thyme and chilli flakes), mushroom sauce (cream, Café de Paris sauce), served with roasted pepper &amp; tomato, rice and fries</t>
+        </is>
+      </c>
+      <c r="H62" s="5" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="I62" s="5" t="inlineStr">
         <is>
           <t>X</t>
@@ -5038,7 +5188,12 @@
       </c>
       <c r="Z62" s="8" t="inlineStr"/>
       <c r="AA62" s="8" t="inlineStr"/>
-      <c r="AB62" s="9" t="inlineStr"/>
+      <c r="AB62" s="8" t="inlineStr">
+        <is>
+          <t>cafedeparis</t>
+        </is>
+      </c>
+      <c r="AC62" s="9" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -5066,15 +5221,19 @@
       </c>
       <c r="F63" s="4" t="inlineStr">
         <is>
-          <t>200 g bonfile, Cafe de Paris sos, közlenmiş biber &amp; domates, pilav ve patates</t>
+          <t>200 g bonfile, Cafe de Paris sos, közlenmiş biber &amp; domates, pilav ve patates eşliğinde</t>
         </is>
       </c>
       <c r="G63" s="4" t="inlineStr">
         <is>
-          <t>200 g tenderloin, Café de Paris sauce, roasted pepper &amp; tomato, rice and fries</t>
-        </is>
-      </c>
-      <c r="H63" s="5" t="inlineStr"/>
+          <t>200 g tenderloin, Café de Paris sauce, served with roasted pepper &amp; tomato, rice and fries</t>
+        </is>
+      </c>
+      <c r="H63" s="5" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="I63" s="5" t="inlineStr">
         <is>
           <t>X</t>
@@ -5110,7 +5269,12 @@
       </c>
       <c r="Z63" s="8" t="inlineStr"/>
       <c r="AA63" s="8" t="inlineStr"/>
-      <c r="AB63" s="9" t="inlineStr"/>
+      <c r="AB63" s="8" t="inlineStr">
+        <is>
+          <t>cafedeparis</t>
+        </is>
+      </c>
+      <c r="AC63" s="9" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -5138,12 +5302,12 @@
       </c>
       <c r="F64" s="4" t="inlineStr">
         <is>
-          <t>200 g kekik ve zeytinyağı ile marine edilmiş et, renkli biberler, soğan, Sweet Chili sos, süzme yoğurt, özel Kule sos (Sweet Chili sos, mayonez, acı sos, salsa sos), lavaş</t>
+          <t>200 g kekik, zeytinyağı ve pul biber ile marine edilmiş et, renkli biberler, soğan, Sweet Chili sos, süzme yoğurt, özel Kule sos (Sweet Chili sos, mayonez, acı sos, pul biber, tuz), lavaş</t>
         </is>
       </c>
       <c r="G64" s="4" t="inlineStr">
         <is>
-          <t>200 g beef marinated in thyme and olive oil, bell peppers, onion, sweet chilli sauce, strained yoghurt, special Kule sauce (sweet chilli sauce, mayonnaise, hot sauce, salsa), lavash</t>
+          <t>200 g beef marinated in thyme, olive oil and chilli flakes, bell peppers, onion, sweet chilli sauce, strained yoghurt, special Kule sauce (sweet chilli sauce, mayonnaise, hot sauce, chilli flakes, salt), lavash</t>
         </is>
       </c>
       <c r="H64" s="5" t="inlineStr">
@@ -5186,7 +5350,12 @@
       </c>
       <c r="Z64" s="8" t="inlineStr"/>
       <c r="AA64" s="8" t="inlineStr"/>
-      <c r="AB64" s="9" t="inlineStr"/>
+      <c r="AB64" s="8" t="inlineStr">
+        <is>
+          <t>sweetchili</t>
+        </is>
+      </c>
+      <c r="AC64" s="9" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -5214,12 +5383,12 @@
       </c>
       <c r="F65" s="4" t="inlineStr">
         <is>
-          <t>150 g et ve 150 g tavuk (kekik ve zeytinyağı ile marine edilmiş), renkli biberler, soğan, Sweet Chili sos, süzme yoğurt, özel Kule sos (Sweet Chili sos, mayonez, acı sos, salsa sos), lavaş</t>
+          <t>150 g et ve 150 g tavuk (kekik, zeytinyağı ve pul biber ile marine edilmiş), renkli biberler, soğan, Sweet Chili sos, süzme yoğurt, özel Kule sos (Sweet Chili sos, mayonez, acı sos, pul biber, tuz), lavaş</t>
         </is>
       </c>
       <c r="G65" s="4" t="inlineStr">
         <is>
-          <t>150 g beef and 150 g chicken (marinated in thyme and olive oil), bell peppers, onion, sweet chilli sauce, strained yoghurt, special Kule sauce (sweet chilli sauce, mayonnaise, hot sauce, salsa), lavash</t>
+          <t>150 g beef and 150 g chicken (marinated in thyme, olive oil and chilli flakes), bell peppers, onion, sweet chilli sauce, strained yoghurt, special Kule sauce (sweet chilli sauce, mayonnaise, hot sauce, chilli flakes, salt), lavash</t>
         </is>
       </c>
       <c r="H65" s="5" t="inlineStr">
@@ -5262,7 +5431,12 @@
       </c>
       <c r="Z65" s="8" t="inlineStr"/>
       <c r="AA65" s="8" t="inlineStr"/>
-      <c r="AB65" s="9" t="inlineStr"/>
+      <c r="AB65" s="8" t="inlineStr">
+        <is>
+          <t>sweetchili</t>
+        </is>
+      </c>
+      <c r="AC65" s="9" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -5338,7 +5512,8 @@
       </c>
       <c r="Z66" s="8" t="inlineStr"/>
       <c r="AA66" s="8" t="inlineStr"/>
-      <c r="AB66" s="9" t="inlineStr"/>
+      <c r="AB66" s="8" t="inlineStr"/>
+      <c r="AC66" s="9" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -5414,7 +5589,8 @@
       </c>
       <c r="Z67" s="8" t="inlineStr"/>
       <c r="AA67" s="8" t="inlineStr"/>
-      <c r="AB67" s="9" t="inlineStr"/>
+      <c r="AB67" s="8" t="inlineStr"/>
+      <c r="AC67" s="9" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -5494,7 +5670,8 @@
       </c>
       <c r="Z68" s="8" t="inlineStr"/>
       <c r="AA68" s="8" t="inlineStr"/>
-      <c r="AB68" s="9" t="inlineStr"/>
+      <c r="AB68" s="8" t="inlineStr"/>
+      <c r="AC68" s="9" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -5574,7 +5751,8 @@
       </c>
       <c r="Z69" s="8" t="inlineStr"/>
       <c r="AA69" s="8" t="inlineStr"/>
-      <c r="AB69" s="9" t="inlineStr"/>
+      <c r="AB69" s="8" t="inlineStr"/>
+      <c r="AC69" s="9" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -5654,7 +5832,8 @@
       </c>
       <c r="Z70" s="8" t="inlineStr"/>
       <c r="AA70" s="8" t="inlineStr"/>
-      <c r="AB70" s="9" t="inlineStr"/>
+      <c r="AB70" s="8" t="inlineStr"/>
+      <c r="AC70" s="9" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -5730,7 +5909,8 @@
       </c>
       <c r="Z71" s="8" t="inlineStr"/>
       <c r="AA71" s="8" t="inlineStr"/>
-      <c r="AB71" s="9" t="inlineStr"/>
+      <c r="AB71" s="8" t="inlineStr"/>
+      <c r="AC71" s="9" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -5814,7 +5994,8 @@
       </c>
       <c r="Z72" s="8" t="inlineStr"/>
       <c r="AA72" s="8" t="inlineStr"/>
-      <c r="AB72" s="9" t="inlineStr"/>
+      <c r="AB72" s="8" t="inlineStr"/>
+      <c r="AC72" s="9" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -5890,7 +6071,8 @@
       </c>
       <c r="Z73" s="8" t="inlineStr"/>
       <c r="AA73" s="8" t="inlineStr"/>
-      <c r="AB73" s="9" t="inlineStr"/>
+      <c r="AB73" s="8" t="inlineStr"/>
+      <c r="AC73" s="9" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -5966,7 +6148,8 @@
       </c>
       <c r="Z74" s="8" t="inlineStr"/>
       <c r="AA74" s="8" t="inlineStr"/>
-      <c r="AB74" s="9" t="inlineStr"/>
+      <c r="AB74" s="8" t="inlineStr"/>
+      <c r="AC74" s="9" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -6042,7 +6225,8 @@
       </c>
       <c r="Z75" s="8" t="inlineStr"/>
       <c r="AA75" s="8" t="inlineStr"/>
-      <c r="AB75" s="9" t="inlineStr"/>
+      <c r="AB75" s="8" t="inlineStr"/>
+      <c r="AC75" s="9" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -6122,7 +6306,8 @@
       </c>
       <c r="Z76" s="8" t="inlineStr"/>
       <c r="AA76" s="8" t="inlineStr"/>
-      <c r="AB76" s="9" t="inlineStr"/>
+      <c r="AB76" s="8" t="inlineStr"/>
+      <c r="AC76" s="9" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -6202,7 +6387,8 @@
       </c>
       <c r="Z77" s="8" t="inlineStr"/>
       <c r="AA77" s="8" t="inlineStr"/>
-      <c r="AB77" s="9" t="inlineStr"/>
+      <c r="AB77" s="8" t="inlineStr"/>
+      <c r="AC77" s="9" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -6278,7 +6464,8 @@
       </c>
       <c r="Z78" s="8" t="inlineStr"/>
       <c r="AA78" s="8" t="inlineStr"/>
-      <c r="AB78" s="9" t="inlineStr"/>
+      <c r="AB78" s="8" t="inlineStr"/>
+      <c r="AC78" s="9" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -6354,7 +6541,8 @@
       </c>
       <c r="Z79" s="8" t="inlineStr"/>
       <c r="AA79" s="8" t="inlineStr"/>
-      <c r="AB79" s="9" t="inlineStr"/>
+      <c r="AB79" s="8" t="inlineStr"/>
+      <c r="AC79" s="9" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -6430,7 +6618,8 @@
       </c>
       <c r="Z80" s="8" t="inlineStr"/>
       <c r="AA80" s="8" t="inlineStr"/>
-      <c r="AB80" s="9" t="inlineStr"/>
+      <c r="AB80" s="8" t="inlineStr"/>
+      <c r="AC80" s="9" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -6494,7 +6683,8 @@
       </c>
       <c r="Z81" s="8" t="inlineStr"/>
       <c r="AA81" s="8" t="inlineStr"/>
-      <c r="AB81" s="9" t="inlineStr"/>
+      <c r="AB81" s="8" t="inlineStr"/>
+      <c r="AC81" s="9" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -6562,7 +6752,8 @@
       </c>
       <c r="Z82" s="8" t="inlineStr"/>
       <c r="AA82" s="8" t="inlineStr"/>
-      <c r="AB82" s="9" t="inlineStr"/>
+      <c r="AB82" s="8" t="inlineStr"/>
+      <c r="AC82" s="9" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -6630,7 +6821,8 @@
       </c>
       <c r="Z83" s="8" t="inlineStr"/>
       <c r="AA83" s="8" t="inlineStr"/>
-      <c r="AB83" s="9" t="inlineStr"/>
+      <c r="AB83" s="8" t="inlineStr"/>
+      <c r="AC83" s="9" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -6694,7 +6886,8 @@
       </c>
       <c r="Z84" s="8" t="inlineStr"/>
       <c r="AA84" s="8" t="inlineStr"/>
-      <c r="AB84" s="9" t="inlineStr"/>
+      <c r="AB84" s="8" t="inlineStr"/>
+      <c r="AC84" s="9" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -6758,7 +6951,8 @@
       </c>
       <c r="Z85" s="8" t="inlineStr"/>
       <c r="AA85" s="8" t="inlineStr"/>
-      <c r="AB85" s="9" t="inlineStr"/>
+      <c r="AB85" s="8" t="inlineStr"/>
+      <c r="AC85" s="9" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -6826,7 +7020,8 @@
       </c>
       <c r="Z86" s="8" t="inlineStr"/>
       <c r="AA86" s="8" t="inlineStr"/>
-      <c r="AB86" s="9" t="inlineStr"/>
+      <c r="AB86" s="8" t="inlineStr"/>
+      <c r="AC86" s="9" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -6890,7 +7085,8 @@
       </c>
       <c r="Z87" s="8" t="inlineStr"/>
       <c r="AA87" s="8" t="inlineStr"/>
-      <c r="AB87" s="9" t="inlineStr"/>
+      <c r="AB87" s="8" t="inlineStr"/>
+      <c r="AC87" s="9" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -6954,7 +7150,8 @@
       </c>
       <c r="Z88" s="8" t="inlineStr"/>
       <c r="AA88" s="8" t="inlineStr"/>
-      <c r="AB88" s="9" t="inlineStr"/>
+      <c r="AB88" s="8" t="inlineStr"/>
+      <c r="AC88" s="9" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -7022,7 +7219,8 @@
       </c>
       <c r="Z89" s="8" t="inlineStr"/>
       <c r="AA89" s="8" t="inlineStr"/>
-      <c r="AB89" s="9" t="inlineStr"/>
+      <c r="AB89" s="8" t="inlineStr"/>
+      <c r="AC89" s="9" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -7090,7 +7288,8 @@
       </c>
       <c r="Z90" s="8" t="inlineStr"/>
       <c r="AA90" s="8" t="inlineStr"/>
-      <c r="AB90" s="9" t="inlineStr"/>
+      <c r="AB90" s="8" t="inlineStr"/>
+      <c r="AC90" s="9" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -7162,7 +7361,8 @@
       </c>
       <c r="Z91" s="8" t="inlineStr"/>
       <c r="AA91" s="8" t="inlineStr"/>
-      <c r="AB91" s="9" t="inlineStr"/>
+      <c r="AB91" s="8" t="inlineStr"/>
+      <c r="AC91" s="9" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -7234,7 +7434,8 @@
       </c>
       <c r="Z92" s="8" t="inlineStr"/>
       <c r="AA92" s="8" t="inlineStr"/>
-      <c r="AB92" s="9" t="inlineStr"/>
+      <c r="AB92" s="8" t="inlineStr"/>
+      <c r="AC92" s="9" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -7302,7 +7503,8 @@
       </c>
       <c r="Z93" s="8" t="inlineStr"/>
       <c r="AA93" s="8" t="inlineStr"/>
-      <c r="AB93" s="9" t="inlineStr"/>
+      <c r="AB93" s="8" t="inlineStr"/>
+      <c r="AC93" s="9" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -7370,7 +7572,8 @@
       </c>
       <c r="Z94" s="8" t="inlineStr"/>
       <c r="AA94" s="8" t="inlineStr"/>
-      <c r="AB94" s="9" t="inlineStr"/>
+      <c r="AB94" s="8" t="inlineStr"/>
+      <c r="AC94" s="9" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -7438,7 +7641,8 @@
       </c>
       <c r="Z95" s="8" t="inlineStr"/>
       <c r="AA95" s="8" t="inlineStr"/>
-      <c r="AB95" s="9" t="inlineStr"/>
+      <c r="AB95" s="8" t="inlineStr"/>
+      <c r="AC95" s="9" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -7506,7 +7710,8 @@
       </c>
       <c r="Z96" s="8" t="inlineStr"/>
       <c r="AA96" s="8" t="inlineStr"/>
-      <c r="AB96" s="9" t="inlineStr"/>
+      <c r="AB96" s="8" t="inlineStr"/>
+      <c r="AC96" s="9" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -7574,7 +7779,8 @@
       </c>
       <c r="Z97" s="8" t="inlineStr"/>
       <c r="AA97" s="8" t="inlineStr"/>
-      <c r="AB97" s="9" t="inlineStr"/>
+      <c r="AB97" s="8" t="inlineStr"/>
+      <c r="AC97" s="9" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -7642,7 +7848,8 @@
       </c>
       <c r="Z98" s="8" t="inlineStr"/>
       <c r="AA98" s="8" t="inlineStr"/>
-      <c r="AB98" s="9" t="inlineStr"/>
+      <c r="AB98" s="8" t="inlineStr"/>
+      <c r="AC98" s="9" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -7714,7 +7921,8 @@
       </c>
       <c r="Z99" s="8" t="inlineStr"/>
       <c r="AA99" s="8" t="inlineStr"/>
-      <c r="AB99" s="9" t="inlineStr"/>
+      <c r="AB99" s="8" t="inlineStr"/>
+      <c r="AC99" s="9" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -7782,7 +7990,8 @@
       </c>
       <c r="Z100" s="8" t="inlineStr"/>
       <c r="AA100" s="8" t="inlineStr"/>
-      <c r="AB100" s="9" t="inlineStr"/>
+      <c r="AB100" s="8" t="inlineStr"/>
+      <c r="AC100" s="9" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -7850,7 +8059,8 @@
       </c>
       <c r="Z101" s="8" t="inlineStr"/>
       <c r="AA101" s="8" t="inlineStr"/>
-      <c r="AB101" s="9" t="inlineStr"/>
+      <c r="AB101" s="8" t="inlineStr"/>
+      <c r="AC101" s="9" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -7922,7 +8132,8 @@
       </c>
       <c r="Z102" s="8" t="inlineStr"/>
       <c r="AA102" s="8" t="inlineStr"/>
-      <c r="AB102" s="9" t="inlineStr"/>
+      <c r="AB102" s="8" t="inlineStr"/>
+      <c r="AC102" s="9" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -7994,7 +8205,8 @@
       </c>
       <c r="Z103" s="8" t="inlineStr"/>
       <c r="AA103" s="8" t="inlineStr"/>
-      <c r="AB103" s="9" t="inlineStr"/>
+      <c r="AB103" s="8" t="inlineStr"/>
+      <c r="AC103" s="9" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -8066,7 +8278,8 @@
       </c>
       <c r="Z104" s="8" t="inlineStr"/>
       <c r="AA104" s="8" t="inlineStr"/>
-      <c r="AB104" s="9" t="inlineStr"/>
+      <c r="AB104" s="8" t="inlineStr"/>
+      <c r="AC104" s="9" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -8134,7 +8347,8 @@
       </c>
       <c r="Z105" s="8" t="inlineStr"/>
       <c r="AA105" s="8" t="inlineStr"/>
-      <c r="AB105" s="9" t="inlineStr"/>
+      <c r="AB105" s="8" t="inlineStr"/>
+      <c r="AC105" s="9" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -8198,7 +8412,8 @@
       </c>
       <c r="Z106" s="8" t="inlineStr"/>
       <c r="AA106" s="8" t="inlineStr"/>
-      <c r="AB106" s="9" t="inlineStr"/>
+      <c r="AB106" s="8" t="inlineStr"/>
+      <c r="AC106" s="9" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -8266,7 +8481,8 @@
       </c>
       <c r="Z107" s="8" t="inlineStr"/>
       <c r="AA107" s="8" t="inlineStr"/>
-      <c r="AB107" s="9" t="inlineStr"/>
+      <c r="AB107" s="8" t="inlineStr"/>
+      <c r="AC107" s="9" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -8334,7 +8550,8 @@
       </c>
       <c r="Z108" s="8" t="inlineStr"/>
       <c r="AA108" s="8" t="inlineStr"/>
-      <c r="AB108" s="9" t="inlineStr"/>
+      <c r="AB108" s="8" t="inlineStr"/>
+      <c r="AC108" s="9" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -8406,7 +8623,8 @@
       </c>
       <c r="Z109" s="8" t="inlineStr"/>
       <c r="AA109" s="8" t="inlineStr"/>
-      <c r="AB109" s="9" t="inlineStr"/>
+      <c r="AB109" s="8" t="inlineStr"/>
+      <c r="AC109" s="9" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -8478,7 +8696,8 @@
       </c>
       <c r="Z110" s="8" t="inlineStr"/>
       <c r="AA110" s="8" t="inlineStr"/>
-      <c r="AB110" s="9" t="inlineStr"/>
+      <c r="AB110" s="8" t="inlineStr"/>
+      <c r="AC110" s="9" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -8546,7 +8765,8 @@
       </c>
       <c r="Z111" s="8" t="inlineStr"/>
       <c r="AA111" s="8" t="inlineStr"/>
-      <c r="AB111" s="9" t="inlineStr"/>
+      <c r="AB111" s="8" t="inlineStr"/>
+      <c r="AC111" s="9" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -8614,7 +8834,8 @@
       </c>
       <c r="Z112" s="8" t="inlineStr"/>
       <c r="AA112" s="8" t="inlineStr"/>
-      <c r="AB112" s="9" t="inlineStr"/>
+      <c r="AB112" s="8" t="inlineStr"/>
+      <c r="AC112" s="9" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -8682,7 +8903,8 @@
       </c>
       <c r="Z113" s="8" t="inlineStr"/>
       <c r="AA113" s="8" t="inlineStr"/>
-      <c r="AB113" s="9" t="inlineStr"/>
+      <c r="AB113" s="8" t="inlineStr"/>
+      <c r="AC113" s="9" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -8750,7 +8972,8 @@
       </c>
       <c r="Z114" s="8" t="inlineStr"/>
       <c r="AA114" s="8" t="inlineStr"/>
-      <c r="AB114" s="9" t="inlineStr"/>
+      <c r="AB114" s="8" t="inlineStr"/>
+      <c r="AC114" s="9" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -8814,7 +9037,8 @@
       </c>
       <c r="Z115" s="8" t="inlineStr"/>
       <c r="AA115" s="8" t="inlineStr"/>
-      <c r="AB115" s="9" t="inlineStr"/>
+      <c r="AB115" s="8" t="inlineStr"/>
+      <c r="AC115" s="9" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -8878,7 +9102,8 @@
       </c>
       <c r="Z116" s="8" t="inlineStr"/>
       <c r="AA116" s="8" t="inlineStr"/>
-      <c r="AB116" s="9" t="inlineStr"/>
+      <c r="AB116" s="8" t="inlineStr"/>
+      <c r="AC116" s="9" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -8942,7 +9167,8 @@
       </c>
       <c r="Z117" s="8" t="inlineStr"/>
       <c r="AA117" s="8" t="inlineStr"/>
-      <c r="AB117" s="9" t="inlineStr"/>
+      <c r="AB117" s="8" t="inlineStr"/>
+      <c r="AC117" s="9" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -9006,7 +9232,8 @@
       </c>
       <c r="Z118" s="8" t="inlineStr"/>
       <c r="AA118" s="8" t="inlineStr"/>
-      <c r="AB118" s="9" t="inlineStr"/>
+      <c r="AB118" s="8" t="inlineStr"/>
+      <c r="AC118" s="9" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -9070,7 +9297,8 @@
       </c>
       <c r="Z119" s="8" t="inlineStr"/>
       <c r="AA119" s="8" t="inlineStr"/>
-      <c r="AB119" s="9" t="inlineStr"/>
+      <c r="AB119" s="8" t="inlineStr"/>
+      <c r="AC119" s="9" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -9134,7 +9362,8 @@
       </c>
       <c r="Z120" s="8" t="inlineStr"/>
       <c r="AA120" s="8" t="inlineStr"/>
-      <c r="AB120" s="9" t="inlineStr"/>
+      <c r="AB120" s="8" t="inlineStr"/>
+      <c r="AC120" s="9" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -9198,7 +9427,8 @@
       </c>
       <c r="Z121" s="8" t="inlineStr"/>
       <c r="AA121" s="8" t="inlineStr"/>
-      <c r="AB121" s="9" t="inlineStr"/>
+      <c r="AB121" s="8" t="inlineStr"/>
+      <c r="AC121" s="9" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -9262,7 +9492,8 @@
       </c>
       <c r="Z122" s="8" t="inlineStr"/>
       <c r="AA122" s="8" t="inlineStr"/>
-      <c r="AB122" s="9" t="inlineStr"/>
+      <c r="AB122" s="8" t="inlineStr"/>
+      <c r="AC122" s="9" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -9326,7 +9557,8 @@
       </c>
       <c r="Z123" s="8" t="inlineStr"/>
       <c r="AA123" s="8" t="inlineStr"/>
-      <c r="AB123" s="9" t="inlineStr"/>
+      <c r="AB123" s="8" t="inlineStr"/>
+      <c r="AC123" s="9" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -9390,7 +9622,8 @@
       </c>
       <c r="Z124" s="8" t="inlineStr"/>
       <c r="AA124" s="8" t="inlineStr"/>
-      <c r="AB124" s="9" t="inlineStr"/>
+      <c r="AB124" s="8" t="inlineStr"/>
+      <c r="AC124" s="9" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -9454,7 +9687,8 @@
       </c>
       <c r="Z125" s="8" t="inlineStr"/>
       <c r="AA125" s="8" t="inlineStr"/>
-      <c r="AB125" s="9" t="inlineStr"/>
+      <c r="AB125" s="8" t="inlineStr"/>
+      <c r="AC125" s="9" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -9518,7 +9752,8 @@
       </c>
       <c r="Z126" s="8" t="inlineStr"/>
       <c r="AA126" s="8" t="inlineStr"/>
-      <c r="AB126" s="9" t="inlineStr"/>
+      <c r="AB126" s="8" t="inlineStr"/>
+      <c r="AC126" s="9" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -9582,7 +9817,8 @@
       </c>
       <c r="Z127" s="8" t="inlineStr"/>
       <c r="AA127" s="8" t="inlineStr"/>
-      <c r="AB127" s="9" t="inlineStr"/>
+      <c r="AB127" s="8" t="inlineStr"/>
+      <c r="AC127" s="9" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -9646,7 +9882,8 @@
       </c>
       <c r="Z128" s="8" t="inlineStr"/>
       <c r="AA128" s="8" t="inlineStr"/>
-      <c r="AB128" s="9" t="inlineStr"/>
+      <c r="AB128" s="8" t="inlineStr"/>
+      <c r="AC128" s="9" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -9710,7 +9947,8 @@
       </c>
       <c r="Z129" s="8" t="inlineStr"/>
       <c r="AA129" s="8" t="inlineStr"/>
-      <c r="AB129" s="9" t="inlineStr"/>
+      <c r="AB129" s="8" t="inlineStr"/>
+      <c r="AC129" s="9" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -9774,7 +10012,8 @@
       </c>
       <c r="Z130" s="8" t="inlineStr"/>
       <c r="AA130" s="8" t="inlineStr"/>
-      <c r="AB130" s="9" t="inlineStr"/>
+      <c r="AB130" s="8" t="inlineStr"/>
+      <c r="AC130" s="9" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -9838,7 +10077,8 @@
       </c>
       <c r="Z131" s="8" t="inlineStr"/>
       <c r="AA131" s="8" t="inlineStr"/>
-      <c r="AB131" s="9" t="inlineStr"/>
+      <c r="AB131" s="8" t="inlineStr"/>
+      <c r="AC131" s="9" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -9902,7 +10142,8 @@
       </c>
       <c r="Z132" s="8" t="inlineStr"/>
       <c r="AA132" s="8" t="inlineStr"/>
-      <c r="AB132" s="9" t="inlineStr"/>
+      <c r="AB132" s="8" t="inlineStr"/>
+      <c r="AC132" s="9" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -9970,7 +10211,8 @@
       </c>
       <c r="Z133" s="8" t="inlineStr"/>
       <c r="AA133" s="8" t="inlineStr"/>
-      <c r="AB133" s="9" t="inlineStr"/>
+      <c r="AB133" s="8" t="inlineStr"/>
+      <c r="AC133" s="9" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -10034,7 +10276,8 @@
       </c>
       <c r="Z134" s="8" t="inlineStr"/>
       <c r="AA134" s="8" t="inlineStr"/>
-      <c r="AB134" s="9" t="inlineStr"/>
+      <c r="AB134" s="8" t="inlineStr"/>
+      <c r="AC134" s="9" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -10098,7 +10341,8 @@
       </c>
       <c r="Z135" s="8" t="inlineStr"/>
       <c r="AA135" s="8" t="inlineStr"/>
-      <c r="AB135" s="9" t="inlineStr"/>
+      <c r="AB135" s="8" t="inlineStr"/>
+      <c r="AC135" s="9" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -10162,7 +10406,8 @@
       </c>
       <c r="Z136" s="8" t="inlineStr"/>
       <c r="AA136" s="8" t="inlineStr"/>
-      <c r="AB136" s="9" t="inlineStr"/>
+      <c r="AB136" s="8" t="inlineStr"/>
+      <c r="AC136" s="9" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -10226,7 +10471,8 @@
       </c>
       <c r="Z137" s="8" t="inlineStr"/>
       <c r="AA137" s="8" t="inlineStr"/>
-      <c r="AB137" s="9" t="inlineStr"/>
+      <c r="AB137" s="8" t="inlineStr"/>
+      <c r="AC137" s="9" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -10290,7 +10536,8 @@
       </c>
       <c r="Z138" s="8" t="inlineStr"/>
       <c r="AA138" s="8" t="inlineStr"/>
-      <c r="AB138" s="9" t="inlineStr"/>
+      <c r="AB138" s="8" t="inlineStr"/>
+      <c r="AC138" s="9" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -10354,7 +10601,8 @@
       </c>
       <c r="Z139" s="8" t="inlineStr"/>
       <c r="AA139" s="8" t="inlineStr"/>
-      <c r="AB139" s="9" t="inlineStr"/>
+      <c r="AB139" s="8" t="inlineStr"/>
+      <c r="AC139" s="9" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -10418,7 +10666,8 @@
       </c>
       <c r="Z140" s="8" t="inlineStr"/>
       <c r="AA140" s="8" t="inlineStr"/>
-      <c r="AB140" s="9" t="inlineStr"/>
+      <c r="AB140" s="8" t="inlineStr"/>
+      <c r="AC140" s="9" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -10486,7 +10735,8 @@
       </c>
       <c r="Z141" s="8" t="inlineStr"/>
       <c r="AA141" s="8" t="inlineStr"/>
-      <c r="AB141" s="9" t="inlineStr"/>
+      <c r="AB141" s="8" t="inlineStr"/>
+      <c r="AC141" s="9" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -10558,7 +10808,8 @@
       </c>
       <c r="Z142" s="8" t="inlineStr"/>
       <c r="AA142" s="8" t="inlineStr"/>
-      <c r="AB142" s="9" t="inlineStr"/>
+      <c r="AB142" s="8" t="inlineStr"/>
+      <c r="AC142" s="9" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -10626,7 +10877,8 @@
       </c>
       <c r="Z143" s="8" t="inlineStr"/>
       <c r="AA143" s="8" t="inlineStr"/>
-      <c r="AB143" s="9" t="inlineStr"/>
+      <c r="AB143" s="8" t="inlineStr"/>
+      <c r="AC143" s="9" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -10702,7 +10954,8 @@
       </c>
       <c r="Z144" s="8" t="inlineStr"/>
       <c r="AA144" s="8" t="inlineStr"/>
-      <c r="AB144" s="9" t="inlineStr"/>
+      <c r="AB144" s="8" t="inlineStr"/>
+      <c r="AC144" s="9" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -10770,7 +11023,8 @@
       </c>
       <c r="Z145" s="8" t="inlineStr"/>
       <c r="AA145" s="8" t="inlineStr"/>
-      <c r="AB145" s="9" t="inlineStr"/>
+      <c r="AB145" s="8" t="inlineStr"/>
+      <c r="AC145" s="9" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -10834,7 +11088,8 @@
       </c>
       <c r="Z146" s="8" t="inlineStr"/>
       <c r="AA146" s="8" t="inlineStr"/>
-      <c r="AB146" s="9" t="inlineStr"/>
+      <c r="AB146" s="8" t="inlineStr"/>
+      <c r="AC146" s="9" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -10898,7 +11153,8 @@
       </c>
       <c r="Z147" s="8" t="inlineStr"/>
       <c r="AA147" s="8" t="inlineStr"/>
-      <c r="AB147" s="9" t="inlineStr"/>
+      <c r="AB147" s="8" t="inlineStr"/>
+      <c r="AC147" s="9" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -10962,7 +11218,8 @@
       </c>
       <c r="Z148" s="8" t="inlineStr"/>
       <c r="AA148" s="8" t="inlineStr"/>
-      <c r="AB148" s="9" t="inlineStr"/>
+      <c r="AB148" s="8" t="inlineStr"/>
+      <c r="AC148" s="9" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -11026,7 +11283,8 @@
       </c>
       <c r="Z149" s="8" t="inlineStr"/>
       <c r="AA149" s="8" t="inlineStr"/>
-      <c r="AB149" s="9" t="inlineStr"/>
+      <c r="AB149" s="8" t="inlineStr"/>
+      <c r="AC149" s="9" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -11090,7 +11348,8 @@
       </c>
       <c r="Z150" s="8" t="inlineStr"/>
       <c r="AA150" s="8" t="inlineStr"/>
-      <c r="AB150" s="9" t="inlineStr"/>
+      <c r="AB150" s="8" t="inlineStr"/>
+      <c r="AC150" s="9" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -11154,7 +11413,8 @@
       </c>
       <c r="Z151" s="8" t="inlineStr"/>
       <c r="AA151" s="8" t="inlineStr"/>
-      <c r="AB151" s="9" t="inlineStr"/>
+      <c r="AB151" s="8" t="inlineStr"/>
+      <c r="AC151" s="9" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -11218,7 +11478,8 @@
       </c>
       <c r="Z152" s="8" t="inlineStr"/>
       <c r="AA152" s="8" t="inlineStr"/>
-      <c r="AB152" s="9" t="inlineStr"/>
+      <c r="AB152" s="8" t="inlineStr"/>
+      <c r="AC152" s="9" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -11282,7 +11543,8 @@
       </c>
       <c r="Z153" s="8" t="inlineStr"/>
       <c r="AA153" s="8" t="inlineStr"/>
-      <c r="AB153" s="9" t="inlineStr"/>
+      <c r="AB153" s="8" t="inlineStr"/>
+      <c r="AC153" s="9" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -11346,7 +11608,8 @@
       </c>
       <c r="Z154" s="8" t="inlineStr"/>
       <c r="AA154" s="8" t="inlineStr"/>
-      <c r="AB154" s="9" t="inlineStr"/>
+      <c r="AB154" s="8" t="inlineStr"/>
+      <c r="AC154" s="9" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -11410,7 +11673,8 @@
       </c>
       <c r="Z155" s="8" t="inlineStr"/>
       <c r="AA155" s="8" t="inlineStr"/>
-      <c r="AB155" s="9" t="inlineStr"/>
+      <c r="AB155" s="8" t="inlineStr"/>
+      <c r="AC155" s="9" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -11474,7 +11738,8 @@
       </c>
       <c r="Z156" s="8" t="inlineStr"/>
       <c r="AA156" s="8" t="inlineStr"/>
-      <c r="AB156" s="9" t="inlineStr"/>
+      <c r="AB156" s="8" t="inlineStr"/>
+      <c r="AC156" s="9" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -11538,7 +11803,8 @@
       </c>
       <c r="Z157" s="8" t="inlineStr"/>
       <c r="AA157" s="8" t="inlineStr"/>
-      <c r="AB157" s="9" t="inlineStr"/>
+      <c r="AB157" s="8" t="inlineStr"/>
+      <c r="AC157" s="9" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -11602,7 +11868,8 @@
       </c>
       <c r="Z158" s="8" t="inlineStr"/>
       <c r="AA158" s="8" t="inlineStr"/>
-      <c r="AB158" s="9" t="inlineStr"/>
+      <c r="AB158" s="8" t="inlineStr"/>
+      <c r="AC158" s="9" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -11666,7 +11933,8 @@
       </c>
       <c r="Z159" s="8" t="inlineStr"/>
       <c r="AA159" s="8" t="inlineStr"/>
-      <c r="AB159" s="9" t="inlineStr"/>
+      <c r="AB159" s="8" t="inlineStr"/>
+      <c r="AC159" s="9" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -11722,7 +11990,8 @@
       <c r="Y160" s="7" t="inlineStr"/>
       <c r="Z160" s="8" t="inlineStr"/>
       <c r="AA160" s="8" t="inlineStr"/>
-      <c r="AB160" s="9" t="inlineStr"/>
+      <c r="AB160" s="8" t="inlineStr"/>
+      <c r="AC160" s="9" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -11778,7 +12047,8 @@
       <c r="Y161" s="7" t="inlineStr"/>
       <c r="Z161" s="8" t="inlineStr"/>
       <c r="AA161" s="8" t="inlineStr"/>
-      <c r="AB161" s="9" t="inlineStr"/>
+      <c r="AB161" s="8" t="inlineStr"/>
+      <c r="AC161" s="9" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -11834,7 +12104,8 @@
       <c r="Y162" s="7" t="inlineStr"/>
       <c r="Z162" s="8" t="inlineStr"/>
       <c r="AA162" s="8" t="inlineStr"/>
-      <c r="AB162" s="9" t="inlineStr"/>
+      <c r="AB162" s="8" t="inlineStr"/>
+      <c r="AC162" s="9" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -11890,7 +12161,8 @@
       <c r="Y163" s="7" t="inlineStr"/>
       <c r="Z163" s="8" t="inlineStr"/>
       <c r="AA163" s="8" t="inlineStr"/>
-      <c r="AB163" s="9" t="inlineStr"/>
+      <c r="AB163" s="8" t="inlineStr"/>
+      <c r="AC163" s="9" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -11946,7 +12218,8 @@
       <c r="Y164" s="7" t="inlineStr"/>
       <c r="Z164" s="8" t="inlineStr"/>
       <c r="AA164" s="8" t="inlineStr"/>
-      <c r="AB164" s="9" t="inlineStr"/>
+      <c r="AB164" s="8" t="inlineStr"/>
+      <c r="AC164" s="9" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -12002,7 +12275,8 @@
       <c r="Y165" s="7" t="inlineStr"/>
       <c r="Z165" s="8" t="inlineStr"/>
       <c r="AA165" s="8" t="inlineStr"/>
-      <c r="AB165" s="9" t="inlineStr"/>
+      <c r="AB165" s="8" t="inlineStr"/>
+      <c r="AC165" s="9" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
@@ -12058,7 +12332,8 @@
       <c r="Y166" s="7" t="inlineStr"/>
       <c r="Z166" s="8" t="inlineStr"/>
       <c r="AA166" s="8" t="inlineStr"/>
-      <c r="AB166" s="9" t="inlineStr"/>
+      <c r="AB166" s="8" t="inlineStr"/>
+      <c r="AC166" s="9" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" s="2" t="inlineStr">
@@ -12114,7 +12389,8 @@
       <c r="Y167" s="7" t="inlineStr"/>
       <c r="Z167" s="8" t="inlineStr"/>
       <c r="AA167" s="8" t="inlineStr"/>
-      <c r="AB167" s="9" t="inlineStr"/>
+      <c r="AB167" s="8" t="inlineStr"/>
+      <c r="AC167" s="9" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
@@ -12170,7 +12446,8 @@
       <c r="Y168" s="7" t="inlineStr"/>
       <c r="Z168" s="8" t="inlineStr"/>
       <c r="AA168" s="8" t="inlineStr"/>
-      <c r="AB168" s="9" t="inlineStr"/>
+      <c r="AB168" s="8" t="inlineStr"/>
+      <c r="AC168" s="9" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
@@ -12226,7 +12503,8 @@
       <c r="Y169" s="7" t="inlineStr"/>
       <c r="Z169" s="8" t="inlineStr"/>
       <c r="AA169" s="8" t="inlineStr"/>
-      <c r="AB169" s="9" t="inlineStr"/>
+      <c r="AB169" s="8" t="inlineStr"/>
+      <c r="AC169" s="9" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" s="2" t="inlineStr">
@@ -12282,7 +12560,8 @@
       <c r="Y170" s="7" t="inlineStr"/>
       <c r="Z170" s="8" t="inlineStr"/>
       <c r="AA170" s="8" t="inlineStr"/>
-      <c r="AB170" s="9" t="inlineStr"/>
+      <c r="AB170" s="8" t="inlineStr"/>
+      <c r="AC170" s="9" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
@@ -12338,7 +12617,8 @@
       <c r="Y171" s="7" t="inlineStr"/>
       <c r="Z171" s="8" t="inlineStr"/>
       <c r="AA171" s="8" t="inlineStr"/>
-      <c r="AB171" s="9" t="inlineStr"/>
+      <c r="AB171" s="8" t="inlineStr"/>
+      <c r="AC171" s="9" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" s="2" t="inlineStr">
@@ -12394,7 +12674,8 @@
       <c r="Y172" s="7" t="inlineStr"/>
       <c r="Z172" s="8" t="inlineStr"/>
       <c r="AA172" s="8" t="inlineStr"/>
-      <c r="AB172" s="9" t="inlineStr"/>
+      <c r="AB172" s="8" t="inlineStr"/>
+      <c r="AC172" s="9" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" s="2" t="inlineStr">
@@ -12450,7 +12731,8 @@
       <c r="Y173" s="7" t="inlineStr"/>
       <c r="Z173" s="8" t="inlineStr"/>
       <c r="AA173" s="8" t="inlineStr"/>
-      <c r="AB173" s="9" t="inlineStr"/>
+      <c r="AB173" s="8" t="inlineStr"/>
+      <c r="AC173" s="9" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" s="2" t="inlineStr">
@@ -12506,10 +12788,11 @@
       <c r="Y174" s="7" t="inlineStr"/>
       <c r="Z174" s="8" t="inlineStr"/>
       <c r="AA174" s="8" t="inlineStr"/>
-      <c r="AB174" s="9" t="inlineStr"/>
+      <c r="AB174" s="8" t="inlineStr"/>
+      <c r="AC174" s="9" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AB174"/>
+  <autoFilter ref="A1:AC174"/>
   <dataValidations count="1">
     <dataValidation sqref="H2:U174 Z2:AA174" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"X,"</formula1>
@@ -12525,7 +12808,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A37"/>
+  <dimension ref="A1:A38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="95" customWidth="1" min="1" max="1"/>
@@ -12577,198 +12860,205 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="11" t="inlineStr"/>
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>Sos kartı sütunu: o üründe hangi hazır sosun ayrı kartı gösteriliyor (sweetchili / cafedeparis / demiglace).</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="inlineStr">
+      <c r="A9" s="11" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="10" t="inlineStr">
         <is>
           <t>Nasıl düzeltirsiniz:</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="11" t="inlineStr">
-        <is>
-          <t>1. "Menü" sekmesinde her satır bir üründür.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="11" t="inlineStr">
         <is>
-          <t>2. Alerjen sütunlarında (G, M, Y, ...) ürün o alerjeni içeriyorsa hücreye X yazın,</t>
+          <t>1. "Menü" sekmesinde her satır bir üründür.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">   içermiyorsa hücreyi boş bırakın. Sarı hücreler doldurulacak alanlardır.</t>
+          <t>2. Alerjen sütunlarında (G, M, Y, ...) ürün o alerjeni içeriyorsa hücreye X yazın,</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="11" t="inlineStr">
         <is>
-          <t>3. İçindekiler sütunlarını serbestçe düzeltebilir, boş olanları doldurabilirsiniz.</t>
+          <t xml:space="preserve">   içermiyorsa hücreyi boş bırakın. Sarı hücreler doldurulacak alanlardır.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="11" t="inlineStr">
         <is>
-          <t>4. Enerji / protein / yağ / karbonhidrat sütunlarına porsiyon başına değerleri yazın; Alkol / Domuz türevi sütunlarına içeriyorsa X.</t>
+          <t>3. İçindekiler sütunlarını serbestçe düzeltebilir, boş olanları doldurabilirsiniz.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="11" t="inlineStr">
         <is>
-          <t>5. Fiyat değişikliklerini de bu dosyada yapabilirsiniz.</t>
+          <t>4. Enerji / protein / yağ / karbonhidrat sütunlarına porsiyon başına değerleri yazın; Alkol / Domuz türevi sütunlarına içeriyorsa X.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="11" t="inlineStr">
         <is>
+          <t>5. Fiyat değişikliklerini de bu dosyada yapabilirsiniz.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="11" t="inlineStr">
+        <is>
           <t>6. Dosyayı bana geri gönderin; menüyü güncellerim. QR kod değişmez.</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="11" t="inlineStr"/>
-    </row>
     <row r="18">
-      <c r="A18" s="10" t="inlineStr">
+      <c r="A18" s="11" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="10" t="inlineStr">
         <is>
           <t>Örnek satır:</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="11" t="inlineStr">
-        <is>
-          <t>Bölüm: Tatlılar | Grup: Tatlılar | Ürün: Künefe | Fiyat: 420</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="11" t="inlineStr">
         <is>
-          <t>İçindekiler: Kadayıf, dil peyniri, tereyağı, şerbet, Antep fıstığı</t>
+          <t>Bölüm: Tatlılar | Grup: Tatlılar | Ürün: Künefe | Fiyat: 420</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="11" t="inlineStr">
         <is>
+          <t>İçindekiler: Kadayıf, dil peyniri, tereyağı, şerbet, Antep fıstığı</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="11" t="inlineStr">
+        <is>
           <t>G: X   M: X   N: X   (gluten, süt ve sert kabuklu yemiş içerir)</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="11" t="inlineStr"/>
-    </row>
     <row r="23">
-      <c r="A23" s="10" t="inlineStr">
+      <c r="A23" s="11" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="10" t="inlineStr">
         <is>
           <t>Alerjen kodları:</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   G  =  Gluten</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">   M  =  Süt</t>
+          <t xml:space="preserve">   G  =  Gluten</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Y  =  Yumurta</t>
+          <t xml:space="preserve">   M  =  Süt</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">   B  =  Balık</t>
+          <t xml:space="preserve">   Y  =  Yumurta</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">   K  =  Kabuklu deniz ürünleri</t>
+          <t xml:space="preserve">   B  =  Balık</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">   S  =  Soya</t>
+          <t xml:space="preserve">   K  =  Kabuklu deniz ürünleri</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">   SS  =  Susam</t>
+          <t xml:space="preserve">   S  =  Soya</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">   N  =  Sert kabuklu yemişler</t>
+          <t xml:space="preserve">   SS  =  Susam</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">   F  =  Yer fıstığı</t>
+          <t xml:space="preserve">   N  =  Sert kabuklu yemişler</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">   H  =  Hardal</t>
+          <t xml:space="preserve">   F  =  Yer fıstığı</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">   C  =  Kereviz</t>
+          <t xml:space="preserve">   H  =  Hardal</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">   SO  =  Sülfit</t>
+          <t xml:space="preserve">   C  =  Kereviz</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">   MO  =  Yumuşakçalar</t>
+          <t xml:space="preserve">   SO  =  Sülfit</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   MO  =  Yumuşakçalar</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">   L  =  Acı bakla</t>
         </is>

</xml_diff>

<commit_message>
Menü güncelleme 18.09.2026 14:12
</commit_message>
<xml_diff>
--- a/KULE-alerjen-kontrol.xlsx
+++ b/KULE-alerjen-kontrol.xlsx
@@ -9,9 +9,10 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Menü" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nasıl kullanılır" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Teyit gerekenler" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Menü'!$A$1:$AC$174</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Menü'!$A$1:$AD$174</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -101,7 +102,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -128,10 +129,25 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -497,7 +513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC174"/>
+  <dimension ref="A1:AD174"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -527,8 +543,9 @@
     <col width="13" customWidth="1" min="25" max="25"/>
     <col width="9" customWidth="1" min="26" max="26"/>
     <col width="11" customWidth="1" min="27" max="27"/>
-    <col width="18" customWidth="1" min="28" max="28"/>
-    <col width="26" customWidth="1" min="29" max="29"/>
+    <col width="16" customWidth="1" min="28" max="28"/>
+    <col width="46" customWidth="1" min="29" max="29"/>
+    <col width="26" customWidth="1" min="30" max="30"/>
   </cols>
   <sheetData>
     <row r="1" ht="40" customHeight="1">
@@ -674,6 +691,11 @@
       </c>
       <c r="AC1" s="1" t="inlineStr">
         <is>
+          <t>Alerjen kaynağı (otomatik)</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
           <t>Notunuz</t>
         </is>
       </c>
@@ -729,7 +751,11 @@
       </c>
       <c r="K2" s="5" t="inlineStr"/>
       <c r="L2" s="5" t="inlineStr"/>
-      <c r="M2" s="5" t="inlineStr"/>
+      <c r="M2" s="5" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="N2" s="5" t="inlineStr"/>
       <c r="O2" s="5" t="inlineStr">
         <is>
@@ -757,7 +783,12 @@
       <c r="Z2" s="8" t="inlineStr"/>
       <c r="AA2" s="8" t="inlineStr"/>
       <c r="AB2" s="8" t="inlineStr"/>
-      <c r="AC2" s="9" t="inlineStr"/>
+      <c r="AC2" s="9" t="inlineStr">
+        <is>
+          <t>Y: sahanda yumurta, menemen · G: kalem böreği, sınırsız ekmek sepeti · M: kalem böreği, beyaz peynir, taze kaşar, çeçil peyniri, burgu peynir, lor peyniri, kaymak, tereyağı, nutella · N: acuka, nutella · S: nutella</t>
+        </is>
+      </c>
+      <c r="AD2" s="10" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -830,7 +861,12 @@
       <c r="Z3" s="8" t="inlineStr"/>
       <c r="AA3" s="8" t="inlineStr"/>
       <c r="AB3" s="8" t="inlineStr"/>
-      <c r="AC3" s="9" t="inlineStr"/>
+      <c r="AC3" s="9" t="inlineStr">
+        <is>
+          <t>Y: yumurta · M: tereyağı</t>
+        </is>
+      </c>
+      <c r="AD3" s="10" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -903,7 +939,12 @@
       <c r="Z4" s="8" t="inlineStr"/>
       <c r="AA4" s="8" t="inlineStr"/>
       <c r="AB4" s="8" t="inlineStr"/>
-      <c r="AC4" s="9" t="inlineStr"/>
+      <c r="AC4" s="9" t="inlineStr">
+        <is>
+          <t>Y: yumurta · M: beyaz peynir, tereyağı</t>
+        </is>
+      </c>
+      <c r="AD4" s="10" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -976,7 +1017,12 @@
       <c r="Z5" s="8" t="inlineStr"/>
       <c r="AA5" s="8" t="inlineStr"/>
       <c r="AB5" s="8" t="inlineStr"/>
-      <c r="AC5" s="9" t="inlineStr"/>
+      <c r="AC5" s="9" t="inlineStr">
+        <is>
+          <t>Y: yumurta · M: kaşar peyniri, tereyağı</t>
+        </is>
+      </c>
+      <c r="AD5" s="10" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1012,7 +1058,11 @@
           <t>Egg, kashar cheese, sucuk, sausage, pepper, butter, salt, sunflower oil</t>
         </is>
       </c>
-      <c r="H6" s="5" t="inlineStr"/>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="I6" s="5" t="inlineStr">
         <is>
           <t>X</t>
@@ -1049,7 +1099,12 @@
       <c r="Z6" s="8" t="inlineStr"/>
       <c r="AA6" s="8" t="inlineStr"/>
       <c r="AB6" s="8" t="inlineStr"/>
-      <c r="AC6" s="9" t="inlineStr"/>
+      <c r="AC6" s="9" t="inlineStr">
+        <is>
+          <t>Y: yumurta · M: kaşar peyniri, tereyağı · G: sosis</t>
+        </is>
+      </c>
+      <c r="AD6" s="10" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1122,7 +1177,12 @@
       <c r="Z7" s="8" t="inlineStr"/>
       <c r="AA7" s="8" t="inlineStr"/>
       <c r="AB7" s="8" t="inlineStr"/>
-      <c r="AC7" s="9" t="inlineStr"/>
+      <c r="AC7" s="9" t="inlineStr">
+        <is>
+          <t>Y: yumurta · M: tereyağı</t>
+        </is>
+      </c>
+      <c r="AD7" s="10" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1195,7 +1255,12 @@
       <c r="Z8" s="8" t="inlineStr"/>
       <c r="AA8" s="8" t="inlineStr"/>
       <c r="AB8" s="8" t="inlineStr"/>
-      <c r="AC8" s="9" t="inlineStr"/>
+      <c r="AC8" s="9" t="inlineStr">
+        <is>
+          <t>Y: yumurta · M: tereyağı</t>
+        </is>
+      </c>
+      <c r="AD8" s="10" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1268,7 +1333,12 @@
       <c r="Z9" s="8" t="inlineStr"/>
       <c r="AA9" s="8" t="inlineStr"/>
       <c r="AB9" s="8" t="inlineStr"/>
-      <c r="AC9" s="9" t="inlineStr"/>
+      <c r="AC9" s="9" t="inlineStr">
+        <is>
+          <t>Y: yumurta · M: tereyağı</t>
+        </is>
+      </c>
+      <c r="AD9" s="10" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1337,7 +1407,12 @@
       <c r="Z10" s="8" t="inlineStr"/>
       <c r="AA10" s="8" t="inlineStr"/>
       <c r="AB10" s="8" t="inlineStr"/>
-      <c r="AC10" s="9" t="inlineStr"/>
+      <c r="AC10" s="9" t="inlineStr">
+        <is>
+          <t>M: tereyağı</t>
+        </is>
+      </c>
+      <c r="AD10" s="10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1410,7 +1485,12 @@
       <c r="Z11" s="8" t="inlineStr"/>
       <c r="AA11" s="8" t="inlineStr"/>
       <c r="AB11" s="8" t="inlineStr"/>
-      <c r="AC11" s="9" t="inlineStr"/>
+      <c r="AC11" s="9" t="inlineStr">
+        <is>
+          <t>Y: yumurta · M: tereyağı</t>
+        </is>
+      </c>
+      <c r="AD11" s="10" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1483,7 +1563,12 @@
       <c r="Z12" s="8" t="inlineStr"/>
       <c r="AA12" s="8" t="inlineStr"/>
       <c r="AB12" s="8" t="inlineStr"/>
-      <c r="AC12" s="9" t="inlineStr"/>
+      <c r="AC12" s="9" t="inlineStr">
+        <is>
+          <t>Y: yumurta · M: kaşar peyniri, tereyağı</t>
+        </is>
+      </c>
+      <c r="AD12" s="10" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1552,7 +1637,12 @@
       <c r="Z13" s="8" t="inlineStr"/>
       <c r="AA13" s="8" t="inlineStr"/>
       <c r="AB13" s="8" t="inlineStr"/>
-      <c r="AC13" s="9" t="inlineStr"/>
+      <c r="AC13" s="9" t="inlineStr">
+        <is>
+          <t>M: tereyağı, kolot, dil peyniri</t>
+        </is>
+      </c>
+      <c r="AD13" s="10" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1625,7 +1715,12 @@
       <c r="Z14" s="8" t="inlineStr"/>
       <c r="AA14" s="8" t="inlineStr"/>
       <c r="AB14" s="8" t="inlineStr"/>
-      <c r="AC14" s="9" t="inlineStr"/>
+      <c r="AC14" s="9" t="inlineStr">
+        <is>
+          <t>G: tost ekmeği · M: çift kaşar peyniri, tereyağı</t>
+        </is>
+      </c>
+      <c r="AD14" s="10" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1698,7 +1793,12 @@
       <c r="Z15" s="8" t="inlineStr"/>
       <c r="AA15" s="8" t="inlineStr"/>
       <c r="AB15" s="8" t="inlineStr"/>
-      <c r="AC15" s="9" t="inlineStr"/>
+      <c r="AC15" s="9" t="inlineStr">
+        <is>
+          <t>G: tost ekmeği · M: kaşar peyniri, tereyağı</t>
+        </is>
+      </c>
+      <c r="AD15" s="10" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1763,7 +1863,12 @@
       <c r="Z16" s="8" t="inlineStr"/>
       <c r="AA16" s="8" t="inlineStr"/>
       <c r="AB16" s="8" t="inlineStr"/>
-      <c r="AC16" s="9" t="inlineStr"/>
+      <c r="AC16" s="9" t="inlineStr">
+        <is>
+          <t>içerik günlük değişir</t>
+        </is>
+      </c>
+      <c r="AD16" s="10" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1844,7 +1949,12 @@
       <c r="Z17" s="8" t="inlineStr"/>
       <c r="AA17" s="8" t="inlineStr"/>
       <c r="AB17" s="8" t="inlineStr"/>
-      <c r="AC17" s="9" t="inlineStr"/>
+      <c r="AC17" s="9" t="inlineStr">
+        <is>
+          <t>G: cajun baharatlı çıtır tavuk parçaları, un, soya sosu · Y: cajun baharatlı çıtır tavuk parçaları, yumurta · M: cajun baharatlı çıtır tavuk parçaları, süt · S: soya sosu</t>
+        </is>
+      </c>
+      <c r="AD17" s="10" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1925,7 +2035,12 @@
       <c r="Z18" s="8" t="inlineStr"/>
       <c r="AA18" s="8" t="inlineStr"/>
       <c r="AB18" s="8" t="inlineStr"/>
-      <c r="AC18" s="9" t="inlineStr"/>
+      <c r="AC18" s="9" t="inlineStr">
+        <is>
+          <t>G: çıtır tavuk, un, soya sosu, sigara böreği, soğan halkası, mozzarella stick, sosis · Y: çıtır tavuk, yumurta · M: çıtır tavuk, süt, sigara böreği, mozzarella stick · S: soya sosu</t>
+        </is>
+      </c>
+      <c r="AD18" s="10" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1991,6 +2106,7 @@
       <c r="AA19" s="8" t="inlineStr"/>
       <c r="AB19" s="8" t="inlineStr"/>
       <c r="AC19" s="9" t="inlineStr"/>
+      <c r="AD19" s="10" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -2056,6 +2172,7 @@
       <c r="AA20" s="8" t="inlineStr"/>
       <c r="AB20" s="8" t="inlineStr"/>
       <c r="AC20" s="9" t="inlineStr"/>
+      <c r="AD20" s="10" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -2124,7 +2241,12 @@
       <c r="Z21" s="8" t="inlineStr"/>
       <c r="AA21" s="8" t="inlineStr"/>
       <c r="AB21" s="8" t="inlineStr"/>
-      <c r="AC21" s="9" t="inlineStr"/>
+      <c r="AC21" s="9" t="inlineStr">
+        <is>
+          <t>G: ızgara sosis</t>
+        </is>
+      </c>
+      <c r="AD21" s="10" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -2166,11 +2288,7 @@
         </is>
       </c>
       <c r="I22" s="5" t="inlineStr"/>
-      <c r="J22" s="5" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J22" s="5" t="inlineStr"/>
       <c r="K22" s="5" t="inlineStr"/>
       <c r="L22" s="5" t="inlineStr"/>
       <c r="M22" s="5" t="inlineStr"/>
@@ -2197,7 +2315,12 @@
       <c r="Z22" s="8" t="inlineStr"/>
       <c r="AA22" s="8" t="inlineStr"/>
       <c r="AB22" s="8" t="inlineStr"/>
-      <c r="AC22" s="9" t="inlineStr"/>
+      <c r="AC22" s="9" t="inlineStr">
+        <is>
+          <t>G: soğan halkası, galeta unu</t>
+        </is>
+      </c>
+      <c r="AD22" s="10" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -2270,7 +2393,12 @@
       <c r="Z23" s="8" t="inlineStr"/>
       <c r="AA23" s="8" t="inlineStr"/>
       <c r="AB23" s="8" t="inlineStr"/>
-      <c r="AC23" s="9" t="inlineStr"/>
+      <c r="AC23" s="9" t="inlineStr">
+        <is>
+          <t>G: sigara böreği, yufka · M: sigara böreği, beyaz peynir</t>
+        </is>
+      </c>
+      <c r="AD23" s="10" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -2336,6 +2464,7 @@
       <c r="AA24" s="8" t="inlineStr"/>
       <c r="AB24" s="8" t="inlineStr"/>
       <c r="AC24" s="9" t="inlineStr"/>
+      <c r="AD24" s="10" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -2401,6 +2530,7 @@
       <c r="AA25" s="8" t="inlineStr"/>
       <c r="AB25" s="8" t="inlineStr"/>
       <c r="AC25" s="9" t="inlineStr"/>
+      <c r="AD25" s="10" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -2469,7 +2599,12 @@
       <c r="Z26" s="8" t="inlineStr"/>
       <c r="AA26" s="8" t="inlineStr"/>
       <c r="AB26" s="8" t="inlineStr"/>
-      <c r="AC26" s="9" t="inlineStr"/>
+      <c r="AC26" s="9" t="inlineStr">
+        <is>
+          <t>G: şişte köfte</t>
+        </is>
+      </c>
+      <c r="AD26" s="10" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2554,7 +2689,12 @@
       <c r="Z27" s="8" t="inlineStr"/>
       <c r="AA27" s="8" t="inlineStr"/>
       <c r="AB27" s="8" t="inlineStr"/>
-      <c r="AC27" s="9" t="inlineStr"/>
+      <c r="AC27" s="9" t="inlineStr">
+        <is>
+          <t>G: kruton ekmek · M: parmesan · Y: sezar sos, mayonez · B: sezar sos, ançüez · H: sezar sos, hardal</t>
+        </is>
+      </c>
+      <c r="AD27" s="10" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2639,7 +2779,12 @@
       <c r="Z28" s="8" t="inlineStr"/>
       <c r="AA28" s="8" t="inlineStr"/>
       <c r="AB28" s="8" t="inlineStr"/>
-      <c r="AC28" s="9" t="inlineStr"/>
+      <c r="AC28" s="9" t="inlineStr">
+        <is>
+          <t>G: cajun tavuk, un, pane, galeta unu, soya sosu · Y: cajun tavuk, yumurta · M: cajun tavuk, süt · S: cajun tavuk, soya sosu · H: ballı hardal sos</t>
+        </is>
+      </c>
+      <c r="AD28" s="10" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2716,7 +2861,12 @@
       <c r="Z29" s="8" t="inlineStr"/>
       <c r="AA29" s="8" t="inlineStr"/>
       <c r="AB29" s="8" t="inlineStr"/>
-      <c r="AC29" s="9" t="inlineStr"/>
+      <c r="AC29" s="9" t="inlineStr">
+        <is>
+          <t>G: spagetti · N: fesleğenli pesto sos · M: fesleğenli pesto sos, parmesan</t>
+        </is>
+      </c>
+      <c r="AD29" s="10" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2789,7 +2939,12 @@
       <c r="Z30" s="8" t="inlineStr"/>
       <c r="AA30" s="8" t="inlineStr"/>
       <c r="AB30" s="8" t="inlineStr"/>
-      <c r="AC30" s="9" t="inlineStr"/>
+      <c r="AC30" s="9" t="inlineStr">
+        <is>
+          <t>G: makarna · M: cheddar, kaşar, krema, tereyağı</t>
+        </is>
+      </c>
+      <c r="AD30" s="10" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2866,7 +3021,12 @@
       <c r="Z31" s="8" t="inlineStr"/>
       <c r="AA31" s="8" t="inlineStr"/>
       <c r="AB31" s="8" t="inlineStr"/>
-      <c r="AC31" s="9" t="inlineStr"/>
+      <c r="AC31" s="9" t="inlineStr">
+        <is>
+          <t>G: penne · N: fesleğenli pesto sos · M: fesleğenli pesto sos</t>
+        </is>
+      </c>
+      <c r="AD31" s="10" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2912,11 +3072,7 @@
           <t>X</t>
         </is>
       </c>
-      <c r="J32" s="5" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J32" s="5" t="inlineStr"/>
       <c r="K32" s="5" t="inlineStr"/>
       <c r="L32" s="5" t="inlineStr"/>
       <c r="M32" s="5" t="inlineStr"/>
@@ -2943,7 +3099,12 @@
       <c r="Z32" s="8" t="inlineStr"/>
       <c r="AA32" s="8" t="inlineStr"/>
       <c r="AB32" s="8" t="inlineStr"/>
-      <c r="AC32" s="9" t="inlineStr"/>
+      <c r="AC32" s="9" t="inlineStr">
+        <is>
+          <t>G: fettuccine · M: krema, parmesan, tereyağı</t>
+        </is>
+      </c>
+      <c r="AD32" s="10" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2985,11 +3146,7 @@
         </is>
       </c>
       <c r="I33" s="5" t="inlineStr"/>
-      <c r="J33" s="5" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J33" s="5" t="inlineStr"/>
       <c r="K33" s="5" t="inlineStr"/>
       <c r="L33" s="5" t="inlineStr"/>
       <c r="M33" s="5" t="inlineStr">
@@ -3024,7 +3181,12 @@
       <c r="Z33" s="8" t="inlineStr"/>
       <c r="AA33" s="8" t="inlineStr"/>
       <c r="AB33" s="8" t="inlineStr"/>
-      <c r="AC33" s="9" t="inlineStr"/>
+      <c r="AC33" s="9" t="inlineStr">
+        <is>
+          <t>G: noodle, soya sos · S: soya filizi, soya sos · SS: susam yağı, susam</t>
+        </is>
+      </c>
+      <c r="AD33" s="10" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -3066,11 +3228,7 @@
         </is>
       </c>
       <c r="I34" s="5" t="inlineStr"/>
-      <c r="J34" s="5" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J34" s="5" t="inlineStr"/>
       <c r="K34" s="5" t="inlineStr"/>
       <c r="L34" s="5" t="inlineStr"/>
       <c r="M34" s="5" t="inlineStr">
@@ -3105,7 +3263,12 @@
       <c r="Z34" s="8" t="inlineStr"/>
       <c r="AA34" s="8" t="inlineStr"/>
       <c r="AB34" s="8" t="inlineStr"/>
-      <c r="AC34" s="9" t="inlineStr"/>
+      <c r="AC34" s="9" t="inlineStr">
+        <is>
+          <t>G: noodle, soya sos · S: soya filizi, soya sos · SS: susam yağı, susam</t>
+        </is>
+      </c>
+      <c r="AD34" s="10" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -3133,12 +3296,12 @@
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>180 g burger köftesi, kıvırcık, domates, turşu, mantar sos (mantar, krema, tuz, karabiber), hamburger sosu (mayonez, Sweet Chili sos, az acı, tuz, pul biber), patates ve Sweet Chili sos eşliğinde</t>
+          <t>180 g burger köftesi, susamlı burger ekmeği, kıvırcık, domates, turşu, mantar sos (mantar, krema, tuz, karabiber), hamburger sosu (mayonez, Sweet Chili sos, az acı, tuz, pul biber), patates ve Sweet Chili sos eşliğinde</t>
         </is>
       </c>
       <c r="G35" s="4" t="inlineStr">
         <is>
-          <t>180 g beef patty, lettuce, tomato, pickles, mushroom sauce (mushroom, cream, salt, black pepper), burger sauce (mayonnaise, sweet chilli sauce, mild chilli, salt, chilli flakes), served with fries and sweet chilli sauce</t>
+          <t>180 g beef patty, sesame burger bun, lettuce, tomato, pickles, mushroom sauce (mushroom, cream, salt, black pepper), burger sauce (mayonnaise, sweet chilli sauce, mild chilli, salt, chilli flakes), served with fries and sweet chilli sauce</t>
         </is>
       </c>
       <c r="H35" s="5" t="inlineStr">
@@ -3190,7 +3353,12 @@
           <t>sweetchili</t>
         </is>
       </c>
-      <c r="AC35" s="9" t="inlineStr"/>
+      <c r="AC35" s="9" t="inlineStr">
+        <is>
+          <t>G: burger köftesi, susamlı burger ekmeği · SS: susamlı burger ekmeği · M: mantar sos, krema · Y: hamburger sosu, mayonez</t>
+        </is>
+      </c>
+      <c r="AD35" s="10" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -3218,12 +3386,12 @@
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>180 g burger köftesi, kıvırcık, domates, turşu, cheddar peyniri, hamburger sosu (mayonez, Sweet Chili sos, az acı, tuz, pul biber), patates ve Sweet Chili sos eşliğinde</t>
+          <t>180 g burger köftesi, susamlı burger ekmeği, kıvırcık, domates, turşu, cheddar peyniri, hamburger sosu (mayonez, Sweet Chili sos, az acı, tuz, pul biber), patates ve Sweet Chili sos eşliğinde</t>
         </is>
       </c>
       <c r="G36" s="4" t="inlineStr">
         <is>
-          <t>180 g beef patty, lettuce, tomato, pickles, cheddar, burger sauce (mayonnaise, sweet chilli sauce, mild chilli, salt, chilli flakes), served with fries and sweet chilli sauce</t>
+          <t>180 g beef patty, sesame burger bun, lettuce, tomato, pickles, cheddar, burger sauce (mayonnaise, sweet chilli sauce, mild chilli, salt, chilli flakes), served with fries and sweet chilli sauce</t>
         </is>
       </c>
       <c r="H36" s="5" t="inlineStr">
@@ -3275,7 +3443,12 @@
           <t>sweetchili</t>
         </is>
       </c>
-      <c r="AC36" s="9" t="inlineStr"/>
+      <c r="AC36" s="9" t="inlineStr">
+        <is>
+          <t>G: burger köftesi, susamlı burger ekmeği · SS: susamlı burger ekmeği · M: cheddar peyniri · Y: hamburger sosu, mayonez</t>
+        </is>
+      </c>
+      <c r="AD36" s="10" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -3303,12 +3476,12 @@
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>360 g burger köftesi, kıvırcık, domates, turşu, cheddar peyniri, hamburger sosu (mayonez, Sweet Chili sos, az acı, tuz, pul biber), patates ve Sweet Chili sos eşliğinde</t>
+          <t>360 g burger köftesi, susamlı burger ekmeği, kıvırcık, domates, turşu, cheddar peyniri, hamburger sosu (mayonez, Sweet Chili sos, az acı, tuz, pul biber), patates ve Sweet Chili sos eşliğinde</t>
         </is>
       </c>
       <c r="G37" s="4" t="inlineStr">
         <is>
-          <t>360 g beef patty, lettuce, tomato, pickles, cheddar, burger sauce (mayonnaise, sweet chilli sauce, mild chilli, salt, chilli flakes), served with fries and sweet chilli sauce</t>
+          <t>360 g beef patty, sesame burger bun, lettuce, tomato, pickles, cheddar, burger sauce (mayonnaise, sweet chilli sauce, mild chilli, salt, chilli flakes), served with fries and sweet chilli sauce</t>
         </is>
       </c>
       <c r="H37" s="5" t="inlineStr">
@@ -3360,7 +3533,12 @@
           <t>sweetchili</t>
         </is>
       </c>
-      <c r="AC37" s="9" t="inlineStr"/>
+      <c r="AC37" s="9" t="inlineStr">
+        <is>
+          <t>G: burger köftesi, susamlı burger ekmeği · SS: susamlı burger ekmeği · M: cheddar peyniri · Y: hamburger sosu, mayonez</t>
+        </is>
+      </c>
+      <c r="AD37" s="10" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -3388,12 +3566,12 @@
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>180 g özel soslu tavuk (yumurta, un, süt, panko, galeta unu, pane, soya sosu, tuz, karabiber, Cajun baharatı), kıvırcık, domates, turşu, cheddar peyniri, hamburger sosu (mayonez, Sweet Chili sos, az acı, tuz, pul biber), patates ve Sweet Chili sos eşliğinde</t>
+          <t>180 g özel soslu tavuk (yumurta, un, süt, panko, galeta unu, pane, soya sosu, tuz, karabiber, Cajun baharatı), susamlı burger ekmeği, kıvırcık, domates, turşu, cheddar peyniri, hamburger sosu (mayonez, Sweet Chili sos, az acı, tuz, pul biber), patates ve Sweet Chili sos eşliğinde</t>
         </is>
       </c>
       <c r="G38" s="4" t="inlineStr">
         <is>
-          <t>180 g chicken in special coating (egg, flour, milk, panko, breadcrumbs, breading, soy sauce, salt, black pepper, Cajun spice), lettuce, tomato, pickles, cheddar, burger sauce (mayonnaise, sweet chilli sauce, mild chilli, salt, chilli flakes), served with fries and sweet chilli sauce</t>
+          <t>180 g chicken in special coating (egg, flour, milk, panko, breadcrumbs, breading, soy sauce, salt, black pepper, Cajun spice), sesame burger bun, lettuce, tomato, pickles, cheddar, burger sauce (mayonnaise, sweet chilli sauce, mild chilli, salt, chilli flakes), served with fries and sweet chilli sauce</t>
         </is>
       </c>
       <c r="H38" s="5" t="inlineStr">
@@ -3449,7 +3627,12 @@
           <t>sweetchili</t>
         </is>
       </c>
-      <c r="AC38" s="9" t="inlineStr"/>
+      <c r="AC38" s="9" t="inlineStr">
+        <is>
+          <t>G: özel soslu tavuk, un, panko, galeta unu, pane, soya sosu, susamlı burger ekmeği · Y: özel soslu tavuk, yumurta, hamburger sosu, mayonez · M: özel soslu tavuk, süt, cheddar peyniri · S: özel soslu tavuk, soya sosu · SS: susamlı burger ekmeği</t>
+        </is>
+      </c>
+      <c r="AD38" s="10" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -3477,12 +3660,12 @@
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>170 g jülyen et, soğan, renkli biberler, kaşar peyniri, özel sos (soya sosu, Cajun baharatı), patates ve Sweet Chili sos eşliğinde</t>
+          <t>170 g jülyen et, lavaş, soğan, renkli biberler, kaşar peyniri, özel sos (soya sosu, Cajun baharatı), patates ve Sweet Chili sos eşliğinde</t>
         </is>
       </c>
       <c r="G39" s="4" t="inlineStr">
         <is>
-          <t>170 g julienne beef, onion, bell peppers, kashar cheese, special sauce (soy sauce, Cajun spice), served with fries and sweet chilli sauce</t>
+          <t>170 g julienne beef, lavash, onion, bell peppers, kashar cheese, special sauce (soy sauce, Cajun spice), served with fries and sweet chilli sauce</t>
         </is>
       </c>
       <c r="H39" s="5" t="inlineStr">
@@ -3495,11 +3678,7 @@
           <t>X</t>
         </is>
       </c>
-      <c r="J39" s="5" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J39" s="5" t="inlineStr"/>
       <c r="K39" s="5" t="inlineStr"/>
       <c r="L39" s="5" t="inlineStr"/>
       <c r="M39" s="5" t="inlineStr">
@@ -3534,7 +3713,12 @@
           <t>sweetchili</t>
         </is>
       </c>
-      <c r="AC39" s="9" t="inlineStr"/>
+      <c r="AC39" s="9" t="inlineStr">
+        <is>
+          <t>G: lavaş, soya sosu · M: kaşar peyniri · S: soya sosu</t>
+        </is>
+      </c>
+      <c r="AD39" s="10" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -3562,12 +3746,12 @@
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>170 g jülyen tavuk, soğan, renkli biberler, kaşar peyniri, özel sos (soya sosu, Cajun baharatı), patates ve Sweet Chili sos eşliğinde</t>
+          <t>170 g jülyen tavuk, lavaş, soğan, renkli biberler, kaşar peyniri, özel sos (soya sosu, Cajun baharatı), patates ve Sweet Chili sos eşliğinde</t>
         </is>
       </c>
       <c r="G40" s="4" t="inlineStr">
         <is>
-          <t>170 g julienne chicken, onion, bell peppers, kashar cheese, special sauce (soy sauce, Cajun spice), served with fries and sweet chilli sauce</t>
+          <t>170 g julienne chicken, lavash, onion, bell peppers, kashar cheese, special sauce (soy sauce, Cajun spice), served with fries and sweet chilli sauce</t>
         </is>
       </c>
       <c r="H40" s="5" t="inlineStr">
@@ -3615,7 +3799,12 @@
           <t>sweetchili</t>
         </is>
       </c>
-      <c r="AC40" s="9" t="inlineStr"/>
+      <c r="AC40" s="9" t="inlineStr">
+        <is>
+          <t>G: lavaş, soya sosu · M: kaşar peyniri · S: soya sosu</t>
+        </is>
+      </c>
+      <c r="AD40" s="10" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -3643,12 +3832,12 @@
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>170 g köfte, soğan, renkli biberler, kaşar peyniri, özel sos (soya sosu, Cajun baharatı), patates ve Sweet Chili sos eşliğinde</t>
+          <t>170 g köfte, lavaş, soğan, renkli biberler, kaşar peyniri, özel sos (soya sosu, Cajun baharatı), patates ve Sweet Chili sos eşliğinde</t>
         </is>
       </c>
       <c r="G41" s="4" t="inlineStr">
         <is>
-          <t>170 g meatballs, onion, bell peppers, kashar cheese, special sauce (soy sauce, Cajun spice), served with fries and sweet chilli sauce</t>
+          <t>170 g meatballs, lavash, onion, bell peppers, kashar cheese, special sauce (soy sauce, Cajun spice), served with fries and sweet chilli sauce</t>
         </is>
       </c>
       <c r="H41" s="5" t="inlineStr">
@@ -3696,7 +3885,12 @@
           <t>sweetchili</t>
         </is>
       </c>
-      <c r="AC41" s="9" t="inlineStr"/>
+      <c r="AC41" s="9" t="inlineStr">
+        <is>
+          <t>G: köfte, lavaş, soya sosu · M: kaşar peyniri · S: soya sosu</t>
+        </is>
+      </c>
+      <c r="AD41" s="10" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -3765,7 +3959,12 @@
       <c r="Z42" s="8" t="inlineStr"/>
       <c r="AA42" s="8" t="inlineStr"/>
       <c r="AB42" s="8" t="inlineStr"/>
-      <c r="AC42" s="9" t="inlineStr"/>
+      <c r="AC42" s="9" t="inlineStr">
+        <is>
+          <t>G: anne köfte, lavaş</t>
+        </is>
+      </c>
+      <c r="AD42" s="10" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -3838,7 +4037,12 @@
       <c r="Z43" s="8" t="inlineStr"/>
       <c r="AA43" s="8" t="inlineStr"/>
       <c r="AB43" s="8" t="inlineStr"/>
-      <c r="AC43" s="9" t="inlineStr"/>
+      <c r="AC43" s="9" t="inlineStr">
+        <is>
+          <t>G: köfte · M: süzme yoğurt</t>
+        </is>
+      </c>
+      <c r="AD43" s="10" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -3911,7 +4115,12 @@
       <c r="Z44" s="8" t="inlineStr"/>
       <c r="AA44" s="8" t="inlineStr"/>
       <c r="AB44" s="8" t="inlineStr"/>
-      <c r="AC44" s="9" t="inlineStr"/>
+      <c r="AC44" s="9" t="inlineStr">
+        <is>
+          <t>G: köfte · M: patlıcan beğendi, süt, kaşar peyniri</t>
+        </is>
+      </c>
+      <c r="AD44" s="10" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -3984,7 +4193,12 @@
       <c r="Z45" s="8" t="inlineStr"/>
       <c r="AA45" s="8" t="inlineStr"/>
       <c r="AB45" s="8" t="inlineStr"/>
-      <c r="AC45" s="9" t="inlineStr"/>
+      <c r="AC45" s="9" t="inlineStr">
+        <is>
+          <t>M: süzme yoğurt, özel kaymak sos, kaymak, tereyağı · G: çıtır yufka</t>
+        </is>
+      </c>
+      <c r="AD45" s="10" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -4033,7 +4247,11 @@
       <c r="N46" s="5" t="inlineStr"/>
       <c r="O46" s="5" t="inlineStr"/>
       <c r="P46" s="5" t="inlineStr"/>
-      <c r="Q46" s="5" t="inlineStr"/>
+      <c r="Q46" s="5" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="R46" s="5" t="inlineStr"/>
       <c r="S46" s="5" t="inlineStr"/>
       <c r="T46" s="5" t="inlineStr"/>
@@ -4053,7 +4271,12 @@
       <c r="Z46" s="8" t="inlineStr"/>
       <c r="AA46" s="8" t="inlineStr"/>
       <c r="AB46" s="8" t="inlineStr"/>
-      <c r="AC46" s="9" t="inlineStr"/>
+      <c r="AC46" s="9" t="inlineStr">
+        <is>
+          <t>H: köri sos · M: krema</t>
+        </is>
+      </c>
+      <c r="AD46" s="10" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -4122,7 +4345,12 @@
       <c r="Z47" s="8" t="inlineStr"/>
       <c r="AA47" s="8" t="inlineStr"/>
       <c r="AB47" s="8" t="inlineStr"/>
-      <c r="AC47" s="9" t="inlineStr"/>
+      <c r="AC47" s="9" t="inlineStr">
+        <is>
+          <t>M: krema</t>
+        </is>
+      </c>
+      <c r="AD47" s="10" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -4188,6 +4416,7 @@
       <c r="AA48" s="8" t="inlineStr"/>
       <c r="AB48" s="8" t="inlineStr"/>
       <c r="AC48" s="9" t="inlineStr"/>
+      <c r="AD48" s="10" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -4253,6 +4482,7 @@
       <c r="AA49" s="8" t="inlineStr"/>
       <c r="AB49" s="8" t="inlineStr"/>
       <c r="AC49" s="9" t="inlineStr"/>
+      <c r="AD49" s="10" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -4321,7 +4551,12 @@
       <c r="Z50" s="8" t="inlineStr"/>
       <c r="AA50" s="8" t="inlineStr"/>
       <c r="AB50" s="8" t="inlineStr"/>
-      <c r="AC50" s="9" t="inlineStr"/>
+      <c r="AC50" s="9" t="inlineStr">
+        <is>
+          <t>M: patlıcan beğendi, süt, kaşar peyniri</t>
+        </is>
+      </c>
+      <c r="AD50" s="10" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -4398,7 +4633,12 @@
       <c r="Z51" s="8" t="inlineStr"/>
       <c r="AA51" s="8" t="inlineStr"/>
       <c r="AB51" s="8" t="inlineStr"/>
-      <c r="AC51" s="9" t="inlineStr"/>
+      <c r="AC51" s="9" t="inlineStr">
+        <is>
+          <t>G: panelenmiş tavuk, pane, galeta unu, un, soya sosu · Y: panelenmiş tavuk, yumurta · S: soya sosu</t>
+        </is>
+      </c>
+      <c r="AD51" s="10" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -4479,7 +4719,12 @@
       <c r="Z52" s="8" t="inlineStr"/>
       <c r="AA52" s="8" t="inlineStr"/>
       <c r="AB52" s="8" t="inlineStr"/>
-      <c r="AC52" s="9" t="inlineStr"/>
+      <c r="AC52" s="9" t="inlineStr">
+        <is>
+          <t>G: panelenmiş tavuk, pane, galeta unu, un, soya sosu · Y: panelenmiş tavuk, yumurta · S: soya sosu · M: mantar sos</t>
+        </is>
+      </c>
+      <c r="AD52" s="10" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -4560,7 +4805,12 @@
       <c r="Z53" s="8" t="inlineStr"/>
       <c r="AA53" s="8" t="inlineStr"/>
       <c r="AB53" s="8" t="inlineStr"/>
-      <c r="AC53" s="9" t="inlineStr"/>
+      <c r="AC53" s="9" t="inlineStr">
+        <is>
+          <t>G: panelenmiş tavuk, pane, galeta unu, un, soya sosu · Y: panelenmiş tavuk, yumurta · S: soya sosu · M: cheddar sos, cheddar, krema</t>
+        </is>
+      </c>
+      <c r="AD53" s="10" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -4613,11 +4863,7 @@
       <c r="N54" s="5" t="inlineStr"/>
       <c r="O54" s="5" t="inlineStr"/>
       <c r="P54" s="5" t="inlineStr"/>
-      <c r="Q54" s="5" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="Q54" s="5" t="inlineStr"/>
       <c r="R54" s="5" t="inlineStr"/>
       <c r="S54" s="5" t="inlineStr"/>
       <c r="T54" s="5" t="inlineStr"/>
@@ -4641,7 +4887,12 @@
           <t>cafedeparis</t>
         </is>
       </c>
-      <c r="AC54" s="9" t="inlineStr"/>
+      <c r="AC54" s="9" t="inlineStr">
+        <is>
+          <t>G: cafe de paris sos, Cafe de Paris Sos · M: cafe de paris sos, krema, Cafe de Paris Sos</t>
+        </is>
+      </c>
+      <c r="AD54" s="10" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -4710,7 +4961,12 @@
       <c r="Z55" s="8" t="inlineStr"/>
       <c r="AA55" s="8" t="inlineStr"/>
       <c r="AB55" s="8" t="inlineStr"/>
-      <c r="AC55" s="9" t="inlineStr"/>
+      <c r="AC55" s="9" t="inlineStr">
+        <is>
+          <t>M: cheddar sos, krema</t>
+        </is>
+      </c>
+      <c r="AD55" s="10" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -4787,7 +5043,12 @@
           <t>sweetchili</t>
         </is>
       </c>
-      <c r="AC56" s="9" t="inlineStr"/>
+      <c r="AC56" s="9" t="inlineStr">
+        <is>
+          <t>G: çıtır kaplama · Y: çıtır kaplama</t>
+        </is>
+      </c>
+      <c r="AD56" s="10" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -4856,7 +5117,12 @@
       <c r="Z57" s="8" t="inlineStr"/>
       <c r="AA57" s="8" t="inlineStr"/>
       <c r="AB57" s="8" t="inlineStr"/>
-      <c r="AC57" s="9" t="inlineStr"/>
+      <c r="AC57" s="9" t="inlineStr">
+        <is>
+          <t>G: köfte</t>
+        </is>
+      </c>
+      <c r="AD57" s="10" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -4922,6 +5188,7 @@
       <c r="AA58" s="8" t="inlineStr"/>
       <c r="AB58" s="8" t="inlineStr"/>
       <c r="AC58" s="9" t="inlineStr"/>
+      <c r="AD58" s="10" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -4987,6 +5254,7 @@
       <c r="AA59" s="8" t="inlineStr"/>
       <c r="AB59" s="8" t="inlineStr"/>
       <c r="AC59" s="9" t="inlineStr"/>
+      <c r="AD59" s="10" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -5052,6 +5320,7 @@
       <c r="AA60" s="8" t="inlineStr"/>
       <c r="AB60" s="8" t="inlineStr"/>
       <c r="AC60" s="9" t="inlineStr"/>
+      <c r="AD60" s="10" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -5117,6 +5386,7 @@
       <c r="AA61" s="8" t="inlineStr"/>
       <c r="AB61" s="8" t="inlineStr"/>
       <c r="AC61" s="9" t="inlineStr"/>
+      <c r="AD61" s="10" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -5193,7 +5463,12 @@
           <t>cafedeparis</t>
         </is>
       </c>
-      <c r="AC62" s="9" t="inlineStr"/>
+      <c r="AC62" s="9" t="inlineStr">
+        <is>
+          <t>M: mantar sos, krema, cafe de paris sos, Cafe de Paris Sos · G: cafe de paris sos, Cafe de Paris Sos</t>
+        </is>
+      </c>
+      <c r="AD62" s="10" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -5246,11 +5521,7 @@
       <c r="N63" s="5" t="inlineStr"/>
       <c r="O63" s="5" t="inlineStr"/>
       <c r="P63" s="5" t="inlineStr"/>
-      <c r="Q63" s="5" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="Q63" s="5" t="inlineStr"/>
       <c r="R63" s="5" t="inlineStr"/>
       <c r="S63" s="5" t="inlineStr"/>
       <c r="T63" s="5" t="inlineStr"/>
@@ -5274,7 +5545,12 @@
           <t>cafedeparis</t>
         </is>
       </c>
-      <c r="AC63" s="9" t="inlineStr"/>
+      <c r="AC63" s="9" t="inlineStr">
+        <is>
+          <t>G: cafe de paris sos, Cafe de Paris Sos · M: cafe de paris sos, Cafe de Paris Sos</t>
+        </is>
+      </c>
+      <c r="AD63" s="10" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -5355,7 +5631,12 @@
           <t>sweetchili</t>
         </is>
       </c>
-      <c r="AC64" s="9" t="inlineStr"/>
+      <c r="AC64" s="9" t="inlineStr">
+        <is>
+          <t>M: süzme yoğurt · Y: özel kule sos, mayonez · G: lavaş</t>
+        </is>
+      </c>
+      <c r="AD64" s="10" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -5436,7 +5717,12 @@
           <t>sweetchili</t>
         </is>
       </c>
-      <c r="AC65" s="9" t="inlineStr"/>
+      <c r="AC65" s="9" t="inlineStr">
+        <is>
+          <t>M: süzme yoğurt · Y: özel kule sos, mayonez · G: lavaş</t>
+        </is>
+      </c>
+      <c r="AD65" s="10" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -5482,11 +5768,7 @@
           <t>X</t>
         </is>
       </c>
-      <c r="J66" s="5" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J66" s="5" t="inlineStr"/>
       <c r="K66" s="5" t="inlineStr"/>
       <c r="L66" s="5" t="inlineStr"/>
       <c r="M66" s="5" t="inlineStr"/>
@@ -5513,7 +5795,12 @@
       <c r="Z66" s="8" t="inlineStr"/>
       <c r="AA66" s="8" t="inlineStr"/>
       <c r="AB66" s="8" t="inlineStr"/>
-      <c r="AC66" s="9" t="inlineStr"/>
+      <c r="AC66" s="9" t="inlineStr">
+        <is>
+          <t>G: bisküvi tabanı · M: bisküvi tabanı, krem peynir, krema</t>
+        </is>
+      </c>
+      <c r="AD66" s="10" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -5559,11 +5846,7 @@
           <t>X</t>
         </is>
       </c>
-      <c r="J67" s="5" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J67" s="5" t="inlineStr"/>
       <c r="K67" s="5" t="inlineStr"/>
       <c r="L67" s="5" t="inlineStr"/>
       <c r="M67" s="5" t="inlineStr"/>
@@ -5590,7 +5873,12 @@
       <c r="Z67" s="8" t="inlineStr"/>
       <c r="AA67" s="8" t="inlineStr"/>
       <c r="AB67" s="8" t="inlineStr"/>
-      <c r="AC67" s="9" t="inlineStr"/>
+      <c r="AC67" s="9" t="inlineStr">
+        <is>
+          <t>G: bisküvi tabanı · M: bisküvi tabanı, krem peynir, krema</t>
+        </is>
+      </c>
+      <c r="AD67" s="10" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -5636,11 +5924,7 @@
           <t>X</t>
         </is>
       </c>
-      <c r="J68" s="5" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J68" s="5" t="inlineStr"/>
       <c r="K68" s="5" t="inlineStr"/>
       <c r="L68" s="5" t="inlineStr"/>
       <c r="M68" s="5" t="inlineStr"/>
@@ -5671,7 +5955,12 @@
       <c r="Z68" s="8" t="inlineStr"/>
       <c r="AA68" s="8" t="inlineStr"/>
       <c r="AB68" s="8" t="inlineStr"/>
-      <c r="AC68" s="9" t="inlineStr"/>
+      <c r="AC68" s="9" t="inlineStr">
+        <is>
+          <t>G: bisküvi tabanı · M: bisküvi tabanı, krem peynir, süt reçeli · N: fındık</t>
+        </is>
+      </c>
+      <c r="AD68" s="10" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -5752,7 +6041,12 @@
       <c r="Z69" s="8" t="inlineStr"/>
       <c r="AA69" s="8" t="inlineStr"/>
       <c r="AB69" s="8" t="inlineStr"/>
-      <c r="AC69" s="9" t="inlineStr"/>
+      <c r="AC69" s="9" t="inlineStr">
+        <is>
+          <t>G: kakaolu kek · Y: kakaolu kek · M: kakaolu kek, çikolata krema · S: çikolata krema</t>
+        </is>
+      </c>
+      <c r="AD69" s="10" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -5833,7 +6127,12 @@
       <c r="Z70" s="8" t="inlineStr"/>
       <c r="AA70" s="8" t="inlineStr"/>
       <c r="AB70" s="8" t="inlineStr"/>
-      <c r="AC70" s="9" t="inlineStr"/>
+      <c r="AC70" s="9" t="inlineStr">
+        <is>
+          <t>G: linzer hamuru · Y: linzer hamuru · M: linzer hamuru, krema · N: linzer hamuru</t>
+        </is>
+      </c>
+      <c r="AD70" s="10" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -5910,7 +6209,12 @@
       <c r="Z71" s="8" t="inlineStr"/>
       <c r="AA71" s="8" t="inlineStr"/>
       <c r="AB71" s="8" t="inlineStr"/>
-      <c r="AC71" s="9" t="inlineStr"/>
+      <c r="AC71" s="9" t="inlineStr">
+        <is>
+          <t>G: lotus bisküvi, karamelize bisküvi kreması · S: lotus bisküvi, karamelize bisküvi kreması · M: krema</t>
+        </is>
+      </c>
+      <c r="AD71" s="10" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -5995,7 +6299,12 @@
       <c r="Z72" s="8" t="inlineStr"/>
       <c r="AA72" s="8" t="inlineStr"/>
       <c r="AB72" s="8" t="inlineStr"/>
-      <c r="AC72" s="9" t="inlineStr"/>
+      <c r="AC72" s="9" t="inlineStr">
+        <is>
+          <t>G: kakaolu kek · Y: kakaolu kek · M: kakaolu kek, karamel, çikolata · F: yer fıstığı · S: çikolata</t>
+        </is>
+      </c>
+      <c r="AD72" s="10" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -6044,11 +6353,7 @@
       <c r="J73" s="5" t="inlineStr"/>
       <c r="K73" s="5" t="inlineStr"/>
       <c r="L73" s="5" t="inlineStr"/>
-      <c r="M73" s="5" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="M73" s="5" t="inlineStr"/>
       <c r="N73" s="5" t="inlineStr"/>
       <c r="O73" s="5" t="inlineStr"/>
       <c r="P73" s="5" t="inlineStr"/>
@@ -6072,7 +6377,12 @@
       <c r="Z73" s="8" t="inlineStr"/>
       <c r="AA73" s="8" t="inlineStr"/>
       <c r="AB73" s="8" t="inlineStr"/>
-      <c r="AC73" s="9" t="inlineStr"/>
+      <c r="AC73" s="9" t="inlineStr">
+        <is>
+          <t>G: bisküvi · M: tereyağı, süt</t>
+        </is>
+      </c>
+      <c r="AD73" s="10" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -6149,7 +6459,12 @@
       <c r="Z74" s="8" t="inlineStr"/>
       <c r="AA74" s="8" t="inlineStr"/>
       <c r="AB74" s="8" t="inlineStr"/>
-      <c r="AC74" s="9" t="inlineStr"/>
+      <c r="AC74" s="9" t="inlineStr">
+        <is>
+          <t>G: kedidili bisküvi · Y: kedidili bisküvi, yumurta · M: mascarpone</t>
+        </is>
+      </c>
+      <c r="AD74" s="10" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -6226,7 +6541,12 @@
       <c r="Z75" s="8" t="inlineStr"/>
       <c r="AA75" s="8" t="inlineStr"/>
       <c r="AB75" s="8" t="inlineStr"/>
-      <c r="AC75" s="9" t="inlineStr"/>
+      <c r="AC75" s="9" t="inlineStr">
+        <is>
+          <t>G: kat kat ballı kek · Y: kat kat ballı kek · M: kat kat ballı kek, özel krema</t>
+        </is>
+      </c>
+      <c r="AD75" s="10" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -6307,7 +6627,12 @@
       <c r="Z76" s="8" t="inlineStr"/>
       <c r="AA76" s="8" t="inlineStr"/>
       <c r="AB76" s="8" t="inlineStr"/>
-      <c r="AC76" s="9" t="inlineStr"/>
+      <c r="AC76" s="9" t="inlineStr">
+        <is>
+          <t>M: çikolata, tereyağı · S: çikolata · Y: yumurta · G: un</t>
+        </is>
+      </c>
+      <c r="AD76" s="10" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -6349,11 +6674,7 @@
           <t>X</t>
         </is>
       </c>
-      <c r="J77" s="5" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J77" s="5" t="inlineStr"/>
       <c r="K77" s="5" t="inlineStr"/>
       <c r="L77" s="5" t="inlineStr"/>
       <c r="M77" s="5" t="inlineStr">
@@ -6388,7 +6709,12 @@
       <c r="Z77" s="8" t="inlineStr"/>
       <c r="AA77" s="8" t="inlineStr"/>
       <c r="AB77" s="8" t="inlineStr"/>
-      <c r="AC77" s="9" t="inlineStr"/>
+      <c r="AC77" s="9" t="inlineStr">
+        <is>
+          <t>M: antep fıstığı kreması, beyaz çikolata · N: antep fıstığı kreması · S: beyaz çikolata</t>
+        </is>
+      </c>
+      <c r="AD77" s="10" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -6430,11 +6756,7 @@
           <t>X</t>
         </is>
       </c>
-      <c r="J78" s="5" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J78" s="5" t="inlineStr"/>
       <c r="K78" s="5" t="inlineStr"/>
       <c r="L78" s="5" t="inlineStr"/>
       <c r="M78" s="5" t="inlineStr">
@@ -6465,7 +6787,12 @@
       <c r="Z78" s="8" t="inlineStr"/>
       <c r="AA78" s="8" t="inlineStr"/>
       <c r="AB78" s="8" t="inlineStr"/>
-      <c r="AC78" s="9" t="inlineStr"/>
+      <c r="AC78" s="9" t="inlineStr">
+        <is>
+          <t>M: limon kreması, beyaz çikolata · S: beyaz çikolata</t>
+        </is>
+      </c>
+      <c r="AD78" s="10" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -6507,11 +6834,7 @@
           <t>X</t>
         </is>
       </c>
-      <c r="J79" s="5" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J79" s="5" t="inlineStr"/>
       <c r="K79" s="5" t="inlineStr"/>
       <c r="L79" s="5" t="inlineStr"/>
       <c r="M79" s="5" t="inlineStr">
@@ -6542,7 +6865,12 @@
       <c r="Z79" s="8" t="inlineStr"/>
       <c r="AA79" s="8" t="inlineStr"/>
       <c r="AB79" s="8" t="inlineStr"/>
-      <c r="AC79" s="9" t="inlineStr"/>
+      <c r="AC79" s="9" t="inlineStr">
+        <is>
+          <t>M: mango kreması, beyaz çikolata · S: beyaz çikolata</t>
+        </is>
+      </c>
+      <c r="AD79" s="10" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -6584,11 +6912,7 @@
           <t>X</t>
         </is>
       </c>
-      <c r="J80" s="5" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J80" s="5" t="inlineStr"/>
       <c r="K80" s="5" t="inlineStr"/>
       <c r="L80" s="5" t="inlineStr"/>
       <c r="M80" s="5" t="inlineStr">
@@ -6619,7 +6943,12 @@
       <c r="Z80" s="8" t="inlineStr"/>
       <c r="AA80" s="8" t="inlineStr"/>
       <c r="AB80" s="8" t="inlineStr"/>
-      <c r="AC80" s="9" t="inlineStr"/>
+      <c r="AC80" s="9" t="inlineStr">
+        <is>
+          <t>M: hindistan cevizi kreması, çikolata · S: çikolata</t>
+        </is>
+      </c>
+      <c r="AD80" s="10" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -6685,6 +7014,7 @@
       <c r="AA81" s="8" t="inlineStr"/>
       <c r="AB81" s="8" t="inlineStr"/>
       <c r="AC81" s="9" t="inlineStr"/>
+      <c r="AD81" s="10" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -6753,7 +7083,12 @@
       <c r="Z82" s="8" t="inlineStr"/>
       <c r="AA82" s="8" t="inlineStr"/>
       <c r="AB82" s="8" t="inlineStr"/>
-      <c r="AC82" s="9" t="inlineStr"/>
+      <c r="AC82" s="9" t="inlineStr">
+        <is>
+          <t>M: süt, krema</t>
+        </is>
+      </c>
+      <c r="AD82" s="10" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -6822,7 +7157,12 @@
       <c r="Z83" s="8" t="inlineStr"/>
       <c r="AA83" s="8" t="inlineStr"/>
       <c r="AB83" s="8" t="inlineStr"/>
-      <c r="AC83" s="9" t="inlineStr"/>
+      <c r="AC83" s="9" t="inlineStr">
+        <is>
+          <t>M: süt, krema</t>
+        </is>
+      </c>
+      <c r="AD83" s="10" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -6888,6 +7228,7 @@
       <c r="AA84" s="8" t="inlineStr"/>
       <c r="AB84" s="8" t="inlineStr"/>
       <c r="AC84" s="9" t="inlineStr"/>
+      <c r="AD84" s="10" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -6953,6 +7294,7 @@
       <c r="AA85" s="8" t="inlineStr"/>
       <c r="AB85" s="8" t="inlineStr"/>
       <c r="AC85" s="9" t="inlineStr"/>
+      <c r="AD85" s="10" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -7021,7 +7363,12 @@
       <c r="Z86" s="8" t="inlineStr"/>
       <c r="AA86" s="8" t="inlineStr"/>
       <c r="AB86" s="8" t="inlineStr"/>
-      <c r="AC86" s="9" t="inlineStr"/>
+      <c r="AC86" s="9" t="inlineStr">
+        <is>
+          <t>M: az süt köpüğü</t>
+        </is>
+      </c>
+      <c r="AD86" s="10" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -7087,6 +7434,7 @@
       <c r="AA87" s="8" t="inlineStr"/>
       <c r="AB87" s="8" t="inlineStr"/>
       <c r="AC87" s="9" t="inlineStr"/>
+      <c r="AD87" s="10" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -7152,6 +7500,7 @@
       <c r="AA88" s="8" t="inlineStr"/>
       <c r="AB88" s="8" t="inlineStr"/>
       <c r="AC88" s="9" t="inlineStr"/>
+      <c r="AD88" s="10" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -7220,7 +7569,12 @@
       <c r="Z89" s="8" t="inlineStr"/>
       <c r="AA89" s="8" t="inlineStr"/>
       <c r="AB89" s="8" t="inlineStr"/>
-      <c r="AC89" s="9" t="inlineStr"/>
+      <c r="AC89" s="9" t="inlineStr">
+        <is>
+          <t>M: süt, süt köpüğü</t>
+        </is>
+      </c>
+      <c r="AD89" s="10" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -7289,7 +7643,12 @@
       <c r="Z90" s="8" t="inlineStr"/>
       <c r="AA90" s="8" t="inlineStr"/>
       <c r="AB90" s="8" t="inlineStr"/>
-      <c r="AC90" s="9" t="inlineStr"/>
+      <c r="AC90" s="9" t="inlineStr">
+        <is>
+          <t>M: süt, bol süt köpüğü</t>
+        </is>
+      </c>
+      <c r="AD90" s="10" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -7362,7 +7721,12 @@
       <c r="Z91" s="8" t="inlineStr"/>
       <c r="AA91" s="8" t="inlineStr"/>
       <c r="AB91" s="8" t="inlineStr"/>
-      <c r="AC91" s="9" t="inlineStr"/>
+      <c r="AC91" s="9" t="inlineStr">
+        <is>
+          <t>M: süt, çikolata · S: çikolata</t>
+        </is>
+      </c>
+      <c r="AD91" s="10" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -7435,7 +7799,12 @@
       <c r="Z92" s="8" t="inlineStr"/>
       <c r="AA92" s="8" t="inlineStr"/>
       <c r="AB92" s="8" t="inlineStr"/>
-      <c r="AC92" s="9" t="inlineStr"/>
+      <c r="AC92" s="9" t="inlineStr">
+        <is>
+          <t>M: süt, beyaz çikolata · S: beyaz çikolata</t>
+        </is>
+      </c>
+      <c r="AD92" s="10" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -7504,7 +7873,12 @@
       <c r="Z93" s="8" t="inlineStr"/>
       <c r="AA93" s="8" t="inlineStr"/>
       <c r="AB93" s="8" t="inlineStr"/>
-      <c r="AC93" s="9" t="inlineStr"/>
+      <c r="AC93" s="9" t="inlineStr">
+        <is>
+          <t>M: süt</t>
+        </is>
+      </c>
+      <c r="AD93" s="10" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -7573,7 +7947,12 @@
       <c r="Z94" s="8" t="inlineStr"/>
       <c r="AA94" s="8" t="inlineStr"/>
       <c r="AB94" s="8" t="inlineStr"/>
-      <c r="AC94" s="9" t="inlineStr"/>
+      <c r="AC94" s="9" t="inlineStr">
+        <is>
+          <t>M: süt</t>
+        </is>
+      </c>
+      <c r="AD94" s="10" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -7642,7 +8021,12 @@
       <c r="Z95" s="8" t="inlineStr"/>
       <c r="AA95" s="8" t="inlineStr"/>
       <c r="AB95" s="8" t="inlineStr"/>
-      <c r="AC95" s="9" t="inlineStr"/>
+      <c r="AC95" s="9" t="inlineStr">
+        <is>
+          <t>M: süt</t>
+        </is>
+      </c>
+      <c r="AD95" s="10" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -7711,7 +8095,12 @@
       <c r="Z96" s="8" t="inlineStr"/>
       <c r="AA96" s="8" t="inlineStr"/>
       <c r="AB96" s="8" t="inlineStr"/>
-      <c r="AC96" s="9" t="inlineStr"/>
+      <c r="AC96" s="9" t="inlineStr">
+        <is>
+          <t>M: süt</t>
+        </is>
+      </c>
+      <c r="AD96" s="10" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -7780,7 +8169,12 @@
       <c r="Z97" s="8" t="inlineStr"/>
       <c r="AA97" s="8" t="inlineStr"/>
       <c r="AB97" s="8" t="inlineStr"/>
-      <c r="AC97" s="9" t="inlineStr"/>
+      <c r="AC97" s="9" t="inlineStr">
+        <is>
+          <t>M: süt</t>
+        </is>
+      </c>
+      <c r="AD97" s="10" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -7849,7 +8243,12 @@
       <c r="Z98" s="8" t="inlineStr"/>
       <c r="AA98" s="8" t="inlineStr"/>
       <c r="AB98" s="8" t="inlineStr"/>
-      <c r="AC98" s="9" t="inlineStr"/>
+      <c r="AC98" s="9" t="inlineStr">
+        <is>
+          <t>M: süt</t>
+        </is>
+      </c>
+      <c r="AD98" s="10" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -7922,7 +8321,12 @@
       <c r="Z99" s="8" t="inlineStr"/>
       <c r="AA99" s="8" t="inlineStr"/>
       <c r="AB99" s="8" t="inlineStr"/>
-      <c r="AC99" s="9" t="inlineStr"/>
+      <c r="AC99" s="9" t="inlineStr">
+        <is>
+          <t>M: süt, karamel, çikolata · S: çikolata</t>
+        </is>
+      </c>
+      <c r="AD99" s="10" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -7991,7 +8395,12 @@
       <c r="Z100" s="8" t="inlineStr"/>
       <c r="AA100" s="8" t="inlineStr"/>
       <c r="AB100" s="8" t="inlineStr"/>
-      <c r="AC100" s="9" t="inlineStr"/>
+      <c r="AC100" s="9" t="inlineStr">
+        <is>
+          <t>M: süt</t>
+        </is>
+      </c>
+      <c r="AD100" s="10" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -8060,7 +8469,12 @@
       <c r="Z101" s="8" t="inlineStr"/>
       <c r="AA101" s="8" t="inlineStr"/>
       <c r="AB101" s="8" t="inlineStr"/>
-      <c r="AC101" s="9" t="inlineStr"/>
+      <c r="AC101" s="9" t="inlineStr">
+        <is>
+          <t>M: süt</t>
+        </is>
+      </c>
+      <c r="AD101" s="10" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -8133,7 +8547,12 @@
       <c r="Z102" s="8" t="inlineStr"/>
       <c r="AA102" s="8" t="inlineStr"/>
       <c r="AB102" s="8" t="inlineStr"/>
-      <c r="AC102" s="9" t="inlineStr"/>
+      <c r="AC102" s="9" t="inlineStr">
+        <is>
+          <t>M: süt, çikolata sosu · S: çikolata sosu</t>
+        </is>
+      </c>
+      <c r="AD102" s="10" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -8206,7 +8625,12 @@
       <c r="Z103" s="8" t="inlineStr"/>
       <c r="AA103" s="8" t="inlineStr"/>
       <c r="AB103" s="8" t="inlineStr"/>
-      <c r="AC103" s="9" t="inlineStr"/>
+      <c r="AC103" s="9" t="inlineStr">
+        <is>
+          <t>M: süt, çikolata sosu, karamel · S: çikolata sosu</t>
+        </is>
+      </c>
+      <c r="AD103" s="10" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -8279,7 +8703,12 @@
       <c r="Z104" s="8" t="inlineStr"/>
       <c r="AA104" s="8" t="inlineStr"/>
       <c r="AB104" s="8" t="inlineStr"/>
-      <c r="AC104" s="9" t="inlineStr"/>
+      <c r="AC104" s="9" t="inlineStr">
+        <is>
+          <t>M: süt, beyaz çikolata · S: beyaz çikolata</t>
+        </is>
+      </c>
+      <c r="AD104" s="10" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -8348,7 +8777,12 @@
       <c r="Z105" s="8" t="inlineStr"/>
       <c r="AA105" s="8" t="inlineStr"/>
       <c r="AB105" s="8" t="inlineStr"/>
-      <c r="AC105" s="9" t="inlineStr"/>
+      <c r="AC105" s="9" t="inlineStr">
+        <is>
+          <t>M: soğuk süt</t>
+        </is>
+      </c>
+      <c r="AD105" s="10" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -8414,6 +8848,7 @@
       <c r="AA106" s="8" t="inlineStr"/>
       <c r="AB106" s="8" t="inlineStr"/>
       <c r="AC106" s="9" t="inlineStr"/>
+      <c r="AD106" s="10" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -8482,7 +8917,12 @@
       <c r="Z107" s="8" t="inlineStr"/>
       <c r="AA107" s="8" t="inlineStr"/>
       <c r="AB107" s="8" t="inlineStr"/>
-      <c r="AC107" s="9" t="inlineStr"/>
+      <c r="AC107" s="9" t="inlineStr">
+        <is>
+          <t>M: soğuk süt, karamel</t>
+        </is>
+      </c>
+      <c r="AD107" s="10" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -8551,7 +8991,12 @@
       <c r="Z108" s="8" t="inlineStr"/>
       <c r="AA108" s="8" t="inlineStr"/>
       <c r="AB108" s="8" t="inlineStr"/>
-      <c r="AC108" s="9" t="inlineStr"/>
+      <c r="AC108" s="9" t="inlineStr">
+        <is>
+          <t>M: soğuk süt, karamel</t>
+        </is>
+      </c>
+      <c r="AD108" s="10" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -8624,7 +9069,12 @@
       <c r="Z109" s="8" t="inlineStr"/>
       <c r="AA109" s="8" t="inlineStr"/>
       <c r="AB109" s="8" t="inlineStr"/>
-      <c r="AC109" s="9" t="inlineStr"/>
+      <c r="AC109" s="9" t="inlineStr">
+        <is>
+          <t>M: soğuk süt, çikolata sosu · S: çikolata sosu</t>
+        </is>
+      </c>
+      <c r="AD109" s="10" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -8697,7 +9147,12 @@
       <c r="Z110" s="8" t="inlineStr"/>
       <c r="AA110" s="8" t="inlineStr"/>
       <c r="AB110" s="8" t="inlineStr"/>
-      <c r="AC110" s="9" t="inlineStr"/>
+      <c r="AC110" s="9" t="inlineStr">
+        <is>
+          <t>M: soğuk süt, beyaz çikolata · S: beyaz çikolata</t>
+        </is>
+      </c>
+      <c r="AD110" s="10" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -8766,7 +9221,12 @@
       <c r="Z111" s="8" t="inlineStr"/>
       <c r="AA111" s="8" t="inlineStr"/>
       <c r="AB111" s="8" t="inlineStr"/>
-      <c r="AC111" s="9" t="inlineStr"/>
+      <c r="AC111" s="9" t="inlineStr">
+        <is>
+          <t>M: soğuk süt</t>
+        </is>
+      </c>
+      <c r="AD111" s="10" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -8835,7 +9295,12 @@
       <c r="Z112" s="8" t="inlineStr"/>
       <c r="AA112" s="8" t="inlineStr"/>
       <c r="AB112" s="8" t="inlineStr"/>
-      <c r="AC112" s="9" t="inlineStr"/>
+      <c r="AC112" s="9" t="inlineStr">
+        <is>
+          <t>M: soğuk süt, tuzlu karamel</t>
+        </is>
+      </c>
+      <c r="AD112" s="10" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -8904,7 +9369,12 @@
       <c r="Z113" s="8" t="inlineStr"/>
       <c r="AA113" s="8" t="inlineStr"/>
       <c r="AB113" s="8" t="inlineStr"/>
-      <c r="AC113" s="9" t="inlineStr"/>
+      <c r="AC113" s="9" t="inlineStr">
+        <is>
+          <t>M: soğuk süt</t>
+        </is>
+      </c>
+      <c r="AD113" s="10" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -8973,7 +9443,12 @@
       <c r="Z114" s="8" t="inlineStr"/>
       <c r="AA114" s="8" t="inlineStr"/>
       <c r="AB114" s="8" t="inlineStr"/>
-      <c r="AC114" s="9" t="inlineStr"/>
+      <c r="AC114" s="9" t="inlineStr">
+        <is>
+          <t>M: soğuk süt</t>
+        </is>
+      </c>
+      <c r="AD114" s="10" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -9039,6 +9514,7 @@
       <c r="AA115" s="8" t="inlineStr"/>
       <c r="AB115" s="8" t="inlineStr"/>
       <c r="AC115" s="9" t="inlineStr"/>
+      <c r="AD115" s="10" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -9104,6 +9580,7 @@
       <c r="AA116" s="8" t="inlineStr"/>
       <c r="AB116" s="8" t="inlineStr"/>
       <c r="AC116" s="9" t="inlineStr"/>
+      <c r="AD116" s="10" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -9169,6 +9646,7 @@
       <c r="AA117" s="8" t="inlineStr"/>
       <c r="AB117" s="8" t="inlineStr"/>
       <c r="AC117" s="9" t="inlineStr"/>
+      <c r="AD117" s="10" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -9234,6 +9712,7 @@
       <c r="AA118" s="8" t="inlineStr"/>
       <c r="AB118" s="8" t="inlineStr"/>
       <c r="AC118" s="9" t="inlineStr"/>
+      <c r="AD118" s="10" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -9299,6 +9778,7 @@
       <c r="AA119" s="8" t="inlineStr"/>
       <c r="AB119" s="8" t="inlineStr"/>
       <c r="AC119" s="9" t="inlineStr"/>
+      <c r="AD119" s="10" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -9364,6 +9844,7 @@
       <c r="AA120" s="8" t="inlineStr"/>
       <c r="AB120" s="8" t="inlineStr"/>
       <c r="AC120" s="9" t="inlineStr"/>
+      <c r="AD120" s="10" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -9429,6 +9910,7 @@
       <c r="AA121" s="8" t="inlineStr"/>
       <c r="AB121" s="8" t="inlineStr"/>
       <c r="AC121" s="9" t="inlineStr"/>
+      <c r="AD121" s="10" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -9494,6 +9976,7 @@
       <c r="AA122" s="8" t="inlineStr"/>
       <c r="AB122" s="8" t="inlineStr"/>
       <c r="AC122" s="9" t="inlineStr"/>
+      <c r="AD122" s="10" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -9559,6 +10042,7 @@
       <c r="AA123" s="8" t="inlineStr"/>
       <c r="AB123" s="8" t="inlineStr"/>
       <c r="AC123" s="9" t="inlineStr"/>
+      <c r="AD123" s="10" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -9624,6 +10108,7 @@
       <c r="AA124" s="8" t="inlineStr"/>
       <c r="AB124" s="8" t="inlineStr"/>
       <c r="AC124" s="9" t="inlineStr"/>
+      <c r="AD124" s="10" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -9689,6 +10174,7 @@
       <c r="AA125" s="8" t="inlineStr"/>
       <c r="AB125" s="8" t="inlineStr"/>
       <c r="AC125" s="9" t="inlineStr"/>
+      <c r="AD125" s="10" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -9754,6 +10240,7 @@
       <c r="AA126" s="8" t="inlineStr"/>
       <c r="AB126" s="8" t="inlineStr"/>
       <c r="AC126" s="9" t="inlineStr"/>
+      <c r="AD126" s="10" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -9819,6 +10306,7 @@
       <c r="AA127" s="8" t="inlineStr"/>
       <c r="AB127" s="8" t="inlineStr"/>
       <c r="AC127" s="9" t="inlineStr"/>
+      <c r="AD127" s="10" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -9884,6 +10372,7 @@
       <c r="AA128" s="8" t="inlineStr"/>
       <c r="AB128" s="8" t="inlineStr"/>
       <c r="AC128" s="9" t="inlineStr"/>
+      <c r="AD128" s="10" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -9949,6 +10438,7 @@
       <c r="AA129" s="8" t="inlineStr"/>
       <c r="AB129" s="8" t="inlineStr"/>
       <c r="AC129" s="9" t="inlineStr"/>
+      <c r="AD129" s="10" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -10014,6 +10504,7 @@
       <c r="AA130" s="8" t="inlineStr"/>
       <c r="AB130" s="8" t="inlineStr"/>
       <c r="AC130" s="9" t="inlineStr"/>
+      <c r="AD130" s="10" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -10079,6 +10570,7 @@
       <c r="AA131" s="8" t="inlineStr"/>
       <c r="AB131" s="8" t="inlineStr"/>
       <c r="AC131" s="9" t="inlineStr"/>
+      <c r="AD131" s="10" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -10144,6 +10636,7 @@
       <c r="AA132" s="8" t="inlineStr"/>
       <c r="AB132" s="8" t="inlineStr"/>
       <c r="AC132" s="9" t="inlineStr"/>
+      <c r="AD132" s="10" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -10212,7 +10705,12 @@
       <c r="Z133" s="8" t="inlineStr"/>
       <c r="AA133" s="8" t="inlineStr"/>
       <c r="AB133" s="8" t="inlineStr"/>
-      <c r="AC133" s="9" t="inlineStr"/>
+      <c r="AC133" s="9" t="inlineStr">
+        <is>
+          <t>M: yoğurt</t>
+        </is>
+      </c>
+      <c r="AD133" s="10" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -10278,6 +10776,7 @@
       <c r="AA134" s="8" t="inlineStr"/>
       <c r="AB134" s="8" t="inlineStr"/>
       <c r="AC134" s="9" t="inlineStr"/>
+      <c r="AD134" s="10" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -10343,6 +10842,7 @@
       <c r="AA135" s="8" t="inlineStr"/>
       <c r="AB135" s="8" t="inlineStr"/>
       <c r="AC135" s="9" t="inlineStr"/>
+      <c r="AD135" s="10" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -10408,6 +10908,7 @@
       <c r="AA136" s="8" t="inlineStr"/>
       <c r="AB136" s="8" t="inlineStr"/>
       <c r="AC136" s="9" t="inlineStr"/>
+      <c r="AD136" s="10" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -10473,6 +10974,7 @@
       <c r="AA137" s="8" t="inlineStr"/>
       <c r="AB137" s="8" t="inlineStr"/>
       <c r="AC137" s="9" t="inlineStr"/>
+      <c r="AD137" s="10" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -10538,6 +11040,7 @@
       <c r="AA138" s="8" t="inlineStr"/>
       <c r="AB138" s="8" t="inlineStr"/>
       <c r="AC138" s="9" t="inlineStr"/>
+      <c r="AD138" s="10" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -10603,6 +11106,7 @@
       <c r="AA139" s="8" t="inlineStr"/>
       <c r="AB139" s="8" t="inlineStr"/>
       <c r="AC139" s="9" t="inlineStr"/>
+      <c r="AD139" s="10" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -10668,6 +11172,7 @@
       <c r="AA140" s="8" t="inlineStr"/>
       <c r="AB140" s="8" t="inlineStr"/>
       <c r="AC140" s="9" t="inlineStr"/>
+      <c r="AD140" s="10" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -10736,7 +11241,12 @@
       <c r="Z141" s="8" t="inlineStr"/>
       <c r="AA141" s="8" t="inlineStr"/>
       <c r="AB141" s="8" t="inlineStr"/>
-      <c r="AC141" s="9" t="inlineStr"/>
+      <c r="AC141" s="9" t="inlineStr">
+        <is>
+          <t>M: süt, dondurma</t>
+        </is>
+      </c>
+      <c r="AD141" s="10" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -10809,7 +11319,12 @@
       <c r="Z142" s="8" t="inlineStr"/>
       <c r="AA142" s="8" t="inlineStr"/>
       <c r="AB142" s="8" t="inlineStr"/>
-      <c r="AC142" s="9" t="inlineStr"/>
+      <c r="AC142" s="9" t="inlineStr">
+        <is>
+          <t>M: süt, dondurma, çikolata sosu · S: çikolata sosu</t>
+        </is>
+      </c>
+      <c r="AD142" s="10" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -10878,7 +11393,12 @@
       <c r="Z143" s="8" t="inlineStr"/>
       <c r="AA143" s="8" t="inlineStr"/>
       <c r="AB143" s="8" t="inlineStr"/>
-      <c r="AC143" s="9" t="inlineStr"/>
+      <c r="AC143" s="9" t="inlineStr">
+        <is>
+          <t>M: süt, dondurma</t>
+        </is>
+      </c>
+      <c r="AD143" s="10" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -10955,7 +11475,12 @@
       <c r="Z144" s="8" t="inlineStr"/>
       <c r="AA144" s="8" t="inlineStr"/>
       <c r="AB144" s="8" t="inlineStr"/>
-      <c r="AC144" s="9" t="inlineStr"/>
+      <c r="AC144" s="9" t="inlineStr">
+        <is>
+          <t>M: süt, dondurma · G: oreo bisküvi · S: oreo bisküvi</t>
+        </is>
+      </c>
+      <c r="AD144" s="10" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -11024,7 +11549,12 @@
       <c r="Z145" s="8" t="inlineStr"/>
       <c r="AA145" s="8" t="inlineStr"/>
       <c r="AB145" s="8" t="inlineStr"/>
-      <c r="AC145" s="9" t="inlineStr"/>
+      <c r="AC145" s="9" t="inlineStr">
+        <is>
+          <t>M: süt, dondurma</t>
+        </is>
+      </c>
+      <c r="AD145" s="10" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -11090,6 +11620,7 @@
       <c r="AA146" s="8" t="inlineStr"/>
       <c r="AB146" s="8" t="inlineStr"/>
       <c r="AC146" s="9" t="inlineStr"/>
+      <c r="AD146" s="10" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -11155,6 +11686,7 @@
       <c r="AA147" s="8" t="inlineStr"/>
       <c r="AB147" s="8" t="inlineStr"/>
       <c r="AC147" s="9" t="inlineStr"/>
+      <c r="AD147" s="10" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -11220,6 +11752,7 @@
       <c r="AA148" s="8" t="inlineStr"/>
       <c r="AB148" s="8" t="inlineStr"/>
       <c r="AC148" s="9" t="inlineStr"/>
+      <c r="AD148" s="10" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -11285,6 +11818,7 @@
       <c r="AA149" s="8" t="inlineStr"/>
       <c r="AB149" s="8" t="inlineStr"/>
       <c r="AC149" s="9" t="inlineStr"/>
+      <c r="AD149" s="10" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -11350,6 +11884,7 @@
       <c r="AA150" s="8" t="inlineStr"/>
       <c r="AB150" s="8" t="inlineStr"/>
       <c r="AC150" s="9" t="inlineStr"/>
+      <c r="AD150" s="10" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -11415,6 +11950,7 @@
       <c r="AA151" s="8" t="inlineStr"/>
       <c r="AB151" s="8" t="inlineStr"/>
       <c r="AC151" s="9" t="inlineStr"/>
+      <c r="AD151" s="10" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -11480,6 +12016,7 @@
       <c r="AA152" s="8" t="inlineStr"/>
       <c r="AB152" s="8" t="inlineStr"/>
       <c r="AC152" s="9" t="inlineStr"/>
+      <c r="AD152" s="10" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -11545,6 +12082,7 @@
       <c r="AA153" s="8" t="inlineStr"/>
       <c r="AB153" s="8" t="inlineStr"/>
       <c r="AC153" s="9" t="inlineStr"/>
+      <c r="AD153" s="10" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -11610,6 +12148,7 @@
       <c r="AA154" s="8" t="inlineStr"/>
       <c r="AB154" s="8" t="inlineStr"/>
       <c r="AC154" s="9" t="inlineStr"/>
+      <c r="AD154" s="10" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -11675,6 +12214,7 @@
       <c r="AA155" s="8" t="inlineStr"/>
       <c r="AB155" s="8" t="inlineStr"/>
       <c r="AC155" s="9" t="inlineStr"/>
+      <c r="AD155" s="10" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -11740,6 +12280,7 @@
       <c r="AA156" s="8" t="inlineStr"/>
       <c r="AB156" s="8" t="inlineStr"/>
       <c r="AC156" s="9" t="inlineStr"/>
+      <c r="AD156" s="10" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -11805,6 +12346,7 @@
       <c r="AA157" s="8" t="inlineStr"/>
       <c r="AB157" s="8" t="inlineStr"/>
       <c r="AC157" s="9" t="inlineStr"/>
+      <c r="AD157" s="10" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -11870,6 +12412,7 @@
       <c r="AA158" s="8" t="inlineStr"/>
       <c r="AB158" s="8" t="inlineStr"/>
       <c r="AC158" s="9" t="inlineStr"/>
+      <c r="AD158" s="10" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -11935,6 +12478,7 @@
       <c r="AA159" s="8" t="inlineStr"/>
       <c r="AB159" s="8" t="inlineStr"/>
       <c r="AC159" s="9" t="inlineStr"/>
+      <c r="AD159" s="10" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -11991,7 +12535,12 @@
       <c r="Z160" s="8" t="inlineStr"/>
       <c r="AA160" s="8" t="inlineStr"/>
       <c r="AB160" s="8" t="inlineStr"/>
-      <c r="AC160" s="9" t="inlineStr"/>
+      <c r="AC160" s="9" t="inlineStr">
+        <is>
+          <t>içerik günlük değişir</t>
+        </is>
+      </c>
+      <c r="AD160" s="10" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -12048,7 +12597,12 @@
       <c r="Z161" s="8" t="inlineStr"/>
       <c r="AA161" s="8" t="inlineStr"/>
       <c r="AB161" s="8" t="inlineStr"/>
-      <c r="AC161" s="9" t="inlineStr"/>
+      <c r="AC161" s="9" t="inlineStr">
+        <is>
+          <t>içerik günlük değişir</t>
+        </is>
+      </c>
+      <c r="AD161" s="10" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -12105,7 +12659,12 @@
       <c r="Z162" s="8" t="inlineStr"/>
       <c r="AA162" s="8" t="inlineStr"/>
       <c r="AB162" s="8" t="inlineStr"/>
-      <c r="AC162" s="9" t="inlineStr"/>
+      <c r="AC162" s="9" t="inlineStr">
+        <is>
+          <t>içerik günlük değişir</t>
+        </is>
+      </c>
+      <c r="AD162" s="10" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -12162,7 +12721,12 @@
       <c r="Z163" s="8" t="inlineStr"/>
       <c r="AA163" s="8" t="inlineStr"/>
       <c r="AB163" s="8" t="inlineStr"/>
-      <c r="AC163" s="9" t="inlineStr"/>
+      <c r="AC163" s="9" t="inlineStr">
+        <is>
+          <t>içerik günlük değişir</t>
+        </is>
+      </c>
+      <c r="AD163" s="10" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -12219,7 +12783,12 @@
       <c r="Z164" s="8" t="inlineStr"/>
       <c r="AA164" s="8" t="inlineStr"/>
       <c r="AB164" s="8" t="inlineStr"/>
-      <c r="AC164" s="9" t="inlineStr"/>
+      <c r="AC164" s="9" t="inlineStr">
+        <is>
+          <t>içerik günlük değişir</t>
+        </is>
+      </c>
+      <c r="AD164" s="10" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -12276,7 +12845,12 @@
       <c r="Z165" s="8" t="inlineStr"/>
       <c r="AA165" s="8" t="inlineStr"/>
       <c r="AB165" s="8" t="inlineStr"/>
-      <c r="AC165" s="9" t="inlineStr"/>
+      <c r="AC165" s="9" t="inlineStr">
+        <is>
+          <t>içerik günlük değişir</t>
+        </is>
+      </c>
+      <c r="AD165" s="10" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
@@ -12333,7 +12907,12 @@
       <c r="Z166" s="8" t="inlineStr"/>
       <c r="AA166" s="8" t="inlineStr"/>
       <c r="AB166" s="8" t="inlineStr"/>
-      <c r="AC166" s="9" t="inlineStr"/>
+      <c r="AC166" s="9" t="inlineStr">
+        <is>
+          <t>içerik günlük değişir</t>
+        </is>
+      </c>
+      <c r="AD166" s="10" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" s="2" t="inlineStr">
@@ -12390,7 +12969,12 @@
       <c r="Z167" s="8" t="inlineStr"/>
       <c r="AA167" s="8" t="inlineStr"/>
       <c r="AB167" s="8" t="inlineStr"/>
-      <c r="AC167" s="9" t="inlineStr"/>
+      <c r="AC167" s="9" t="inlineStr">
+        <is>
+          <t>içerik günlük değişir</t>
+        </is>
+      </c>
+      <c r="AD167" s="10" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
@@ -12447,7 +13031,12 @@
       <c r="Z168" s="8" t="inlineStr"/>
       <c r="AA168" s="8" t="inlineStr"/>
       <c r="AB168" s="8" t="inlineStr"/>
-      <c r="AC168" s="9" t="inlineStr"/>
+      <c r="AC168" s="9" t="inlineStr">
+        <is>
+          <t>içerik günlük değişir</t>
+        </is>
+      </c>
+      <c r="AD168" s="10" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
@@ -12504,7 +13093,12 @@
       <c r="Z169" s="8" t="inlineStr"/>
       <c r="AA169" s="8" t="inlineStr"/>
       <c r="AB169" s="8" t="inlineStr"/>
-      <c r="AC169" s="9" t="inlineStr"/>
+      <c r="AC169" s="9" t="inlineStr">
+        <is>
+          <t>içerik günlük değişir</t>
+        </is>
+      </c>
+      <c r="AD169" s="10" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" s="2" t="inlineStr">
@@ -12561,7 +13155,12 @@
       <c r="Z170" s="8" t="inlineStr"/>
       <c r="AA170" s="8" t="inlineStr"/>
       <c r="AB170" s="8" t="inlineStr"/>
-      <c r="AC170" s="9" t="inlineStr"/>
+      <c r="AC170" s="9" t="inlineStr">
+        <is>
+          <t>içerik günlük değişir</t>
+        </is>
+      </c>
+      <c r="AD170" s="10" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
@@ -12618,7 +13217,12 @@
       <c r="Z171" s="8" t="inlineStr"/>
       <c r="AA171" s="8" t="inlineStr"/>
       <c r="AB171" s="8" t="inlineStr"/>
-      <c r="AC171" s="9" t="inlineStr"/>
+      <c r="AC171" s="9" t="inlineStr">
+        <is>
+          <t>içerik günlük değişir</t>
+        </is>
+      </c>
+      <c r="AD171" s="10" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" s="2" t="inlineStr">
@@ -12675,7 +13279,12 @@
       <c r="Z172" s="8" t="inlineStr"/>
       <c r="AA172" s="8" t="inlineStr"/>
       <c r="AB172" s="8" t="inlineStr"/>
-      <c r="AC172" s="9" t="inlineStr"/>
+      <c r="AC172" s="9" t="inlineStr">
+        <is>
+          <t>içerik günlük değişir</t>
+        </is>
+      </c>
+      <c r="AD172" s="10" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" s="2" t="inlineStr">
@@ -12732,7 +13341,12 @@
       <c r="Z173" s="8" t="inlineStr"/>
       <c r="AA173" s="8" t="inlineStr"/>
       <c r="AB173" s="8" t="inlineStr"/>
-      <c r="AC173" s="9" t="inlineStr"/>
+      <c r="AC173" s="9" t="inlineStr">
+        <is>
+          <t>içerik günlük değişir</t>
+        </is>
+      </c>
+      <c r="AD173" s="10" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" s="2" t="inlineStr">
@@ -12789,10 +13403,15 @@
       <c r="Z174" s="8" t="inlineStr"/>
       <c r="AA174" s="8" t="inlineStr"/>
       <c r="AB174" s="8" t="inlineStr"/>
-      <c r="AC174" s="9" t="inlineStr"/>
+      <c r="AC174" s="9" t="inlineStr">
+        <is>
+          <t>içerik günlük değişir</t>
+        </is>
+      </c>
+      <c r="AD174" s="10" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AC174"/>
+  <autoFilter ref="A1:AD174"/>
   <dataValidations count="1">
     <dataValidation sqref="H2:U174 Z2:AA174" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"X,"</formula1>
@@ -12815,252 +13434,510 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="10" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>KULE CAFE — Alerjen, içerik ve enerji kontrol listesi</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="11" t="inlineStr"/>
+      <c r="A2" s="12" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="11" t="inlineStr">
+      <c r="A3" s="12" t="inlineStr">
         <is>
           <t>İçindekiler: mutfağın 16.09.2026 tarihli düzeltmeleri işlenmiştir.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="11" t="inlineStr">
+      <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Alerjen işaretleri ve BESİN DEĞERLERİ (kcal, protein, yağ, karbonhidrat) TASLAKTIR: standart tarif ve porsiyon</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="11" t="inlineStr">
+      <c r="A5" s="12" t="inlineStr">
         <is>
           <t>büyüklüklerinden hesaplanmış yaklaşık değerlerdir. Mevzuata uygun beyan için mutfak</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="11" t="inlineStr">
+      <c r="A6" s="12" t="inlineStr">
         <is>
           <t>gramajlarıyla bir gıda mühendisi / diyetisyen tarafından doğrulanmalıdır.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="inlineStr">
+      <c r="A7" s="12" t="inlineStr">
         <is>
           <t>Alkol ve Domuz türevi sütunları: ürün içeriyorsa X yazın (şu an hepsi boş = içermez).</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="11" t="inlineStr">
+      <c r="A8" s="12" t="inlineStr">
         <is>
           <t>Sos kartı sütunu: o üründe hangi hazır sosun ayrı kartı gösteriliyor (sweetchili / cafedeparis / demiglace).</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="11" t="inlineStr"/>
+      <c r="A9" s="12" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="10" t="inlineStr">
+      <c r="A10" s="11" t="inlineStr">
         <is>
           <t>Nasıl düzeltirsiniz:</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="11" t="inlineStr">
+      <c r="A11" s="12" t="inlineStr">
         <is>
           <t>1. "Menü" sekmesinde her satır bir üründür.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="11" t="inlineStr">
+      <c r="A12" s="12" t="inlineStr">
         <is>
           <t>2. Alerjen sütunlarında (G, M, Y, ...) ürün o alerjeni içeriyorsa hücreye X yazın,</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="11" t="inlineStr">
+      <c r="A13" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">   içermiyorsa hücreyi boş bırakın. Sarı hücreler doldurulacak alanlardır.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="11" t="inlineStr">
+      <c r="A14" s="12" t="inlineStr">
         <is>
           <t>3. İçindekiler sütunlarını serbestçe düzeltebilir, boş olanları doldurabilirsiniz.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="11" t="inlineStr">
+      <c r="A15" s="12" t="inlineStr">
         <is>
           <t>4. Enerji / protein / yağ / karbonhidrat sütunlarına porsiyon başına değerleri yazın; Alkol / Domuz türevi sütunlarına içeriyorsa X.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="11" t="inlineStr">
+      <c r="A16" s="12" t="inlineStr">
         <is>
           <t>5. Fiyat değişikliklerini de bu dosyada yapabilirsiniz.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="11" t="inlineStr">
+      <c r="A17" s="12" t="inlineStr">
         <is>
           <t>6. Dosyayı bana geri gönderin; menüyü güncellerim. QR kod değişmez.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="11" t="inlineStr"/>
+      <c r="A18" s="12" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="10" t="inlineStr">
+      <c r="A19" s="11" t="inlineStr">
         <is>
           <t>Örnek satır:</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="11" t="inlineStr">
+      <c r="A20" s="12" t="inlineStr">
         <is>
           <t>Bölüm: Tatlılar | Grup: Tatlılar | Ürün: Künefe | Fiyat: 420</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="11" t="inlineStr">
+      <c r="A21" s="12" t="inlineStr">
         <is>
           <t>İçindekiler: Kadayıf, dil peyniri, tereyağı, şerbet, Antep fıstığı</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="11" t="inlineStr">
+      <c r="A22" s="12" t="inlineStr">
         <is>
           <t>G: X   M: X   N: X   (gluten, süt ve sert kabuklu yemiş içerir)</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="11" t="inlineStr"/>
+      <c r="A23" s="12" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="10" t="inlineStr">
+      <c r="A24" s="11" t="inlineStr">
         <is>
           <t>Alerjen kodları:</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="11" t="inlineStr">
+      <c r="A25" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">   G  =  Gluten</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="11" t="inlineStr">
+      <c r="A26" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">   M  =  Süt</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="11" t="inlineStr">
+      <c r="A27" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">   Y  =  Yumurta</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="11" t="inlineStr">
+      <c r="A28" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">   B  =  Balık</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="11" t="inlineStr">
+      <c r="A29" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">   K  =  Kabuklu deniz ürünleri</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="11" t="inlineStr">
+      <c r="A30" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">   S  =  Soya</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="11" t="inlineStr">
+      <c r="A31" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">   SS  =  Susam</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="11" t="inlineStr">
+      <c r="A32" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">   N  =  Sert kabuklu yemişler</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="11" t="inlineStr">
+      <c r="A33" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">   F  =  Yer fıstığı</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="11" t="inlineStr">
+      <c r="A34" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">   H  =  Hardal</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="11" t="inlineStr">
+      <c r="A35" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">   C  =  Kereviz</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="11" t="inlineStr">
+      <c r="A36" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">   SO  =  Sülfit</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="11" t="inlineStr">
+      <c r="A37" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">   MO  =  Yumuşakçalar</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="11" t="inlineStr">
+      <c r="A38" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">   L  =  Acı bakla</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="95" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="13" t="inlineStr">
+        <is>
+          <t>MUTFAK / TEDARİKÇİ TEYİDİ GEREKEN ALERJEN MADDELERİ</t>
+        </is>
+      </c>
+      <c r="B1" s="14" t="inlineStr"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="15" t="inlineStr"/>
+      <c r="B2" s="16" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="15" t="inlineStr">
+        <is>
+          <t>Alerjenler ürünlerin içindekiler listesinden kural tabanlı çıkarılmıştır. Aşağıdaki maddeler</t>
+        </is>
+      </c>
+      <c r="B3" s="16" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="15" t="inlineStr">
+        <is>
+          <t>sektör normuna göre işaretlendi; ürün etiketinden doğrulanmalı. Farklıysa bana bildirin.</t>
+        </is>
+      </c>
+      <c r="B4" s="16" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="15" t="inlineStr"/>
+      <c r="B5" s="16" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="13" t="inlineStr">
+        <is>
+          <t>MALZEME / ÜRÜN</t>
+        </is>
+      </c>
+      <c r="B6" s="14" t="inlineStr">
+        <is>
+          <t>DURUM — NE TEYİT EDİLMELİ</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="15" t="inlineStr">
+        <is>
+          <t>Soya sosu</t>
+        </is>
+      </c>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>GLUTEN olarak işaretlendi (soya sosları genelde buğday içerir). Glutensiz tamari kullanılıyorsa kaldırılır.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="15" t="inlineStr">
+        <is>
+          <t>Sosis</t>
+        </is>
+      </c>
+      <c r="B8" s="16" t="inlineStr">
+        <is>
+          <t>GLUTEN olarak işaretlendi (nişasta/galeta unu). Etiketi kontrol edin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="15" t="inlineStr">
+        <is>
+          <t>Köri sos</t>
+        </is>
+      </c>
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>HARDAL olarak işaretlendi (köri karışımları çoğunlukla hardal içerir). Etiketi kontrol edin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="15" t="inlineStr">
+        <is>
+          <t>Köfte (tüm köfteler)</t>
+        </is>
+      </c>
+      <c r="B10" s="16" t="inlineStr">
+        <is>
+          <t>GLUTEN işaretli (galeta unu/ekmek içi). Harcında YUMURTA da varsa yumurta eklenmeli.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="15" t="inlineStr">
+        <is>
+          <t>Sweet Chili Kule Topları</t>
+        </is>
+      </c>
+      <c r="B11" s="16" t="inlineStr">
+        <is>
+          <t>GLUTEN + YUMURTA işaretli (çıtır kaplama varsayıldı). Kaplamasız ise kaldırılacak.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="15" t="inlineStr">
+        <is>
+          <t>Soğan halkası</t>
+        </is>
+      </c>
+      <c r="B12" s="16" t="inlineStr">
+        <is>
+          <t>Sadece GLUTEN işaretli. Kaplamasında yumurta varsa YUMURTA eklenmeli.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>Fettuccine / noodle</t>
+        </is>
+      </c>
+      <c r="B13" s="16" t="inlineStr">
+        <is>
+          <t>Sadece GLUTEN işaretli. Yumurtalı makarna/noodle kullanılıyorsa YUMURTA eklenmeli.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="15" t="inlineStr">
+        <is>
+          <t>Cheesecake'ler, Cedric tatlıları</t>
+        </is>
+      </c>
+      <c r="B14" s="16" t="inlineStr">
+        <is>
+          <t>Yumurta işaretlenmedi (içindekilerde yok). Fırınlanan/yumurtalı tarif varsa YUMURTA eklenmeli.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="15" t="inlineStr">
+        <is>
+          <t>Barbekü sos</t>
+        </is>
+      </c>
+      <c r="B15" s="16" t="inlineStr">
+        <is>
+          <t>Alerjen işaretlenmedi. Hazır BBQ sosları HARDAL / KEREVİZ / SOYA içerebilir — etiketi kontrol edin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="15" t="inlineStr">
+        <is>
+          <t>Cajun baharatı</t>
+        </is>
+      </c>
+      <c r="B16" s="16" t="inlineStr">
+        <is>
+          <t>Alerjen işaretlenmedi. Baharat karışımları HARDAL / KEREVİZ içerebilir — etiketi kontrol edin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="15" t="inlineStr">
+        <is>
+          <t>Acı sos</t>
+        </is>
+      </c>
+      <c r="B17" s="16" t="inlineStr">
+        <is>
+          <t>Alerjen işaretlenmedi. Etiketi kontrol edin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="15" t="inlineStr">
+        <is>
+          <t>Turşu</t>
+        </is>
+      </c>
+      <c r="B18" s="16" t="inlineStr">
+        <is>
+          <t>SÜLFİT işaretlenmedi. Hazır turşu kullanılıyorsa etiketinde sülfit olabilir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="15" t="inlineStr">
+        <is>
+          <t>Jambon (serpme kahvaltı)</t>
+        </is>
+      </c>
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>DOMUZ TÜREVİ beyanı 'içermez' olarak duruyor. Hindi/dana jambon ise doğru; domuz jambonu ise beyan değişmeli.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="15" t="inlineStr">
+        <is>
+          <t>Demi Glace et sosu</t>
+        </is>
+      </c>
+      <c r="B20" s="16" t="inlineStr">
+        <is>
+          <t>Sos kartı hazır (GLUTEN, SÜT, KEREVİZ) ama hiçbir ürüne bağlı değil. Hangi yemeklerde kullanılıyor?</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="15" t="inlineStr">
+        <is>
+          <t>Susamlı burger ekmeği / lavaş</t>
+        </is>
+      </c>
+      <c r="B21" s="16" t="inlineStr">
+        <is>
+          <t>İçindekiler listesine eklendi (gluten + susam kaynağı). Farklı ekmek kullanılıyorsa bildirin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="15" t="inlineStr"/>
+      <c r="B22" s="16" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="13" t="inlineStr">
+        <is>
+          <t>BESİN DEĞERLERİ</t>
+        </is>
+      </c>
+      <c r="B23" s="14" t="inlineStr">
+        <is>
+          <t>Tüm kcal / protein / yağ / karbonhidrat değerleri TAHMİNDİR — diyetisyen doğrulaması gerekir.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Menü güncelleme 18.09.2026 15:32
</commit_message>
<xml_diff>
--- a/KULE-alerjen-kontrol.xlsx
+++ b/KULE-alerjen-kontrol.xlsx
@@ -1982,12 +1982,12 @@
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>2 adet çıtır tavuk (yumurta, un, süt, Cajun baharatı, tuz, karabiber, soya sosu), 2 adet sigara böreği, 2 adet soğan halkası, 2 adet mozzarella stick, 2 adet sosis, elma dilim patates eşliğinde</t>
+          <t>2 adet çıtır tavuk (yumurta, un, süt, Cajun baharatı, tuz, karabiber, soya sosu), 2 adet sigara böreği, 2 adet soğan halkası, 2 adet mozzarella stick, 2 adet sosis. Yanında: elma dilim patates, Sweet Chili sos, hamburger sosu (mayonez, Sweet Chili sos, az acı, tuz, pul biber)</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>2 crispy chicken pieces (egg, flour, milk, Cajun spice, salt, black pepper, soy sauce), 2 cheese rolls, 2 onion rings, 2 mozzarella sticks, 2 sausages, served with wedge potatoes</t>
+          <t>2 crispy chicken pieces (egg, flour, milk, Cajun spice, salt, black pepper, soy sauce), 2 cheese rolls, 2 onion rings, 2 mozzarella sticks, 2 sausages. Served with: wedge potatoes, sweet chilli sauce, burger sauce (mayonnaise, sweet chilli sauce, mild chilli, salt, chilli flakes)</t>
         </is>
       </c>
       <c r="H18" s="5" t="inlineStr">
@@ -2021,23 +2021,27 @@
       <c r="T18" s="5" t="inlineStr"/>
       <c r="U18" s="5" t="inlineStr"/>
       <c r="V18" s="6" t="n">
-        <v>1180</v>
+        <v>1310</v>
       </c>
       <c r="W18" s="7" t="n">
         <v>50</v>
       </c>
       <c r="X18" s="7" t="n">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="Y18" s="7" t="n">
-        <v>92</v>
+        <v>100</v>
       </c>
       <c r="Z18" s="8" t="inlineStr"/>
       <c r="AA18" s="8" t="inlineStr"/>
-      <c r="AB18" s="8" t="inlineStr"/>
+      <c r="AB18" s="8" t="inlineStr">
+        <is>
+          <t>sweetchili</t>
+        </is>
+      </c>
       <c r="AC18" s="9" t="inlineStr">
         <is>
-          <t>G: çıtır tavuk, un, soya sosu, sigara böreği, soğan halkası, mozzarella stick, sosis · Y: çıtır tavuk, yumurta · M: çıtır tavuk, süt, sigara böreği, mozzarella stick · S: soya sosu</t>
+          <t>G: çıtır tavuk, un, soya sosu, sigara böreği, soğan halkası, mozzarella stick, sosis · Y: çıtır tavuk, yumurta, mayonez · M: çıtır tavuk, süt, sigara böreği, mozzarella stick · S: soya sosu</t>
         </is>
       </c>
       <c r="AD18" s="10" t="inlineStr"/>
@@ -2558,12 +2562,12 @@
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>120 g şişte köfte, taze yeşillikler, domates, soğan, zeytinyağı</t>
+          <t>120 g şişte köfte (sarımsak, galeta unu, karabiber, kimyon, pul biber), taze yeşillikler, domates, soğan, zeytinyağı</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
         <is>
-          <t>120 g skewered meatballs, fresh greens, tomato, onion, olive oil</t>
+          <t>120 g skewered meatballs (garlic, breadcrumbs, black pepper, cumin, chilli flakes), fresh greens, tomato, onion, olive oil</t>
         </is>
       </c>
       <c r="H26" s="5" t="inlineStr">
@@ -2601,7 +2605,7 @@
       <c r="AB26" s="8" t="inlineStr"/>
       <c r="AC26" s="9" t="inlineStr">
         <is>
-          <t>G: şişte köfte</t>
+          <t>G: şişte köfte, galeta unu</t>
         </is>
       </c>
       <c r="AD26" s="10" t="inlineStr"/>
@@ -2722,12 +2726,12 @@
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>160 g Cajun tavuk (yumurta, süt, un, pane, galeta unu, soya sosu, Cajun baharatı, tuz), taze yeşillikler, ballı hardal sos</t>
+          <t>160 g Cajun tavuk (yumurta, süt, un, pane, galeta unu, soya sosu, Cajun baharatı, tuz), taze yeşillikler, ballı hardal sos (bal, hardal)</t>
         </is>
       </c>
       <c r="G28" s="4" t="inlineStr">
         <is>
-          <t>160 g Cajun chicken (egg, milk, flour, breading, breadcrumbs, soy sauce, Cajun spice, salt), fresh greens, honey mustard dressing</t>
+          <t>160 g Cajun chicken (egg, milk, flour, breading, breadcrumbs, soy sauce, Cajun spice, salt), fresh greens, honey mustard dressing (honey, mustard)</t>
         </is>
       </c>
       <c r="H28" s="5" t="inlineStr">
@@ -2781,7 +2785,7 @@
       <c r="AB28" s="8" t="inlineStr"/>
       <c r="AC28" s="9" t="inlineStr">
         <is>
-          <t>G: cajun tavuk, un, pane, galeta unu, soya sosu · Y: cajun tavuk, yumurta · M: cajun tavuk, süt · S: cajun tavuk, soya sosu · H: ballı hardal sos</t>
+          <t>G: cajun tavuk, un, pane, galeta unu, soya sosu · Y: cajun tavuk, yumurta · M: cajun tavuk, süt · S: cajun tavuk, soya sosu · H: hardal</t>
         </is>
       </c>
       <c r="AD28" s="10" t="inlineStr"/>
@@ -3355,7 +3359,7 @@
       </c>
       <c r="AC35" s="9" t="inlineStr">
         <is>
-          <t>G: burger köftesi, susamlı burger ekmeği · SS: susamlı burger ekmeği · M: mantar sos, krema · Y: hamburger sosu, mayonez</t>
+          <t>G: burger köftesi, susamlı burger ekmeği · SS: susamlı burger ekmeği · M: krema · Y: mayonez</t>
         </is>
       </c>
       <c r="AD35" s="10" t="inlineStr"/>
@@ -3445,7 +3449,7 @@
       </c>
       <c r="AC36" s="9" t="inlineStr">
         <is>
-          <t>G: burger köftesi, susamlı burger ekmeği · SS: susamlı burger ekmeği · M: cheddar peyniri · Y: hamburger sosu, mayonez</t>
+          <t>G: burger köftesi, susamlı burger ekmeği · SS: susamlı burger ekmeği · M: cheddar peyniri · Y: mayonez</t>
         </is>
       </c>
       <c r="AD36" s="10" t="inlineStr"/>
@@ -3535,7 +3539,7 @@
       </c>
       <c r="AC37" s="9" t="inlineStr">
         <is>
-          <t>G: burger köftesi, susamlı burger ekmeği · SS: susamlı burger ekmeği · M: cheddar peyniri · Y: hamburger sosu, mayonez</t>
+          <t>G: burger köftesi, susamlı burger ekmeği · SS: susamlı burger ekmeği · M: cheddar peyniri · Y: mayonez</t>
         </is>
       </c>
       <c r="AD37" s="10" t="inlineStr"/>
@@ -3629,7 +3633,7 @@
       </c>
       <c r="AC38" s="9" t="inlineStr">
         <is>
-          <t>G: özel soslu tavuk, un, panko, galeta unu, pane, soya sosu, susamlı burger ekmeği · Y: özel soslu tavuk, yumurta, hamburger sosu, mayonez · M: özel soslu tavuk, süt, cheddar peyniri · S: özel soslu tavuk, soya sosu · SS: susamlı burger ekmeği</t>
+          <t>G: özel soslu tavuk, un, panko, galeta unu, pane, soya sosu, susamlı burger ekmeği · Y: özel soslu tavuk, yumurta, mayonez · M: özel soslu tavuk, süt, cheddar peyniri · S: özel soslu tavuk, soya sosu · SS: susamlı burger ekmeği</t>
         </is>
       </c>
       <c r="AD38" s="10" t="inlineStr"/>
@@ -3832,12 +3836,12 @@
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>170 g köfte, lavaş, soğan, renkli biberler, kaşar peyniri, özel sos (soya sosu, Cajun baharatı), patates ve Sweet Chili sos eşliğinde</t>
+          <t>170 g köfte (sarımsak, galeta unu, karabiber, kimyon, pul biber), lavaş, soğan, renkli biberler, kaşar peyniri, özel sos (soya sosu, Cajun baharatı), patates ve Sweet Chili sos eşliğinde</t>
         </is>
       </c>
       <c r="G41" s="4" t="inlineStr">
         <is>
-          <t>170 g meatballs, lavash, onion, bell peppers, kashar cheese, special sauce (soy sauce, Cajun spice), served with fries and sweet chilli sauce</t>
+          <t>170 g meatballs (garlic, breadcrumbs, black pepper, cumin, chilli flakes), lavash, onion, bell peppers, kashar cheese, special sauce (soy sauce, Cajun spice), served with fries and sweet chilli sauce</t>
         </is>
       </c>
       <c r="H41" s="5" t="inlineStr">
@@ -3887,7 +3891,7 @@
       </c>
       <c r="AC41" s="9" t="inlineStr">
         <is>
-          <t>G: köfte, lavaş, soya sosu · M: kaşar peyniri · S: soya sosu</t>
+          <t>G: köfte, galeta unu, lavaş, soya sosu · M: kaşar peyniri · S: soya sosu</t>
         </is>
       </c>
       <c r="AD41" s="10" t="inlineStr"/>
@@ -3918,12 +3922,12 @@
       </c>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t>180 g anne köfte, lavaş, közlenmiş biber &amp; domates, pilav ve patates eşliğinde</t>
+          <t>180 g anne köfte (sarımsak, galeta unu, karabiber, kimyon, pul biber), lavaş, közlenmiş biber &amp; domates, pilav ve patates eşliğinde</t>
         </is>
       </c>
       <c r="G42" s="4" t="inlineStr">
         <is>
-          <t>180 g homestyle meatballs, lavash, served with roasted pepper &amp; tomato, rice and fries</t>
+          <t>180 g homestyle meatballs (garlic, breadcrumbs, black pepper, cumin, chilli flakes), lavash, served with roasted pepper &amp; tomato, rice and fries</t>
         </is>
       </c>
       <c r="H42" s="5" t="inlineStr">
@@ -3961,7 +3965,7 @@
       <c r="AB42" s="8" t="inlineStr"/>
       <c r="AC42" s="9" t="inlineStr">
         <is>
-          <t>G: anne köfte, lavaş</t>
+          <t>G: anne köfte, galeta unu, lavaş</t>
         </is>
       </c>
       <c r="AD42" s="10" t="inlineStr"/>
@@ -3992,12 +3996,12 @@
       </c>
       <c r="F43" s="4" t="inlineStr">
         <is>
-          <t>180 g köfte, domates sos (domates, salça, tuz, karabiber), süzme yoğurt, közlenmiş biber &amp; domates, patates eşliğinde</t>
+          <t>180 g köfte (sarımsak, galeta unu, karabiber, kimyon, pul biber), domates sos (domates, salça, tuz, karabiber), süzme yoğurt, közlenmiş biber &amp; domates, patates eşliğinde</t>
         </is>
       </c>
       <c r="G43" s="4" t="inlineStr">
         <is>
-          <t>180 g meatballs, tomato sauce (tomato, tomato paste, salt, black pepper), strained yoghurt, roasted pepper &amp; tomato, served with fries</t>
+          <t>180 g meatballs (garlic, breadcrumbs, black pepper, cumin, chilli flakes), tomato sauce (tomato, tomato paste, salt, black pepper), strained yoghurt, roasted pepper &amp; tomato, served with fries</t>
         </is>
       </c>
       <c r="H43" s="5" t="inlineStr">
@@ -4039,7 +4043,7 @@
       <c r="AB43" s="8" t="inlineStr"/>
       <c r="AC43" s="9" t="inlineStr">
         <is>
-          <t>G: köfte · M: süzme yoğurt</t>
+          <t>G: köfte, galeta unu · M: süzme yoğurt</t>
         </is>
       </c>
       <c r="AD43" s="10" t="inlineStr"/>
@@ -4070,12 +4074,12 @@
       </c>
       <c r="F44" s="4" t="inlineStr">
         <is>
-          <t>180 g köfte, patlıcan beğendi (süt, kaşar peyniri, tuz, karabiber), közlenmiş biber &amp; domates, patates eşliğinde</t>
+          <t>180 g köfte (sarımsak, galeta unu, karabiber, kimyon, pul biber), patlıcan beğendi (süt, kaşar peyniri, tuz, karabiber), közlenmiş biber &amp; domates, patates eşliğinde</t>
         </is>
       </c>
       <c r="G44" s="4" t="inlineStr">
         <is>
-          <t>180 g meatballs, smoked aubergine purée (milk, kashar cheese, salt, black pepper), roasted pepper &amp; tomato, served with fries</t>
+          <t>180 g meatballs (garlic, breadcrumbs, black pepper, cumin, chilli flakes), smoked aubergine purée (milk, kashar cheese, salt, black pepper), roasted pepper &amp; tomato, served with fries</t>
         </is>
       </c>
       <c r="H44" s="5" t="inlineStr">
@@ -4117,7 +4121,7 @@
       <c r="AB44" s="8" t="inlineStr"/>
       <c r="AC44" s="9" t="inlineStr">
         <is>
-          <t>G: köfte · M: patlıcan beğendi, süt, kaşar peyniri</t>
+          <t>G: köfte, galeta unu · M: patlıcan beğendi, süt, kaşar peyniri</t>
         </is>
       </c>
       <c r="AD44" s="10" t="inlineStr"/>
@@ -4192,10 +4196,14 @@
       </c>
       <c r="Z45" s="8" t="inlineStr"/>
       <c r="AA45" s="8" t="inlineStr"/>
-      <c r="AB45" s="8" t="inlineStr"/>
+      <c r="AB45" s="8" t="inlineStr">
+        <is>
+          <t>bbq</t>
+        </is>
+      </c>
       <c r="AC45" s="9" t="inlineStr">
         <is>
-          <t>M: süzme yoğurt, özel kaymak sos, kaymak, tereyağı · G: çıtır yufka</t>
+          <t>M: süzme yoğurt, kaymak, tereyağı · G: çıtır yufka, barbekü sos</t>
         </is>
       </c>
       <c r="AD45" s="10" t="inlineStr"/>
@@ -4247,11 +4255,7 @@
       <c r="N46" s="5" t="inlineStr"/>
       <c r="O46" s="5" t="inlineStr"/>
       <c r="P46" s="5" t="inlineStr"/>
-      <c r="Q46" s="5" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="Q46" s="5" t="inlineStr"/>
       <c r="R46" s="5" t="inlineStr"/>
       <c r="S46" s="5" t="inlineStr"/>
       <c r="T46" s="5" t="inlineStr"/>
@@ -4270,10 +4274,14 @@
       </c>
       <c r="Z46" s="8" t="inlineStr"/>
       <c r="AA46" s="8" t="inlineStr"/>
-      <c r="AB46" s="8" t="inlineStr"/>
+      <c r="AB46" s="8" t="inlineStr">
+        <is>
+          <t>kori</t>
+        </is>
+      </c>
       <c r="AC46" s="9" t="inlineStr">
         <is>
-          <t>H: köri sos · M: krema</t>
+          <t>M: krema</t>
         </is>
       </c>
       <c r="AD46" s="10" t="inlineStr"/>
@@ -4304,15 +4312,19 @@
       </c>
       <c r="F47" s="4" t="inlineStr">
         <is>
-          <t>180 g tavuk, barbekü sos (barbekü, krema, tuz, karabiber), renkli biberler, mantar, krema, tuz, karabiber, pilav ve patates eşliğinde</t>
+          <t>180 g tavuk, barbekü sos, renkli biberler, mantar, krema, tuz, karabiber, pilav ve patates eşliğinde</t>
         </is>
       </c>
       <c r="G47" s="4" t="inlineStr">
         <is>
-          <t>180 g chicken, BBQ sauce (BBQ, cream, salt, black pepper), bell peppers, mushroom, cream, salt, black pepper, served with rice and fries</t>
-        </is>
-      </c>
-      <c r="H47" s="5" t="inlineStr"/>
+          <t>180 g chicken, BBQ sauce, bell peppers, mushroom, cream, salt, black pepper, served with rice and fries</t>
+        </is>
+      </c>
+      <c r="H47" s="5" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="I47" s="5" t="inlineStr">
         <is>
           <t>X</t>
@@ -4344,10 +4356,14 @@
       </c>
       <c r="Z47" s="8" t="inlineStr"/>
       <c r="AA47" s="8" t="inlineStr"/>
-      <c r="AB47" s="8" t="inlineStr"/>
+      <c r="AB47" s="8" t="inlineStr">
+        <is>
+          <t>bbq</t>
+        </is>
+      </c>
       <c r="AC47" s="9" t="inlineStr">
         <is>
-          <t>M: krema</t>
+          <t>G: barbekü sos · M: krema</t>
         </is>
       </c>
       <c r="AD47" s="10" t="inlineStr"/>
@@ -4679,11 +4695,7 @@
           <t>X</t>
         </is>
       </c>
-      <c r="I52" s="5" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="I52" s="5" t="inlineStr"/>
       <c r="J52" s="5" t="inlineStr">
         <is>
           <t>X</t>
@@ -4721,7 +4733,7 @@
       <c r="AB52" s="8" t="inlineStr"/>
       <c r="AC52" s="9" t="inlineStr">
         <is>
-          <t>G: panelenmiş tavuk, pane, galeta unu, un, soya sosu · Y: panelenmiş tavuk, yumurta · S: soya sosu · M: mantar sos</t>
+          <t>G: panelenmiş tavuk, pane, galeta unu, un, soya sosu · Y: panelenmiş tavuk, yumurta · S: soya sosu</t>
         </is>
       </c>
       <c r="AD52" s="10" t="inlineStr"/>
@@ -4807,7 +4819,7 @@
       <c r="AB53" s="8" t="inlineStr"/>
       <c r="AC53" s="9" t="inlineStr">
         <is>
-          <t>G: panelenmiş tavuk, pane, galeta unu, un, soya sosu · Y: panelenmiş tavuk, yumurta · S: soya sosu · M: cheddar sos, cheddar, krema</t>
+          <t>G: panelenmiş tavuk, pane, galeta unu, un, soya sosu · Y: panelenmiş tavuk, yumurta · S: soya sosu · M: cheddar, krema</t>
         </is>
       </c>
       <c r="AD53" s="10" t="inlineStr"/>
@@ -4838,12 +4850,12 @@
       </c>
       <c r="F54" s="4" t="inlineStr">
         <is>
-          <t>180 g tavuk parçaları, Cafe de Paris sos, krema</t>
+          <t>180 g tavuk parçaları (süt, un, soya sosu, Cajun baharatı, galeta unu, pane, tuz, karabiber), Cafe de Paris sos, krema</t>
         </is>
       </c>
       <c r="G54" s="4" t="inlineStr">
         <is>
-          <t>180 g chicken pieces, Café de Paris sauce, cream</t>
+          <t>180 g chicken pieces (milk, flour, soy sauce, Cajun spice, breadcrumbs, breading, salt, black pepper), Café de Paris sauce, cream</t>
         </is>
       </c>
       <c r="H54" s="5" t="inlineStr">
@@ -4859,7 +4871,11 @@
       <c r="J54" s="5" t="inlineStr"/>
       <c r="K54" s="5" t="inlineStr"/>
       <c r="L54" s="5" t="inlineStr"/>
-      <c r="M54" s="5" t="inlineStr"/>
+      <c r="M54" s="5" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="N54" s="5" t="inlineStr"/>
       <c r="O54" s="5" t="inlineStr"/>
       <c r="P54" s="5" t="inlineStr"/>
@@ -4889,7 +4905,7 @@
       </c>
       <c r="AC54" s="9" t="inlineStr">
         <is>
-          <t>G: cafe de paris sos, Cafe de Paris Sos · M: cafe de paris sos, krema, Cafe de Paris Sos</t>
+          <t>M: süt, cafe de paris sos, krema · G: un, soya sosu, galeta unu, pane, cafe de paris sos · S: soya sosu</t>
         </is>
       </c>
       <c r="AD54" s="10" t="inlineStr"/>
@@ -4920,15 +4936,19 @@
       </c>
       <c r="F55" s="4" t="inlineStr">
         <is>
-          <t>180 g tavuk parçaları, cheddar sos, krema</t>
+          <t>180 g tavuk parçaları (süt, un, soya sosu, Cajun baharatı, galeta unu, pane, tuz, karabiber), cheddar sos (cheddar, krema)</t>
         </is>
       </c>
       <c r="G55" s="4" t="inlineStr">
         <is>
-          <t>180 g chicken pieces, cheddar sauce, cream</t>
-        </is>
-      </c>
-      <c r="H55" s="5" t="inlineStr"/>
+          <t>180 g chicken pieces (milk, flour, soy sauce, Cajun spice, breadcrumbs, breading, salt, black pepper), cheddar sauce (cheddar, cream)</t>
+        </is>
+      </c>
+      <c r="H55" s="5" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="I55" s="5" t="inlineStr">
         <is>
           <t>X</t>
@@ -4937,7 +4957,11 @@
       <c r="J55" s="5" t="inlineStr"/>
       <c r="K55" s="5" t="inlineStr"/>
       <c r="L55" s="5" t="inlineStr"/>
-      <c r="M55" s="5" t="inlineStr"/>
+      <c r="M55" s="5" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="N55" s="5" t="inlineStr"/>
       <c r="O55" s="5" t="inlineStr"/>
       <c r="P55" s="5" t="inlineStr"/>
@@ -4963,7 +4987,7 @@
       <c r="AB55" s="8" t="inlineStr"/>
       <c r="AC55" s="9" t="inlineStr">
         <is>
-          <t>M: cheddar sos, krema</t>
+          <t>M: süt, cheddar, krema · G: un, soya sosu, galeta unu, pane · S: soya sosu</t>
         </is>
       </c>
       <c r="AD55" s="10" t="inlineStr"/>
@@ -4994,12 +5018,12 @@
       </c>
       <c r="F56" s="4" t="inlineStr">
         <is>
-          <t>180 g tavuk parçaları, Sweet Chili sos, maydanoz</t>
+          <t>180 g tavuk parçaları (süt, un, soya sosu, Cajun baharatı, galeta unu, pane, tuz, karabiber), Sweet Chili sos, görsel maydanoz</t>
         </is>
       </c>
       <c r="G56" s="4" t="inlineStr">
         <is>
-          <t>180 g chicken pieces, sweet chilli sauce, parsley</t>
+          <t>180 g chicken pieces (milk, flour, soy sauce, Cajun spice, breadcrumbs, breading, salt, black pepper), sweet chilli sauce, parsley (garnish)</t>
         </is>
       </c>
       <c r="H56" s="5" t="inlineStr">
@@ -5007,15 +5031,19 @@
           <t>X</t>
         </is>
       </c>
-      <c r="I56" s="5" t="inlineStr"/>
-      <c r="J56" s="5" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="I56" s="5" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J56" s="5" t="inlineStr"/>
       <c r="K56" s="5" t="inlineStr"/>
       <c r="L56" s="5" t="inlineStr"/>
-      <c r="M56" s="5" t="inlineStr"/>
+      <c r="M56" s="5" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="N56" s="5" t="inlineStr"/>
       <c r="O56" s="5" t="inlineStr"/>
       <c r="P56" s="5" t="inlineStr"/>
@@ -5045,7 +5073,7 @@
       </c>
       <c r="AC56" s="9" t="inlineStr">
         <is>
-          <t>G: çıtır kaplama · Y: çıtır kaplama</t>
+          <t>M: süt · G: un, soya sosu, galeta unu, pane · S: soya sosu</t>
         </is>
       </c>
       <c r="AD56" s="10" t="inlineStr"/>
@@ -5076,12 +5104,12 @@
       </c>
       <c r="F57" s="4" t="inlineStr">
         <is>
-          <t>1 kuzu pirzola, 200 g antrikot, 2 köfte, 2 tavuk kanat, 1 tavuk bonfile (zeytinyağı, kekik ve pul biber ile marine edilmiş), közlenmiş biber &amp; domates, pilav ve patates eşliğinde</t>
+          <t>1 kuzu pirzola, 200 g antrikot, 2 köfte (sarımsak, galeta unu, karabiber, kimyon, pul biber), 2 tavuk kanat, 1 tavuk bonfile (zeytinyağı, kekik ve pul biber ile marine edilmiş), lavaş, közlenmiş biber &amp; domates, pilav ve elma dilim patates eşliğinde</t>
         </is>
       </c>
       <c r="G57" s="4" t="inlineStr">
         <is>
-          <t>1 lamb chop, 200 g ribeye, 2 meatballs, 2 chicken wings, 1 chicken fillet (marinated in olive oil, thyme and chilli flakes), served with roasted pepper &amp; tomato, rice and fries</t>
+          <t>1 lamb chop, 200 g ribeye, 2 meatballs (garlic, breadcrumbs, black pepper, cumin, chilli flakes), 2 chicken wings, 1 chicken fillet (marinated in olive oil, thyme and chilli flakes), lavash, served with roasted pepper &amp; tomato, rice and wedge potatoes</t>
         </is>
       </c>
       <c r="H57" s="5" t="inlineStr">
@@ -5103,23 +5131,23 @@
       <c r="T57" s="5" t="inlineStr"/>
       <c r="U57" s="5" t="inlineStr"/>
       <c r="V57" s="6" t="n">
-        <v>1900</v>
+        <v>2100</v>
       </c>
       <c r="W57" s="7" t="n">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="X57" s="7" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="Y57" s="7" t="n">
-        <v>90</v>
+        <v>130</v>
       </c>
       <c r="Z57" s="8" t="inlineStr"/>
       <c r="AA57" s="8" t="inlineStr"/>
       <c r="AB57" s="8" t="inlineStr"/>
       <c r="AC57" s="9" t="inlineStr">
         <is>
-          <t>G: köfte</t>
+          <t>G: köfte, galeta unu, lavaş</t>
         </is>
       </c>
       <c r="AD57" s="10" t="inlineStr"/>
@@ -5150,15 +5178,19 @@
       </c>
       <c r="F58" s="4" t="inlineStr">
         <is>
-          <t>3 parça kuzu pirzola (zeytinyağı, kekik ve pul biber ile marine edilmiş), közlenmiş biber &amp; domates, pilav ve patates eşliğinde</t>
+          <t>3 parça kuzu pirzola (zeytinyağı, kekik ve pul biber ile marine edilmiş), lavaş, közlenmiş biber &amp; domates, pilav ve elma dilim patates eşliğinde</t>
         </is>
       </c>
       <c r="G58" s="4" t="inlineStr">
         <is>
-          <t>3 lamb chops (marinated in olive oil, thyme and chilli flakes), served with roasted pepper &amp; tomato, rice and fries</t>
-        </is>
-      </c>
-      <c r="H58" s="5" t="inlineStr"/>
+          <t>3 lamb chops (marinated in olive oil, thyme and chilli flakes), lavash, served with roasted pepper &amp; tomato, rice and wedge potatoes</t>
+        </is>
+      </c>
+      <c r="H58" s="5" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="I58" s="5" t="inlineStr"/>
       <c r="J58" s="5" t="inlineStr"/>
       <c r="K58" s="5" t="inlineStr"/>
@@ -5173,21 +5205,25 @@
       <c r="T58" s="5" t="inlineStr"/>
       <c r="U58" s="5" t="inlineStr"/>
       <c r="V58" s="6" t="n">
-        <v>850</v>
+        <v>1050</v>
       </c>
       <c r="W58" s="7" t="n">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="X58" s="7" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="Y58" s="7" t="n">
-        <v>44</v>
+        <v>84</v>
       </c>
       <c r="Z58" s="8" t="inlineStr"/>
       <c r="AA58" s="8" t="inlineStr"/>
       <c r="AB58" s="8" t="inlineStr"/>
-      <c r="AC58" s="9" t="inlineStr"/>
+      <c r="AC58" s="9" t="inlineStr">
+        <is>
+          <t>G: lavaş</t>
+        </is>
+      </c>
       <c r="AD58" s="10" t="inlineStr"/>
     </row>
     <row r="59">
@@ -5216,15 +5252,19 @@
       </c>
       <c r="F59" s="4" t="inlineStr">
         <is>
-          <t>4 parça kuzu pirzola (zeytinyağı, kekik ve pul biber ile marine edilmiş), közlenmiş biber &amp; domates, pilav ve patates eşliğinde</t>
+          <t>4 parça kuzu pirzola (zeytinyağı, kekik ve pul biber ile marine edilmiş), lavaş, közlenmiş biber &amp; domates, pilav ve elma dilim patates eşliğinde</t>
         </is>
       </c>
       <c r="G59" s="4" t="inlineStr">
         <is>
-          <t>4 lamb chops (marinated in olive oil, thyme and chilli flakes), served with roasted pepper &amp; tomato, rice and fries</t>
-        </is>
-      </c>
-      <c r="H59" s="5" t="inlineStr"/>
+          <t>4 lamb chops (marinated in olive oil, thyme and chilli flakes), lavash, served with roasted pepper &amp; tomato, rice and wedge potatoes</t>
+        </is>
+      </c>
+      <c r="H59" s="5" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="I59" s="5" t="inlineStr"/>
       <c r="J59" s="5" t="inlineStr"/>
       <c r="K59" s="5" t="inlineStr"/>
@@ -5239,21 +5279,25 @@
       <c r="T59" s="5" t="inlineStr"/>
       <c r="U59" s="5" t="inlineStr"/>
       <c r="V59" s="6" t="n">
-        <v>1050</v>
+        <v>1250</v>
       </c>
       <c r="W59" s="7" t="n">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="X59" s="7" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="Y59" s="7" t="n">
-        <v>44</v>
+        <v>84</v>
       </c>
       <c r="Z59" s="8" t="inlineStr"/>
       <c r="AA59" s="8" t="inlineStr"/>
       <c r="AB59" s="8" t="inlineStr"/>
-      <c r="AC59" s="9" t="inlineStr"/>
+      <c r="AC59" s="9" t="inlineStr">
+        <is>
+          <t>G: lavaş</t>
+        </is>
+      </c>
       <c r="AD59" s="10" t="inlineStr"/>
     </row>
     <row r="60">
@@ -5282,15 +5326,19 @@
       </c>
       <c r="F60" s="4" t="inlineStr">
         <is>
-          <t>200 g antrikot (zeytinyağı, kekik ve pul biber ile marine edilmiş), közlenmiş biber &amp; domates, pilav ve patates eşliğinde</t>
+          <t>200 g antrikot (zeytinyağı, kekik ve pul biber ile marine edilmiş), lavaş, közlenmiş biber &amp; domates, pilav ve elma dilim patates eşliğinde</t>
         </is>
       </c>
       <c r="G60" s="4" t="inlineStr">
         <is>
-          <t>200 g ribeye (marinated in olive oil, thyme and chilli flakes), served with roasted pepper &amp; tomato, rice and fries</t>
-        </is>
-      </c>
-      <c r="H60" s="5" t="inlineStr"/>
+          <t>200 g ribeye (marinated in olive oil, thyme and chilli flakes), lavash, served with roasted pepper &amp; tomato, rice and wedge potatoes</t>
+        </is>
+      </c>
+      <c r="H60" s="5" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="I60" s="5" t="inlineStr"/>
       <c r="J60" s="5" t="inlineStr"/>
       <c r="K60" s="5" t="inlineStr"/>
@@ -5305,21 +5353,25 @@
       <c r="T60" s="5" t="inlineStr"/>
       <c r="U60" s="5" t="inlineStr"/>
       <c r="V60" s="6" t="n">
-        <v>950</v>
+        <v>1150</v>
       </c>
       <c r="W60" s="7" t="n">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="X60" s="7" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="Y60" s="7" t="n">
-        <v>44</v>
+        <v>84</v>
       </c>
       <c r="Z60" s="8" t="inlineStr"/>
       <c r="AA60" s="8" t="inlineStr"/>
       <c r="AB60" s="8" t="inlineStr"/>
-      <c r="AC60" s="9" t="inlineStr"/>
+      <c r="AC60" s="9" t="inlineStr">
+        <is>
+          <t>G: lavaş</t>
+        </is>
+      </c>
       <c r="AD60" s="10" t="inlineStr"/>
     </row>
     <row r="61">
@@ -5348,15 +5400,19 @@
       </c>
       <c r="F61" s="4" t="inlineStr">
         <is>
-          <t>200 g bonfile (zeytinyağı, kekik ve pul biber ile marine edilmiş), közlenmiş biber &amp; domates, pilav ve patates eşliğinde</t>
+          <t>200 g bonfile (zeytinyağı, kekik ve pul biber ile marine edilmiş), lavaş, közlenmiş biber &amp; domates, pilav ve elma dilim patates eşliğinde</t>
         </is>
       </c>
       <c r="G61" s="4" t="inlineStr">
         <is>
-          <t>200 g tenderloin (marinated in olive oil, thyme and chilli flakes), served with roasted pepper &amp; tomato, rice and fries</t>
-        </is>
-      </c>
-      <c r="H61" s="5" t="inlineStr"/>
+          <t>200 g tenderloin (marinated in olive oil, thyme and chilli flakes), lavash, served with roasted pepper &amp; tomato, rice and wedge potatoes</t>
+        </is>
+      </c>
+      <c r="H61" s="5" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="I61" s="5" t="inlineStr"/>
       <c r="J61" s="5" t="inlineStr"/>
       <c r="K61" s="5" t="inlineStr"/>
@@ -5371,21 +5427,25 @@
       <c r="T61" s="5" t="inlineStr"/>
       <c r="U61" s="5" t="inlineStr"/>
       <c r="V61" s="6" t="n">
-        <v>850</v>
+        <v>1050</v>
       </c>
       <c r="W61" s="7" t="n">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="X61" s="7" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="Y61" s="7" t="n">
-        <v>44</v>
+        <v>84</v>
       </c>
       <c r="Z61" s="8" t="inlineStr"/>
       <c r="AA61" s="8" t="inlineStr"/>
       <c r="AB61" s="8" t="inlineStr"/>
-      <c r="AC61" s="9" t="inlineStr"/>
+      <c r="AC61" s="9" t="inlineStr">
+        <is>
+          <t>G: lavaş</t>
+        </is>
+      </c>
       <c r="AD61" s="10" t="inlineStr"/>
     </row>
     <row r="62">
@@ -5414,12 +5474,12 @@
       </c>
       <c r="F62" s="4" t="inlineStr">
         <is>
-          <t>200 g bonfile (zeytinyağı, kekik ve pul biber ile marine edilmiş), mantar sos (krema, Cafe de Paris sos), közlenmiş biber &amp; domates, pilav ve patates eşliğinde</t>
+          <t>200 g bonfile (zeytinyağı, kekik ve pul biber ile marine edilmiş), mantar sos (krema, Cafe de Paris sos, Demi Glace sos), 200 g fettuccine, közlenmiş biber &amp; domates, pilav ve elma dilim patates eşliğinde</t>
         </is>
       </c>
       <c r="G62" s="4" t="inlineStr">
         <is>
-          <t>200 g tenderloin (marinated in olive oil, thyme and chilli flakes), mushroom sauce (cream, Café de Paris sauce), served with roasted pepper &amp; tomato, rice and fries</t>
+          <t>200 g tenderloin (marinated in olive oil, thyme and chilli flakes), mushroom sauce (cream, Café de Paris sauce, Demi-Glace sauce), 200 g fettuccine, served with roasted pepper &amp; tomato, rice and wedge potatoes</t>
         </is>
       </c>
       <c r="H62" s="5" t="inlineStr">
@@ -5440,32 +5500,36 @@
       <c r="O62" s="5" t="inlineStr"/>
       <c r="P62" s="5" t="inlineStr"/>
       <c r="Q62" s="5" t="inlineStr"/>
-      <c r="R62" s="5" t="inlineStr"/>
+      <c r="R62" s="5" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="S62" s="5" t="inlineStr"/>
       <c r="T62" s="5" t="inlineStr"/>
       <c r="U62" s="5" t="inlineStr"/>
       <c r="V62" s="6" t="n">
-        <v>950</v>
+        <v>1240</v>
       </c>
       <c r="W62" s="7" t="n">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="X62" s="7" t="n">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="Y62" s="7" t="n">
-        <v>46</v>
+        <v>102</v>
       </c>
       <c r="Z62" s="8" t="inlineStr"/>
       <c r="AA62" s="8" t="inlineStr"/>
       <c r="AB62" s="8" t="inlineStr">
         <is>
-          <t>cafedeparis</t>
+          <t>cafedeparis, demiglace</t>
         </is>
       </c>
       <c r="AC62" s="9" t="inlineStr">
         <is>
-          <t>M: mantar sos, krema, cafe de paris sos, Cafe de Paris Sos · G: cafe de paris sos, Cafe de Paris Sos</t>
+          <t>M: krema, cafe de paris sos, demi glace sos · G: cafe de paris sos, demi glace sos, fettuccine · C: demi glace sos</t>
         </is>
       </c>
       <c r="AD62" s="10" t="inlineStr"/>
@@ -5496,12 +5560,12 @@
       </c>
       <c r="F63" s="4" t="inlineStr">
         <is>
-          <t>200 g bonfile, Cafe de Paris sos, közlenmiş biber &amp; domates, pilav ve patates eşliğinde</t>
+          <t>200 g bonfile, Cafe de Paris sos, közlenmiş biber &amp; domates, pilav ve elma dilim patates eşliğinde</t>
         </is>
       </c>
       <c r="G63" s="4" t="inlineStr">
         <is>
-          <t>200 g tenderloin, Café de Paris sauce, served with roasted pepper &amp; tomato, rice and fries</t>
+          <t>200 g tenderloin, Café de Paris sauce, served with roasted pepper &amp; tomato, rice and wedge potatoes</t>
         </is>
       </c>
       <c r="H63" s="5" t="inlineStr">
@@ -5547,7 +5611,7 @@
       </c>
       <c r="AC63" s="9" t="inlineStr">
         <is>
-          <t>G: cafe de paris sos, Cafe de Paris Sos · M: cafe de paris sos, Cafe de Paris Sos</t>
+          <t>G: cafe de paris sos · M: cafe de paris sos</t>
         </is>
       </c>
       <c r="AD63" s="10" t="inlineStr"/>
@@ -5578,12 +5642,12 @@
       </c>
       <c r="F64" s="4" t="inlineStr">
         <is>
-          <t>200 g kekik, zeytinyağı ve pul biber ile marine edilmiş et, renkli biberler, soğan, Sweet Chili sos, süzme yoğurt, özel Kule sos (Sweet Chili sos, mayonez, acı sos, pul biber, tuz), lavaş</t>
+          <t>200 g et (kekik, zeytinyağı ve pul biber ile marine edilmiş), renkli biberler, soğan, tereyağı, ayçiçek yağı. Yanında: Sweet Chili sos, Kule sos (Sweet Chili sos, mayonez, acı sos, pul biber, tuz), süzme yoğurt, lavaş</t>
         </is>
       </c>
       <c r="G64" s="4" t="inlineStr">
         <is>
-          <t>200 g beef marinated in thyme, olive oil and chilli flakes, bell peppers, onion, sweet chilli sauce, strained yoghurt, special Kule sauce (sweet chilli sauce, mayonnaise, hot sauce, chilli flakes, salt), lavash</t>
+          <t>200 g beef (marinated in thyme, olive oil and chilli flakes), bell peppers, onion, butter, sunflower oil. Served with: sweet chilli sauce, Kule sauce (sweet chilli sauce, mayonnaise, hot sauce, chilli flakes, salt), strained yoghurt, lavash</t>
         </is>
       </c>
       <c r="H64" s="5" t="inlineStr">
@@ -5613,13 +5677,13 @@
       <c r="T64" s="5" t="inlineStr"/>
       <c r="U64" s="5" t="inlineStr"/>
       <c r="V64" s="6" t="n">
-        <v>1120</v>
+        <v>1330</v>
       </c>
       <c r="W64" s="7" t="n">
         <v>58</v>
       </c>
       <c r="X64" s="7" t="n">
-        <v>54</v>
+        <v>78</v>
       </c>
       <c r="Y64" s="7" t="n">
         <v>92</v>
@@ -5633,7 +5697,7 @@
       </c>
       <c r="AC64" s="9" t="inlineStr">
         <is>
-          <t>M: süzme yoğurt · Y: özel kule sos, mayonez · G: lavaş</t>
+          <t>M: tereyağı, süzme yoğurt · Y: mayonez · G: lavaş</t>
         </is>
       </c>
       <c r="AD64" s="10" t="inlineStr"/>
@@ -5664,12 +5728,12 @@
       </c>
       <c r="F65" s="4" t="inlineStr">
         <is>
-          <t>150 g et ve 150 g tavuk (kekik, zeytinyağı ve pul biber ile marine edilmiş), renkli biberler, soğan, Sweet Chili sos, süzme yoğurt, özel Kule sos (Sweet Chili sos, mayonez, acı sos, pul biber, tuz), lavaş</t>
+          <t>150 g et ve 150 g tavuk (kekik, zeytinyağı ve pul biber ile marine edilmiş), renkli biberler, soğan, tereyağı, ayçiçek yağı. Yanında: Sweet Chili sos, Kule sos (Sweet Chili sos, mayonez, acı sos, pul biber, tuz), süzme yoğurt, lavaş</t>
         </is>
       </c>
       <c r="G65" s="4" t="inlineStr">
         <is>
-          <t>150 g beef and 150 g chicken (marinated in thyme, olive oil and chilli flakes), bell peppers, onion, sweet chilli sauce, strained yoghurt, special Kule sauce (sweet chilli sauce, mayonnaise, hot sauce, chilli flakes, salt), lavash</t>
+          <t>150 g beef and 150 g chicken (marinated in thyme, olive oil and chilli flakes), bell peppers, onion, butter, sunflower oil. Served with: sweet chilli sauce, Kule sauce (sweet chilli sauce, mayonnaise, hot sauce, chilli flakes, salt), strained yoghurt, lavash</t>
         </is>
       </c>
       <c r="H65" s="5" t="inlineStr">
@@ -5699,13 +5763,13 @@
       <c r="T65" s="5" t="inlineStr"/>
       <c r="U65" s="5" t="inlineStr"/>
       <c r="V65" s="6" t="n">
-        <v>1150</v>
+        <v>1360</v>
       </c>
       <c r="W65" s="7" t="n">
         <v>66</v>
       </c>
       <c r="X65" s="7" t="n">
-        <v>52</v>
+        <v>76</v>
       </c>
       <c r="Y65" s="7" t="n">
         <v>92</v>
@@ -5719,7 +5783,7 @@
       </c>
       <c r="AC65" s="9" t="inlineStr">
         <is>
-          <t>M: süzme yoğurt · Y: özel kule sos, mayonez · G: lavaş</t>
+          <t>M: tereyağı, süzme yoğurt · Y: mayonez · G: lavaş</t>
         </is>
       </c>
       <c r="AD65" s="10" t="inlineStr"/>
@@ -13481,7 +13545,7 @@
     <row r="8">
       <c r="A8" s="12" t="inlineStr">
         <is>
-          <t>Sos kartı sütunu: o üründe hangi hazır sosun ayrı kartı gösteriliyor (sweetchili / cafedeparis / demiglace).</t>
+          <t>Sos kartı sütunu: o üründe hangi hazır sosun ayrı kartı gösteriliyor (sweetchili / cafedeparis / demiglace / bbq / kori).</t>
         </is>
       </c>
     </row>
@@ -13777,7 +13841,7 @@
       </c>
       <c r="B9" s="16" t="inlineStr">
         <is>
-          <t>HARDAL olarak işaretlendi (köri karışımları çoğunlukla hardal içerir). Etiketi kontrol edin.</t>
+          <t>ÇÖZÜLDÜ — üretici etiketi alındı (karabiber, kişniş, kimyon, çemen, sarımsak, zerdeçal, tuz, kırmızı tatlı biber, tarçın): beyan edilen alerjen yok. Tabaktaki sos krema ile hazırlandığı için SÜT ürünün kendi içindekilerinden geliyor.</t>
         </is>
       </c>
     </row>
@@ -13789,7 +13853,7 @@
       </c>
       <c r="B10" s="16" t="inlineStr">
         <is>
-          <t>GLUTEN işaretli (galeta unu/ekmek içi). Harcında YUMURTA da varsa yumurta eklenmeli.</t>
+          <t>Harç yazıldı: sarımsak, galeta unu, karabiber, kimyon, pul biber → GLUTEN. Harçta YUMURTA da varsa bildirin, eklenir. Burger köftesine ayrıca uygulanmadı — aynı harç mı?</t>
         </is>
       </c>
     </row>
@@ -13801,7 +13865,7 @@
       </c>
       <c r="B11" s="16" t="inlineStr">
         <is>
-          <t>GLUTEN + YUMURTA işaretli (çıtır kaplama varsayıldı). Kaplamasız ise kaldırılacak.</t>
+          <t>ÇÖZÜLDÜ — gerçek kaplama malzemeleri yazıldı (süt, un, soya sosu, Cajun baharatı, galeta unu, pane): GLUTEN, SÜT ve SOYA artık içindekilerden türüyor.</t>
         </is>
       </c>
     </row>
@@ -13849,7 +13913,7 @@
       </c>
       <c r="B15" s="16" t="inlineStr">
         <is>
-          <t>Alerjen işaretlenmedi. Hazır BBQ sosları HARDAL / KEREVİZ / SOYA içerebilir — etiketi kontrol edin.</t>
+          <t>ÇÖZÜLDÜ — üretici etiketi alındı: renklendirici (amonyak karamel) GLUTEN içeriyor; iz miktarda süt, yumurta, hardal, kereviz uyarısı sos kartında gösteriliyor. Domuz türevi yok.</t>
         </is>
       </c>
     </row>
@@ -13909,7 +13973,7 @@
       </c>
       <c r="B20" s="16" t="inlineStr">
         <is>
-          <t>Sos kartı hazır (GLUTEN, SÜT, KEREVİZ) ama hiçbir ürüne bağlı değil. Hangi yemeklerde kullanılıyor?</t>
+          <t>ÇÖZÜLDÜ — Mantar Soslu Bonfile'nin mantar sosunda kullanılıyor (GLUTEN, SÜT, KEREVİZ). Başka yemekte de kullanılıyorsa bildirin.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Menü güncelleme 05.10.2026 13:53
</commit_message>
<xml_diff>
--- a/KULE-alerjen-kontrol.xlsx
+++ b/KULE-alerjen-kontrol.xlsx
@@ -10208,8 +10208,16 @@
       <c r="E124" s="3" t="n">
         <v>120</v>
       </c>
-      <c r="F124" s="4" t="inlineStr"/>
-      <c r="G124" s="4" t="inlineStr"/>
+      <c r="F124" s="4" t="inlineStr">
+        <is>
+          <t>Gazlı içecek</t>
+        </is>
+      </c>
+      <c r="G124" s="4" t="inlineStr">
+        <is>
+          <t>Carbonated soft drink</t>
+        </is>
+      </c>
       <c r="H124" s="5" t="inlineStr"/>
       <c r="I124" s="5" t="inlineStr"/>
       <c r="J124" s="5" t="inlineStr"/>
@@ -10266,8 +10274,16 @@
       <c r="E125" s="3" t="n">
         <v>120</v>
       </c>
-      <c r="F125" s="4" t="inlineStr"/>
-      <c r="G125" s="4" t="inlineStr"/>
+      <c r="F125" s="4" t="inlineStr">
+        <is>
+          <t>Şekersiz gazlı içecek</t>
+        </is>
+      </c>
+      <c r="G125" s="4" t="inlineStr">
+        <is>
+          <t>Sugar-free carbonated soft drink</t>
+        </is>
+      </c>
       <c r="H125" s="5" t="inlineStr"/>
       <c r="I125" s="5" t="inlineStr"/>
       <c r="J125" s="5" t="inlineStr"/>
@@ -10324,8 +10340,16 @@
       <c r="E126" s="3" t="n">
         <v>120</v>
       </c>
-      <c r="F126" s="4" t="inlineStr"/>
-      <c r="G126" s="4" t="inlineStr"/>
+      <c r="F126" s="4" t="inlineStr">
+        <is>
+          <t>Limon aromalı gazlı içecek</t>
+        </is>
+      </c>
+      <c r="G126" s="4" t="inlineStr">
+        <is>
+          <t>Lemon-lime soft drink</t>
+        </is>
+      </c>
       <c r="H126" s="5" t="inlineStr"/>
       <c r="I126" s="5" t="inlineStr"/>
       <c r="J126" s="5" t="inlineStr"/>
@@ -10382,8 +10406,16 @@
       <c r="E127" s="3" t="n">
         <v>120</v>
       </c>
-      <c r="F127" s="4" t="inlineStr"/>
-      <c r="G127" s="4" t="inlineStr"/>
+      <c r="F127" s="4" t="inlineStr">
+        <is>
+          <t>Portakal aromalı gazlı içecek</t>
+        </is>
+      </c>
+      <c r="G127" s="4" t="inlineStr">
+        <is>
+          <t>Orange soft drink</t>
+        </is>
+      </c>
       <c r="H127" s="5" t="inlineStr"/>
       <c r="I127" s="5" t="inlineStr"/>
       <c r="J127" s="5" t="inlineStr"/>
@@ -10844,8 +10876,16 @@
       <c r="E134" s="3" t="n">
         <v>90</v>
       </c>
-      <c r="F134" s="4" t="inlineStr"/>
-      <c r="G134" s="4" t="inlineStr"/>
+      <c r="F134" s="4" t="inlineStr">
+        <is>
+          <t>Maden suyu</t>
+        </is>
+      </c>
+      <c r="G134" s="4" t="inlineStr">
+        <is>
+          <t>Sparkling mineral water</t>
+        </is>
+      </c>
       <c r="H134" s="5" t="inlineStr"/>
       <c r="I134" s="5" t="inlineStr"/>
       <c r="J134" s="5" t="inlineStr"/>
@@ -10902,8 +10942,16 @@
       <c r="E135" s="3" t="n">
         <v>110</v>
       </c>
-      <c r="F135" s="4" t="inlineStr"/>
-      <c r="G135" s="4" t="inlineStr"/>
+      <c r="F135" s="4" t="inlineStr">
+        <is>
+          <t>Meyve aromalı maden suyu</t>
+        </is>
+      </c>
+      <c r="G135" s="4" t="inlineStr">
+        <is>
+          <t>Fruit-flavoured mineral water</t>
+        </is>
+      </c>
       <c r="H135" s="5" t="inlineStr"/>
       <c r="I135" s="5" t="inlineStr"/>
       <c r="J135" s="5" t="inlineStr"/>
@@ -10962,12 +11010,12 @@
       </c>
       <c r="F136" s="4" t="inlineStr">
         <is>
-          <t>Limon, su, şeker, nane</t>
+          <t>Limon, su, şeker</t>
         </is>
       </c>
       <c r="G136" s="4" t="inlineStr">
         <is>
-          <t>Lemon, water, sugar, mint</t>
+          <t>Lemon, water, sugar</t>
         </is>
       </c>
       <c r="H136" s="5" t="inlineStr"/>

</xml_diff>

<commit_message>
Menü güncelleme 05.10.2026 14:46
</commit_message>
<xml_diff>
--- a/KULE-alerjen-kontrol.xlsx
+++ b/KULE-alerjen-kontrol.xlsx
@@ -13834,7 +13834,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B41"/>
+  <dimension ref="A1:B44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -14252,38 +14252,74 @@
     <row r="38">
       <c r="A38" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Sosis Box</t>
+          <t xml:space="preserve">  TÜM İÇECEKLER (05.10.2026)</t>
         </is>
       </c>
       <c r="B38" s="16" t="inlineStr">
         <is>
-          <t>'8 adet ızgara sosis' -&gt; '8 adet sosis'.</t>
+          <t>İçecekler bölümünün TAMAMINDA (76 ürün) ve Dondurma (1/3 Top)'ta içindekiler artık menüde GÖSTERİLMİYOR. ÖNEMLİ: alerjenler gösterilmeye devam ediyor — sütlü kahveler, milkshake'ler, ayran ve dondurma hâlâ SÜT uyarısı veriyor (mevzuat gereği kaldırmadım; kaldırılsın isterseniz söyleyin). İçindekiler verisi arka planda duruyor, alerjen oradan türetiliyor.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="15" t="inlineStr">
         <is>
+          <t xml:space="preserve">  Limonata</t>
+        </is>
+      </c>
+      <c r="B39" s="16" t="inlineStr">
+        <is>
+          <t>Nane çıkarıldı: limon, su, şeker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Gizleme nasıl değişir</t>
+        </is>
+      </c>
+      <c r="B40" s="16" t="inlineStr">
+        <is>
+          <t>kaynak/build.js içindeki IHIDE_SECTIONS (bölüm id'si) ve IHIDE_ITEMS (ürün adı) listelerine ekleyip çıkararak. Cappy / Fuse Tea zaten içecek bölümünde olduğu için onlar da gizli.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Sosis Box</t>
+        </is>
+      </c>
+      <c r="B41" s="16" t="inlineStr">
+        <is>
+          <t>'8 adet ızgara sosis' -&gt; '8 adet sosis'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="15" t="inlineStr">
+        <is>
           <t xml:space="preserve">  Big Combo Mix</t>
         </is>
       </c>
-      <c r="B39" s="16" t="inlineStr">
+      <c r="B42" s="16" t="inlineStr">
         <is>
           <t>Sigara böreğinin içindekileri yazıldı (yufka, beyaz peynir, maydanoz, soda, tuz) — SÜT artık beyaz peynirden türüyor.</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="15" t="inlineStr"/>
-      <c r="B40" s="16" t="inlineStr"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="13" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="15" t="inlineStr"/>
+      <c r="B43" s="16" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="13" t="inlineStr">
         <is>
           <t>BESİN DEĞERLERİ</t>
         </is>
       </c>
-      <c r="B41" s="14" t="inlineStr">
+      <c r="B44" s="14" t="inlineStr">
         <is>
           <t>Tatlılar bölümündeki Lupin ürünleri üreticinin 100 g beyanı x ürün gramajıdır. DİĞER TÜM ürünlerin kcal / protein / yağ / karbonhidrat değerleri TAHMİNDİR — diyetisyen doğrulaması gerekir.</t>
         </is>

</xml_diff>